<commit_message>
Updated Deepthi & Saranya payments
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3E86F8-2C21-D847-A07F-08EB7B1C8B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89BA3BC0-DE57-0F4E-82A2-AF3C47A34C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2181,9 +2181,6 @@
     <t>Simi (TVM), Saranya Gopalakrishanan (pending-1250)</t>
   </si>
   <si>
-    <t>Saranya Gopalakrishnan(1250 pending)</t>
-  </si>
-  <si>
     <t>Dec, Jan &amp; Feb boosting</t>
   </si>
   <si>
@@ -2200,6 +2197,9 @@
   </si>
   <si>
     <t>Rainbow saree &amp; Golden yello with Butterfly on pallu</t>
+  </si>
+  <si>
+    <t>Saranya Gopalakrishnan(1300 pending)</t>
   </si>
 </sst>
 </file>
@@ -3077,7 +3077,7 @@
                   <c:v>45448</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>19039</c:v>
+                  <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -3332,7 +3332,7 @@
                   <c:v>-1863</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14249</c:v>
+                  <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -7848,7 +7848,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>226634</v>
+        <v>230564</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>230514</v>
+        <v>230564</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-30485</v>
+        <v>-26555</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -8091,15 +8091,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>207485</v>
+        <v>211415</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>75559.775599999994</v>
+        <v>76870.037599999996</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>131925.22440000001</v>
+        <v>134544.96240000002</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>7871.7484000000113</v>
+        <v>10491.486400000023</v>
       </c>
       <c r="G26" s="71" t="s">
         <v>673</v>
@@ -8124,11 +8124,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>75514.448799999998</v>
+        <v>76823.924799999993</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-68895.448799999998</v>
+        <v>-70204.924799999993</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-3934.4967999999935</v>
+        <v>-5243.9727999999886</v>
       </c>
       <c r="G27" s="72" t="s">
         <v>674</v>
@@ -8153,11 +8153,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>75559.775599999994</v>
+        <v>76870.037599999996</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-63029.775599999994</v>
+        <v>-64340.037599999996</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8165,7 +8165,7 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-3937.2515999999887</v>
+        <v>-5247.5135999999911</v>
       </c>
       <c r="G28" s="73" t="s">
         <v>674</v>
@@ -8265,7 +8265,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8281,7 +8281,7 @@
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>226634</v>
+        <v>230564</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-30485</v>
+        <v>-26555</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
@@ -8354,11 +8354,11 @@
       </c>
       <c r="C11" s="19">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A11)*Sales!$C$2:$C$998),0)</f>
-        <v>19039</v>
+        <v>19089</v>
       </c>
       <c r="D11" s="19">
         <f t="shared" si="0"/>
-        <v>14249</v>
+        <v>14299</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>72</v>
@@ -9371,7 +9371,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -14580,7 +14580,7 @@
         <v>669</v>
       </c>
       <c r="I115" s="47" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -14791,7 +14791,7 @@
         <v>693</v>
       </c>
       <c r="C124" s="51">
-        <v>2500</v>
+        <v>2550</v>
       </c>
       <c r="D124" s="50" t="s">
         <v>281</v>
@@ -14805,7 +14805,7 @@
         <v>694</v>
       </c>
       <c r="I124" s="50" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:9" ht="16">
@@ -14827,7 +14827,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -14838,7 +14838,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -14852,7 +14852,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -20120,7 +20120,7 @@
       <c r="S69" s="28"/>
       <c r="T69" s="28"/>
     </row>
-    <row r="70" spans="1:20" ht="15" customHeight="1">
+    <row r="70" spans="1:20" ht="29" customHeight="1">
       <c r="A70" s="26" t="s">
         <v>412</v>
       </c>
@@ -20163,7 +20163,7 @@
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
-        <v>191</v>
+        <v>122</v>
       </c>
       <c r="O70" s="30"/>
       <c r="P70" s="30"/>
@@ -21287,7 +21287,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21339,7 +21339,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -23461,11 +23461,11 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
-        <v>191</v>
+        <v>122</v>
       </c>
       <c r="O132" s="30"/>
       <c r="P132" s="30"/>
@@ -25599,7 +25599,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>207485</v>
+        <v>211415</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -25607,11 +25607,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>75559.775599999994</v>
+        <v>76870.037599999996</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>131925.22440000001</v>
+        <v>134544.96240000002</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25619,7 +25619,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>7871.7484000000113</v>
+        <v>10491.486400000023</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -25636,11 +25636,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>75514.448799999998</v>
+        <v>76823.924799999993</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-68895.448799999998</v>
+        <v>-70204.924799999993</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25648,7 +25648,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-3934.4967999999935</v>
+        <v>-5243.9727999999886</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -25665,11 +25665,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>75559.775599999994</v>
+        <v>76870.037599999996</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-63029.775599999994</v>
+        <v>-64340.037599999996</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25677,7 +25677,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-3937.2515999999887</v>
+        <v>-5247.5135999999911</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
Latest sales & purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89BA3BC0-DE57-0F4E-82A2-AF3C47A34C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944C5450-1DDE-814E-A630-AB3FE64FE254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1756" uniqueCount="705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="718">
   <si>
     <t>Notes:</t>
   </si>
@@ -1679,12 +1679,6 @@
   </si>
   <si>
     <t>Domain Registration (3 years)</t>
-  </si>
-  <si>
-    <t>Jisha (1545-XL), Shiji(1370-L)</t>
-  </si>
-  <si>
-    <t>Sushitha (XL-1600)</t>
   </si>
   <si>
     <t>M, L, XXL</t>
@@ -2158,9 +2152,6 @@
   </si>
   <si>
     <t>Laks Pillai</t>
-  </si>
-  <si>
-    <t>Saranya Gopalakrishnan</t>
   </si>
   <si>
     <t>Semi Silk Black and Cotton Silk Green</t>
@@ -2200,6 +2191,54 @@
   </si>
   <si>
     <t>Saranya Gopalakrishnan(1300 pending)</t>
+  </si>
+  <si>
+    <t>Aanchal cotton salwars</t>
+  </si>
+  <si>
+    <t>Net kota saree - turquoise blue</t>
+  </si>
+  <si>
+    <t>Maheswari Cotton Sil Red/Black</t>
+  </si>
+  <si>
+    <t>Priya (Hosur)</t>
+  </si>
+  <si>
+    <t>Saranya Gopalakrishnan(Hyd)</t>
+  </si>
+  <si>
+    <t>Haris (EKM)</t>
+  </si>
+  <si>
+    <t>Sheeja mol maid</t>
+  </si>
+  <si>
+    <t>Sheeja mol</t>
+  </si>
+  <si>
+    <t>haris(ekm)</t>
+  </si>
+  <si>
+    <t>priya(hosur)</t>
+  </si>
+  <si>
+    <t>Jisha (1545-XL), Shiji(1370-L), Sheejamol(XXL)-850</t>
+  </si>
+  <si>
+    <t>Aanchal Blue - 1200</t>
+  </si>
+  <si>
+    <t>Sheeja mol maid(1200)</t>
+  </si>
+  <si>
+    <t>Sushitha (XL-1600), Sheeja Mol (1400)</t>
+  </si>
+  <si>
+    <t>M, L</t>
+  </si>
+  <si>
+    <t>Roman Silk(XXL), Coral Pink (XXL)</t>
   </si>
 </sst>
 </file>
@@ -2962,7 +3001,7 @@
                   <c:v>4790</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>9492</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3080,7 +3119,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>5400</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3335,7 +3374,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>-4092</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3658,10 +3697,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>175</c:v>
+                  <c:v>182</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>110</c:v>
+                  <c:v>103</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3970,10 +4009,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>106</c:v>
+                  <c:v>108</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>67</c:v>
+                  <c:v>72</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4093,10 +4132,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>52</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>53</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4523,10 +4562,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>58255</c:v>
+                  <c:v>53077</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>43574.18</c:v>
+                  <c:v>42425.18</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -7833,7 +7872,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(Purchases!C:C)</f>
-        <v>257119</v>
+        <v>266611</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>39</v>
@@ -7848,7 +7887,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>230564</v>
+        <v>232514</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7865,7 +7904,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>230564</v>
+        <v>235964</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -7882,7 +7921,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-26555</v>
+        <v>-34097</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -7917,7 +7956,7 @@
       </c>
       <c r="B10" s="52">
         <f>PartnerShares!H8</f>
-        <v>-1596.3333333333285</v>
+        <v>1567.6666666666715</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -7927,7 +7966,7 @@
       </c>
       <c r="B11" s="53">
         <f>PartnerShares!H9</f>
-        <v>1903.006666666668</v>
+        <v>-1260.993333333332</v>
       </c>
       <c r="C11" s="7"/>
     </row>
@@ -7976,15 +8015,15 @@
       </c>
       <c r="B18" s="6">
         <f>PartnerShares!B8</f>
-        <v>97424</v>
+        <v>103752</v>
       </c>
       <c r="C18" s="6">
         <f>PartnerShares!C8</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D18" s="6">
         <f>PartnerShares!D8</f>
-        <v>11717.666666666672</v>
+        <v>14881.666666666672</v>
       </c>
       <c r="E18" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7992,10 +8031,10 @@
       </c>
       <c r="F18" s="8">
         <f>D18-E18</f>
-        <v>-1596.3333333333285</v>
-      </c>
-      <c r="G18" s="71" t="s">
-        <v>673</v>
+        <v>1567.6666666666715</v>
+      </c>
+      <c r="G18" s="73" t="s">
+        <v>672</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8009,11 +8048,11 @@
       </c>
       <c r="C19" s="7">
         <f>PartnerShares!C9</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D19" s="7">
         <f>PartnerShares!D9</f>
-        <v>48475.666666666672</v>
+        <v>45311.666666666672</v>
       </c>
       <c r="E19" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8021,10 +8060,10 @@
       </c>
       <c r="F19" s="9">
         <f>D19-E19</f>
-        <v>1903.006666666668</v>
-      </c>
-      <c r="G19" s="73" t="s">
-        <v>674</v>
+        <v>-1260.993333333332</v>
+      </c>
+      <c r="G19" s="71" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -8034,11 +8073,11 @@
       </c>
       <c r="B20" s="6">
         <f>PartnerShares!B10</f>
-        <v>25513</v>
+        <v>28677</v>
       </c>
       <c r="C20" s="6">
         <f>PartnerShares!C10</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D20" s="6">
         <f>PartnerShares!D10</f>
@@ -8053,7 +8092,7 @@
         <v>-306.67333333332499</v>
       </c>
       <c r="G20" s="71" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1">
@@ -8091,15 +8130,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>211415</v>
+        <v>213365</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>76870.037599999996</v>
+        <v>77520.167600000001</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>134544.96240000002</v>
+        <v>135844.83240000001</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8107,10 +8146,10 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>10491.486400000023</v>
+        <v>11791.356400000019</v>
       </c>
       <c r="G26" s="71" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -8124,11 +8163,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>76823.924799999993</v>
+        <v>77473.664799999999</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-70204.924799999993</v>
+        <v>-70854.664799999999</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8136,10 +8175,10 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-5243.9727999999886</v>
+        <v>-5893.7127999999939</v>
       </c>
       <c r="G27" s="72" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -8153,11 +8192,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>76870.037599999996</v>
+        <v>77520.167600000001</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-64340.037599999996</v>
+        <v>-64990.167600000001</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8165,10 +8204,10 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-5247.5135999999911</v>
+        <v>-5897.6435999999958</v>
       </c>
       <c r="G28" s="73" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1">
@@ -8265,7 +8304,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46085</v>
+        <v>46090</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8274,14 +8313,14 @@
       </c>
       <c r="B5" s="15">
         <f>Summary!B3</f>
-        <v>257119</v>
+        <v>266611</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>230564</v>
+        <v>232514</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8290,14 +8329,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-26555</v>
+        <v>-34097</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>98809.68</v>
+        <v>94434.68</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8341,7 +8380,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>175</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8365,7 +8404,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8374,15 +8413,15 @@
       </c>
       <c r="B12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A12)*Purchases!$C$2:$C$998),0)</f>
-        <v>0</v>
+        <v>9492</v>
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>0</v>
+        <v>5400</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-4092</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8561,18 +8600,18 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
       </c>
       <c r="K47" s="77" cm="1">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$479=J47)*(INVENTORY!$D$2:$D$479)*(INVENTORY!$G$2:$G$479))</f>
-        <v>58255</v>
+        <v>53077</v>
       </c>
     </row>
     <row r="48" spans="6:11">
@@ -8581,18 +8620,18 @@
       </c>
       <c r="G48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="H48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="J48" s="76" t="s">
         <v>120</v>
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$479=J48)*(INVENTORY!$D$2:$D$479)*(INVENTORY!$G$2:$G$479))</f>
-        <v>43574.18</v>
+        <v>42425.18</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9202,7 +9241,7 @@
         <v>1760</v>
       </c>
       <c r="D37" s="37" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -9216,7 +9255,7 @@
         <v>1330</v>
       </c>
       <c r="D38" s="39" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -9230,7 +9269,7 @@
         <v>5940</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -9272,7 +9311,7 @@
         <v>4425</v>
       </c>
       <c r="D42" s="39" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -9286,7 +9325,7 @@
         <v>1370</v>
       </c>
       <c r="D43" s="37" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -9314,7 +9353,7 @@
         <v>106</v>
       </c>
       <c r="D45" s="37" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -9356,7 +9395,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9371,20 +9410,36 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="41"/>
-      <c r="B50" s="39"/>
-      <c r="C50" s="40"/>
-      <c r="D50" s="39"/>
+      <c r="A50" s="41">
+        <v>46087</v>
+      </c>
+      <c r="B50" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="40">
+        <v>6328</v>
+      </c>
+      <c r="D50" s="39" t="s">
+        <v>702</v>
+      </c>
     </row>
     <row r="51" spans="1:4">
-      <c r="A51" s="36"/>
-      <c r="B51" s="37"/>
-      <c r="C51" s="38"/>
-      <c r="D51" s="37"/>
+      <c r="A51" s="36">
+        <v>46087</v>
+      </c>
+      <c r="B51" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="C51" s="38">
+        <v>3164</v>
+      </c>
+      <c r="D51" s="37" t="s">
+        <v>702</v>
+      </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="41"/>
@@ -13713,7 +13768,7 @@
         <v>46024</v>
       </c>
       <c r="B81" s="50" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C81" s="51">
         <v>2750</v>
@@ -13727,7 +13782,7 @@
       <c r="F81" s="50"/>
       <c r="G81" s="50"/>
       <c r="H81" s="69" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="I81" s="50" t="s">
         <v>276</v>
@@ -13738,7 +13793,7 @@
         <v>46024</v>
       </c>
       <c r="B82" s="47" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C82" s="48">
         <v>1400</v>
@@ -13752,7 +13807,7 @@
       <c r="F82" s="49"/>
       <c r="G82" s="49"/>
       <c r="H82" s="68" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="I82" s="47" t="s">
         <v>276</v>
@@ -13763,7 +13818,7 @@
         <v>46024</v>
       </c>
       <c r="B83" s="50" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C83" s="51">
         <v>1600</v>
@@ -13777,7 +13832,7 @@
       <c r="F83" s="50"/>
       <c r="G83" s="50"/>
       <c r="H83" s="69" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="I83" s="50" t="s">
         <v>276</v>
@@ -13802,7 +13857,7 @@
       <c r="F84" s="49"/>
       <c r="G84" s="49"/>
       <c r="H84" s="68" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="I84" s="47" t="s">
         <v>276</v>
@@ -13813,7 +13868,7 @@
         <v>46027</v>
       </c>
       <c r="B85" s="50" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C85" s="51">
         <v>1250</v>
@@ -13827,7 +13882,7 @@
       <c r="F85" s="50"/>
       <c r="G85" s="50"/>
       <c r="H85" s="69" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="I85" s="50" t="s">
         <v>276</v>
@@ -13838,7 +13893,7 @@
         <v>46028</v>
       </c>
       <c r="B86" s="50" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C86" s="51">
         <v>1380</v>
@@ -13852,7 +13907,7 @@
       <c r="F86" s="50"/>
       <c r="G86" s="50"/>
       <c r="H86" s="69" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="I86" s="50" t="s">
         <v>276</v>
@@ -13863,7 +13918,7 @@
         <v>46029</v>
       </c>
       <c r="B87" s="47" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C87" s="48">
         <v>1380</v>
@@ -13888,7 +13943,7 @@
         <v>46032</v>
       </c>
       <c r="B88" s="50" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C88" s="51">
         <v>1100</v>
@@ -13902,7 +13957,7 @@
       <c r="F88" s="50"/>
       <c r="G88" s="50"/>
       <c r="H88" s="69" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="I88" s="50" t="s">
         <v>276</v>
@@ -13913,7 +13968,7 @@
         <v>46033</v>
       </c>
       <c r="B89" s="47" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C89" s="48">
         <v>1380</v>
@@ -13938,7 +13993,7 @@
         <v>46033</v>
       </c>
       <c r="B90" s="50" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C90" s="51">
         <v>1100</v>
@@ -13952,7 +14007,7 @@
       <c r="F90" s="50"/>
       <c r="G90" s="50"/>
       <c r="H90" s="69" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="I90" s="50" t="s">
         <v>276</v>
@@ -13963,7 +14018,7 @@
         <v>46034</v>
       </c>
       <c r="B91" s="47" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="C91" s="48">
         <v>1100</v>
@@ -13977,7 +14032,7 @@
       <c r="F91" s="49"/>
       <c r="G91" s="49"/>
       <c r="H91" s="68" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="I91" s="47" t="s">
         <v>276</v>
@@ -13988,7 +14043,7 @@
         <v>46034</v>
       </c>
       <c r="B92" s="50" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="C92" s="51">
         <v>3000</v>
@@ -14002,7 +14057,7 @@
       <c r="F92" s="50"/>
       <c r="G92" s="50"/>
       <c r="H92" s="69" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="I92" s="50" t="s">
         <v>276</v>
@@ -14013,7 +14068,7 @@
         <v>46035</v>
       </c>
       <c r="B93" s="47" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="C93" s="48">
         <v>1450</v>
@@ -14027,7 +14082,7 @@
       <c r="F93" s="49"/>
       <c r="G93" s="49"/>
       <c r="H93" s="68" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="I93" s="47" t="s">
         <v>276</v>
@@ -14038,7 +14093,7 @@
         <v>46036</v>
       </c>
       <c r="B94" s="50" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C94" s="51">
         <v>1599</v>
@@ -14052,7 +14107,7 @@
       <c r="F94" s="50"/>
       <c r="G94" s="50"/>
       <c r="H94" s="69" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="I94" s="50" t="s">
         <v>276</v>
@@ -14063,7 +14118,7 @@
         <v>46038</v>
       </c>
       <c r="B95" s="47" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="C95" s="48">
         <v>1100</v>
@@ -14077,7 +14132,7 @@
       <c r="F95" s="49"/>
       <c r="G95" s="49"/>
       <c r="H95" s="68" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="I95" s="47" t="s">
         <v>276</v>
@@ -14088,7 +14143,7 @@
         <v>46038</v>
       </c>
       <c r="B96" s="50" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C96" s="51">
         <v>1650</v>
@@ -14102,7 +14157,7 @@
       <c r="F96" s="50"/>
       <c r="G96" s="50"/>
       <c r="H96" s="69" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="I96" s="50" t="s">
         <v>276</v>
@@ -14113,7 +14168,7 @@
         <v>46039</v>
       </c>
       <c r="B97" s="47" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C97" s="48">
         <v>2300</v>
@@ -14127,7 +14182,7 @@
       <c r="F97" s="49"/>
       <c r="G97" s="49"/>
       <c r="H97" s="68" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="I97" s="47" t="s">
         <v>276</v>
@@ -14138,7 +14193,7 @@
         <v>46040</v>
       </c>
       <c r="B98" s="50" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C98" s="51">
         <v>1399</v>
@@ -14152,7 +14207,7 @@
       <c r="F98" s="50"/>
       <c r="G98" s="50"/>
       <c r="H98" s="69" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="I98" s="50" t="s">
         <v>276</v>
@@ -14163,7 +14218,7 @@
         <v>46041</v>
       </c>
       <c r="B99" s="47" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="C99" s="48">
         <v>1100</v>
@@ -14177,7 +14232,7 @@
       <c r="F99" s="49"/>
       <c r="G99" s="49"/>
       <c r="H99" s="68" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="I99" s="47" t="s">
         <v>276</v>
@@ -14188,7 +14243,7 @@
         <v>46042</v>
       </c>
       <c r="B100" s="50" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C100" s="51">
         <v>1250</v>
@@ -14202,7 +14257,7 @@
       <c r="F100" s="50"/>
       <c r="G100" s="50"/>
       <c r="H100" s="69" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="I100" s="50" t="s">
         <v>276</v>
@@ -14213,7 +14268,7 @@
         <v>46043</v>
       </c>
       <c r="B101" s="47" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="C101" s="48">
         <v>1380</v>
@@ -14227,7 +14282,7 @@
       <c r="F101" s="49"/>
       <c r="G101" s="49"/>
       <c r="H101" s="68" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="I101" s="47" t="s">
         <v>276</v>
@@ -14238,7 +14293,7 @@
         <v>46046</v>
       </c>
       <c r="B102" s="50" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C102" s="51">
         <v>950</v>
@@ -14252,7 +14307,7 @@
       <c r="F102" s="50"/>
       <c r="G102" s="50"/>
       <c r="H102" s="69" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="I102" s="50" t="s">
         <v>276</v>
@@ -14263,7 +14318,7 @@
         <v>46048</v>
       </c>
       <c r="B103" s="47" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C103" s="48">
         <v>1380</v>
@@ -14277,7 +14332,7 @@
       <c r="F103" s="49"/>
       <c r="G103" s="49"/>
       <c r="H103" s="69" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="I103" s="47" t="s">
         <v>276</v>
@@ -14288,7 +14343,7 @@
         <v>46048</v>
       </c>
       <c r="B104" s="50" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C104" s="51">
         <v>2700</v>
@@ -14302,7 +14357,7 @@
       <c r="F104" s="50"/>
       <c r="G104" s="50"/>
       <c r="H104" s="69" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="I104" s="50" t="s">
         <v>276</v>
@@ -14313,7 +14368,7 @@
         <v>46049</v>
       </c>
       <c r="B105" s="47" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C105" s="48">
         <v>1380</v>
@@ -14338,7 +14393,7 @@
         <v>46049</v>
       </c>
       <c r="B106" s="50" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="C106" s="51">
         <v>1380</v>
@@ -14352,7 +14407,7 @@
       <c r="F106" s="50"/>
       <c r="G106" s="50"/>
       <c r="H106" s="69" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="I106" s="50" t="s">
         <v>276</v>
@@ -14363,7 +14418,7 @@
         <v>46049</v>
       </c>
       <c r="B107" s="47" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C107" s="48">
         <v>1200</v>
@@ -14377,7 +14432,7 @@
       <c r="F107" s="49"/>
       <c r="G107" s="49"/>
       <c r="H107" s="68" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="I107" s="47" t="s">
         <v>276</v>
@@ -14388,7 +14443,7 @@
         <v>46050</v>
       </c>
       <c r="B108" s="50" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="C108" s="51">
         <v>1250</v>
@@ -14402,7 +14457,7 @@
       <c r="F108" s="50"/>
       <c r="G108" s="50"/>
       <c r="H108" s="69" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="I108" s="50" t="s">
         <v>276</v>
@@ -14413,7 +14468,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14427,7 +14482,7 @@
       <c r="F109" s="49"/>
       <c r="G109" s="49"/>
       <c r="H109" s="68" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="I109" s="47" t="s">
         <v>276</v>
@@ -14438,7 +14493,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14452,7 +14507,7 @@
       <c r="F110" s="50"/>
       <c r="G110" s="50"/>
       <c r="H110" s="69" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="I110" s="50" t="s">
         <v>276</v>
@@ -14463,13 +14518,13 @@
         <v>46051</v>
       </c>
       <c r="B111" s="47" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C111" s="48">
         <v>580</v>
       </c>
       <c r="D111" s="47" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E111" s="47" t="s">
         <v>48</v>
@@ -14477,7 +14532,7 @@
       <c r="F111" s="49"/>
       <c r="G111" s="49"/>
       <c r="H111" s="68" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="I111" s="47" t="s">
         <v>276</v>
@@ -14488,7 +14543,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14502,7 +14557,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14513,7 +14568,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14527,7 +14582,7 @@
       <c r="F113" s="49"/>
       <c r="G113" s="49"/>
       <c r="H113" s="68" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="I113" s="47" t="s">
         <v>276</v>
@@ -14577,7 +14632,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14588,7 +14643,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14602,7 +14657,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14613,7 +14668,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14638,7 +14693,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14663,7 +14718,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14688,13 +14743,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14702,7 +14757,7 @@
       <c r="F120" s="50"/>
       <c r="G120" s="50"/>
       <c r="H120" s="69" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="I120" s="50" t="s">
         <v>276</v>
@@ -14727,7 +14782,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14738,7 +14793,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14752,7 +14807,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14763,7 +14818,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -14788,7 +14843,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>693</v>
+        <v>706</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -14802,7 +14857,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -14827,7 +14882,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -14838,7 +14893,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -14852,55 +14907,111 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="127" spans="1:9">
-      <c r="A127" s="46"/>
-      <c r="B127" s="47"/>
-      <c r="C127" s="48"/>
-      <c r="D127" s="47"/>
-      <c r="E127" s="47"/>
+      <c r="A127" s="46">
+        <v>46090</v>
+      </c>
+      <c r="B127" s="47" t="s">
+        <v>705</v>
+      </c>
+      <c r="C127" s="48">
+        <v>850</v>
+      </c>
+      <c r="D127" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E127" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
-      <c r="H127" s="68"/>
-      <c r="I127" s="47"/>
+      <c r="H127" s="28" t="s">
+        <v>703</v>
+      </c>
+      <c r="I127" s="47" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="128" spans="1:9">
-      <c r="A128" s="43"/>
-      <c r="B128" s="50"/>
-      <c r="C128" s="51"/>
-      <c r="D128" s="50"/>
-      <c r="E128" s="50"/>
+      <c r="A128" s="43">
+        <v>46090</v>
+      </c>
+      <c r="B128" s="50" t="s">
+        <v>707</v>
+      </c>
+      <c r="C128" s="51">
+        <v>1100</v>
+      </c>
+      <c r="D128" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E128" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
-      <c r="H128" s="69"/>
-      <c r="I128" s="50"/>
-    </row>
-    <row r="129" spans="1:9">
-      <c r="A129" s="46"/>
-      <c r="B129" s="47"/>
-      <c r="C129" s="48"/>
-      <c r="D129" s="47"/>
-      <c r="E129" s="47"/>
+      <c r="H128" s="69" t="s">
+        <v>704</v>
+      </c>
+      <c r="I128" s="50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" ht="16">
+      <c r="A129" s="46">
+        <v>46090</v>
+      </c>
+      <c r="B129" s="47" t="s">
+        <v>708</v>
+      </c>
+      <c r="C129" s="48">
+        <v>1200</v>
+      </c>
+      <c r="D129" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E129" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="F129" s="49"/>
       <c r="G129" s="49"/>
-      <c r="H129" s="68"/>
-      <c r="I129" s="47"/>
+      <c r="H129" s="68" t="s">
+        <v>713</v>
+      </c>
+      <c r="I129" s="47" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="130" spans="1:9">
-      <c r="A130" s="43"/>
-      <c r="B130" s="50"/>
-      <c r="C130" s="51"/>
-      <c r="D130" s="50"/>
-      <c r="E130" s="50"/>
+      <c r="A130" s="43">
+        <v>46090</v>
+      </c>
+      <c r="B130" s="50" t="s">
+        <v>709</v>
+      </c>
+      <c r="C130" s="51">
+        <v>2250</v>
+      </c>
+      <c r="D130" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E130" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
-      <c r="H130" s="69"/>
-      <c r="I130" s="50"/>
+      <c r="H130" s="69" t="s">
+        <v>717</v>
+      </c>
+      <c r="I130" s="50" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="131" spans="1:9">
       <c r="A131" s="46"/>
@@ -18925,10 +19036,10 @@
         <v>1094</v>
       </c>
       <c r="L47" s="28" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="M47" s="28" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="N47" s="28" t="s">
         <v>180</v>
@@ -19197,14 +19308,14 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O52" s="30" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="P52" s="30" t="s">
         <v>193</v>
@@ -19253,7 +19364,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19263,7 +19374,7 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
@@ -19365,7 +19476,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19637,7 +19748,7 @@
         <v>1080</v>
       </c>
       <c r="L60" s="30" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="M60" s="30" t="s">
         <v>46</v>
@@ -19699,7 +19810,7 @@
       </c>
       <c r="O61" s="28"/>
       <c r="P61" s="28" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="Q61" s="28" t="s">
         <v>480</v>
@@ -19747,7 +19858,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -19953,7 +20064,7 @@
         <v>1558</v>
       </c>
       <c r="L66" s="30" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="M66" s="30"/>
       <c r="N66" s="30" t="s">
@@ -20125,7 +20236,7 @@
         <v>412</v>
       </c>
       <c r="B70" s="30" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C70" s="30" t="s">
         <v>120</v>
@@ -20159,7 +20270,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -20541,7 +20652,7 @@
         <v>1990</v>
       </c>
       <c r="L77" s="28" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="M77" s="28"/>
       <c r="N77" s="28" t="s">
@@ -20701,14 +20812,14 @@
         <v>2460</v>
       </c>
       <c r="L80" s="30" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="M80" s="30"/>
       <c r="N80" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O80" s="30" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="P80" s="30"/>
       <c r="Q80" s="30"/>
@@ -20770,7 +20881,7 @@
       <c r="S81" s="28"/>
       <c r="T81" s="28"/>
     </row>
-    <row r="82" spans="1:20" ht="15">
+    <row r="82" spans="1:20" ht="30">
       <c r="A82" s="26" t="s">
         <v>424</v>
       </c>
@@ -20787,10 +20898,10 @@
         <v>1545</v>
       </c>
       <c r="F82" s="31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G82" s="31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H82" s="30">
         <f t="shared" si="6"/>
@@ -20802,22 +20913,20 @@
       </c>
       <c r="J82" s="30">
         <f t="shared" si="7"/>
-        <v>2150</v>
+        <v>3225</v>
       </c>
       <c r="K82" s="30">
         <f t="shared" si="8"/>
-        <v>1075</v>
+        <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>536</v>
+        <v>712</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
-        <v>222</v>
-      </c>
-      <c r="O82" s="30" t="s">
-        <v>497</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="O82" s="30"/>
       <c r="P82" s="30"/>
       <c r="Q82" s="30"/>
       <c r="R82" s="30"/>
@@ -20924,7 +21033,7 @@
         <v>180</v>
       </c>
       <c r="O84" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="P84" s="30"/>
       <c r="Q84" s="30"/>
@@ -20971,7 +21080,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21025,7 +21134,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21198,7 +21307,7 @@
     </row>
     <row r="90" spans="1:20" ht="15" customHeight="1">
       <c r="A90" s="26" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B90" s="30" t="s">
         <v>244</v>
@@ -21235,7 +21344,7 @@
         <v>0</v>
       </c>
       <c r="L90" s="30" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="M90" s="30"/>
       <c r="N90" s="30" t="s">
@@ -21287,7 +21396,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21339,7 +21448,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -21953,10 +22062,10 @@
         <v>1600</v>
       </c>
       <c r="F104" s="31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G104" s="31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H104" s="30">
         <f t="shared" si="9"/>
@@ -21968,11 +22077,11 @@
       </c>
       <c r="J104" s="30">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>976</v>
       </c>
       <c r="K104" s="30">
         <f t="shared" si="11"/>
-        <v>976</v>
+        <v>0</v>
       </c>
       <c r="L104" s="30" t="s">
         <v>148</v>
@@ -22007,10 +22116,10 @@
         <v>1600</v>
       </c>
       <c r="F105" s="29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H105" s="28">
         <f t="shared" si="9"/>
@@ -22022,11 +22131,11 @@
       </c>
       <c r="J105" s="28">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>976</v>
       </c>
       <c r="K105" s="28">
         <f t="shared" si="11"/>
-        <v>976</v>
+        <v>0</v>
       </c>
       <c r="L105" s="28" t="s">
         <v>148</v>
@@ -22061,10 +22170,10 @@
         <v>1600</v>
       </c>
       <c r="F106" s="31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G106" s="31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H106" s="30">
         <f t="shared" si="9"/>
@@ -22076,18 +22185,18 @@
       </c>
       <c r="J106" s="30">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>976</v>
       </c>
       <c r="K106" s="30">
         <f t="shared" si="11"/>
-        <v>976</v>
+        <v>0</v>
       </c>
       <c r="L106" s="30" t="s">
-        <v>261</v>
+        <v>714</v>
       </c>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
-        <v>222</v>
+        <v>122</v>
       </c>
       <c r="O106" s="30" t="s">
         <v>197</v>
@@ -22565,7 +22674,7 @@
         <v>3764.2799999999997</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22573,7 +22682,7 @@
       </c>
       <c r="O115" s="28"/>
       <c r="P115" s="89" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="Q115" s="28"/>
       <c r="R115" s="28"/>
@@ -22619,7 +22728,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -22627,7 +22736,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -22725,7 +22834,7 @@
         <v>1047.9000000000001</v>
       </c>
       <c r="L118" s="30" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="M118" s="30"/>
       <c r="N118" s="30" t="s">
@@ -22733,7 +22842,7 @@
       </c>
       <c r="O118" s="30"/>
       <c r="P118" s="30" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="Q118" s="30"/>
       <c r="R118" s="30"/>
@@ -22919,10 +23028,10 @@
         <v>1600</v>
       </c>
       <c r="F122" s="31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G122" s="31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H122" s="30">
         <f t="shared" si="9"/>
@@ -22934,21 +23043,21 @@
       </c>
       <c r="J122" s="30">
         <f t="shared" si="10"/>
-        <v>1175</v>
+        <v>2350</v>
       </c>
       <c r="K122" s="30">
         <f t="shared" si="11"/>
-        <v>3525</v>
+        <v>2350</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>537</v>
+        <v>715</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>538</v>
+        <v>716</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -22995,7 +23104,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23047,7 +23156,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="84" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="M124" s="84"/>
       <c r="N124" s="84" t="s">
@@ -23101,7 +23210,7 @@
         <v>1816.5</v>
       </c>
       <c r="L125" s="81" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="M125" s="81"/>
       <c r="N125" s="81" t="s">
@@ -23121,7 +23230,7 @@
         <v>467</v>
       </c>
       <c r="B126" s="30" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C126" s="30" t="s">
         <v>135</v>
@@ -23160,7 +23269,7 @@
         <v>191</v>
       </c>
       <c r="O126" s="30" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="P126" s="30"/>
       <c r="Q126" s="30"/>
@@ -23173,7 +23282,7 @@
         <v>468</v>
       </c>
       <c r="B127" s="28" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C127" s="28" t="s">
         <v>135</v>
@@ -23207,7 +23316,7 @@
         <v>0</v>
       </c>
       <c r="L127" s="28" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="M127" s="28"/>
       <c r="N127" s="28" t="s">
@@ -23227,7 +23336,7 @@
         <v>469</v>
       </c>
       <c r="B128" s="30" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C128" s="30" t="s">
         <v>120</v>
@@ -23277,7 +23386,7 @@
         <v>470</v>
       </c>
       <c r="B129" s="28" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C129" s="28" t="s">
         <v>120</v>
@@ -23327,7 +23436,7 @@
         <v>471</v>
       </c>
       <c r="B130" s="30" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C130" s="30" t="s">
         <v>120</v>
@@ -23377,7 +23486,7 @@
         <v>472</v>
       </c>
       <c r="B131" s="28" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="C131" s="28" t="s">
         <v>120</v>
@@ -23427,7 +23536,7 @@
         <v>473</v>
       </c>
       <c r="B132" s="30" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C132" s="30" t="s">
         <v>120</v>
@@ -23461,7 +23570,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -23479,7 +23588,7 @@
         <v>474</v>
       </c>
       <c r="B133" s="28" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>120</v>
@@ -23529,7 +23638,7 @@
         <v>475</v>
       </c>
       <c r="B134" s="30" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="C134" s="30" t="s">
         <v>120</v>
@@ -23579,7 +23688,7 @@
         <v>476</v>
       </c>
       <c r="B135" s="28" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="C135" s="28" t="s">
         <v>120</v>
@@ -23591,10 +23700,10 @@
         <v>850</v>
       </c>
       <c r="F135" s="82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G135" s="82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H135" s="80">
         <f t="shared" si="15"/>
@@ -23606,16 +23715,18 @@
       </c>
       <c r="J135" s="81">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="K135" s="81">
         <f t="shared" si="17"/>
-        <v>450</v>
-      </c>
-      <c r="L135" s="28"/>
+        <v>0</v>
+      </c>
+      <c r="L135" s="28" t="s">
+        <v>711</v>
+      </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
-        <v>222</v>
+        <v>122</v>
       </c>
       <c r="O135" s="28"/>
       <c r="P135" s="28"/>
@@ -23626,10 +23737,10 @@
     </row>
     <row r="136" spans="1:20" ht="15">
       <c r="A136" s="83" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B136" s="30" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="C136" s="30" t="s">
         <v>120</v>
@@ -23663,7 +23774,7 @@
         <v>1816</v>
       </c>
       <c r="L136" s="30" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="M136" s="30"/>
       <c r="N136" s="30" t="s">
@@ -23671,7 +23782,7 @@
       </c>
       <c r="O136" s="30"/>
       <c r="P136" s="30" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="Q136" s="30"/>
       <c r="R136" s="30"/>
@@ -23680,10 +23791,10 @@
     </row>
     <row r="137" spans="1:20" ht="15">
       <c r="A137" s="80" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B137" s="28" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C137" s="28" t="s">
         <v>120</v>
@@ -23732,10 +23843,10 @@
     </row>
     <row r="138" spans="1:20" ht="15">
       <c r="A138" s="83" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B138" s="30" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C138" s="30" t="s">
         <v>120</v>
@@ -23782,10 +23893,10 @@
     </row>
     <row r="139" spans="1:20" ht="15">
       <c r="A139" s="80" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B139" s="28" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="C139" s="28" t="s">
         <v>120</v>
@@ -23819,7 +23930,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -23834,10 +23945,10 @@
     </row>
     <row r="140" spans="1:20" ht="15">
       <c r="A140" s="83" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B140" s="30" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C140" s="30" t="s">
         <v>120</v>
@@ -23849,10 +23960,10 @@
         <v>1100</v>
       </c>
       <c r="F140" s="85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G140" s="85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H140" s="86">
         <f t="shared" si="18"/>
@@ -23864,16 +23975,18 @@
       </c>
       <c r="J140" s="84">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>699</v>
       </c>
       <c r="K140" s="84">
         <f t="shared" si="20"/>
-        <v>1398</v>
-      </c>
-      <c r="L140" s="30"/>
+        <v>699</v>
+      </c>
+      <c r="L140" s="30" t="s">
+        <v>710</v>
+      </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="O140" s="30"/>
       <c r="P140" s="30"/>
@@ -23884,10 +23997,10 @@
     </row>
     <row r="141" spans="1:20" ht="15">
       <c r="A141" s="80" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B141" s="28" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C141" s="28" t="s">
         <v>120</v>
@@ -23934,10 +24047,10 @@
     </row>
     <row r="142" spans="1:20" ht="30">
       <c r="A142" s="30" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B142" s="30" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="C142" s="30" t="s">
         <v>120</v>
@@ -23971,7 +24084,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -23988,10 +24101,10 @@
     </row>
     <row r="143" spans="1:20" ht="15">
       <c r="A143" s="28" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B143" s="28" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C143" s="28" t="s">
         <v>120</v>
@@ -24038,10 +24151,10 @@
     </row>
     <row r="144" spans="1:20" ht="15">
       <c r="A144" s="30" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B144" s="30" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C144" s="30" t="s">
         <v>120</v>
@@ -24088,10 +24201,10 @@
     </row>
     <row r="145" spans="1:20" ht="15">
       <c r="A145" s="28" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B145" s="28" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C145" s="28" t="s">
         <v>120</v>
@@ -24125,7 +24238,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24140,10 +24253,10 @@
     </row>
     <row r="146" spans="1:20" ht="30">
       <c r="A146" s="30" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B146" s="30" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="C146" s="30" t="s">
         <v>120</v>
@@ -24190,10 +24303,10 @@
     </row>
     <row r="147" spans="1:20" ht="15">
       <c r="A147" s="28" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24240,10 +24353,10 @@
     </row>
     <row r="148" spans="1:20" ht="15">
       <c r="A148" s="30" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B148" s="30" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="C148" s="30" t="s">
         <v>120</v>
@@ -24292,10 +24405,10 @@
     </row>
     <row r="149" spans="1:20" ht="15">
       <c r="A149" s="28" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B149" s="28" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C149" s="28" t="s">
         <v>120</v>
@@ -24342,10 +24455,10 @@
     </row>
     <row r="150" spans="1:20" ht="15">
       <c r="A150" s="30" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B150" s="30" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C150" s="30" t="s">
         <v>120</v>
@@ -24392,10 +24505,10 @@
     </row>
     <row r="151" spans="1:20" ht="15">
       <c r="A151" s="28" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B151" s="28" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C151" s="28" t="s">
         <v>135</v>
@@ -24434,10 +24547,10 @@
         <v>222</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="P151" s="28" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="Q151" s="28"/>
       <c r="R151" s="28"/>
@@ -24446,10 +24559,10 @@
     </row>
     <row r="152" spans="1:20" ht="15">
       <c r="A152" s="30" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B152" s="30" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="C152" s="30" t="s">
         <v>248</v>
@@ -24483,17 +24596,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="30" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="M152" s="30"/>
       <c r="N152" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O152" s="30" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="P152" s="30" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="Q152" s="30"/>
       <c r="R152" s="30"/>
@@ -24502,10 +24615,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="28" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B153" s="28" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C153" s="28" t="s">
         <v>120</v>
@@ -24545,7 +24658,7 @@
       </c>
       <c r="O153" s="28"/>
       <c r="P153" s="28" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="Q153" s="28"/>
       <c r="R153" s="28"/>
@@ -25156,15 +25269,15 @@
       </c>
       <c r="B8" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>97424</v>
+        <v>103752</v>
       </c>
       <c r="C8" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D8" s="6">
         <f>B8-C8</f>
-        <v>11717.666666666672</v>
+        <v>14881.666666666672</v>
       </c>
       <c r="E8" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE),0)</f>
@@ -25172,7 +25285,7 @@
       </c>
       <c r="F8" s="6">
         <f>D8+E8</f>
-        <v>11717.666666666672</v>
+        <v>14881.666666666672</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -25180,7 +25293,7 @@
       </c>
       <c r="H8" s="8">
         <f>F8-G8</f>
-        <v>-1596.3333333333285</v>
+        <v>1567.6666666666715</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -25193,11 +25306,11 @@
       </c>
       <c r="C9" s="7">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D9" s="7">
         <f>B9-C9</f>
-        <v>48475.666666666672</v>
+        <v>45311.666666666672</v>
       </c>
       <c r="E9" s="7">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE),0)</f>
@@ -25205,7 +25318,7 @@
       </c>
       <c r="F9" s="7">
         <f>D9+E9</f>
-        <v>48475.666666666672</v>
+        <v>45311.666666666672</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -25213,7 +25326,7 @@
       </c>
       <c r="H9" s="9">
         <f>F9-G9</f>
-        <v>1903.006666666668</v>
+        <v>-1260.993333333332</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -25222,11 +25335,11 @@
       </c>
       <c r="B10" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A10,Purchases!$C:$C),0)</f>
-        <v>25513</v>
+        <v>28677</v>
       </c>
       <c r="C10" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>85706.333333333328</v>
+        <v>88870.333333333328</v>
       </c>
       <c r="D10" s="6">
         <f>B10-C10</f>
@@ -25599,7 +25712,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>211415</v>
+        <v>213365</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -25607,11 +25720,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>76870.037599999996</v>
+        <v>77520.167600000001</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>134544.96240000002</v>
+        <v>135844.83240000001</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25619,7 +25732,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>10491.486400000023</v>
+        <v>11791.356400000019</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -25636,11 +25749,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>76823.924799999993</v>
+        <v>77473.664799999999</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-70204.924799999993</v>
+        <v>-70854.664799999999</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25648,7 +25761,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-5243.9727999999886</v>
+        <v>-5893.7127999999939</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -25665,11 +25778,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>76870.037599999996</v>
+        <v>77520.167600000001</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-64340.037599999996</v>
+        <v>-64990.167600000001</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25677,7 +25790,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-5247.5135999999911</v>
+        <v>-5897.6435999999958</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
Chikkankari L sale and zinfab purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944C5450-1DDE-814E-A630-AB3FE64FE254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AECEB8D-E683-1B4D-8BEA-726641C37BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="721">
   <si>
     <t>Notes:</t>
   </si>
@@ -1949,9 +1949,6 @@
   </si>
   <si>
     <t>Purple</t>
-  </si>
-  <si>
-    <t>M,L,Xl,XXL</t>
   </si>
   <si>
     <t>CHR-151</t>
@@ -2239,6 +2236,18 @@
   </si>
   <si>
     <t>Roman Silk(XXL), Coral Pink (XXL)</t>
+  </si>
+  <si>
+    <t>Praneetha (Kochi)</t>
+  </si>
+  <si>
+    <t>Chikkankari(L)</t>
+  </si>
+  <si>
+    <t>Praneetha (L)</t>
+  </si>
+  <si>
+    <t>M,Xl,XXL</t>
   </si>
 </sst>
 </file>
@@ -3001,7 +3010,7 @@
                   <c:v>4790</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9492</c:v>
+                  <c:v>11692</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3119,7 +3128,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5400</c:v>
+                  <c:v>6499</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3374,7 +3383,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-4092</c:v>
+                  <c:v>-5193</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -7872,7 +7881,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(Purchases!C:C)</f>
-        <v>266611</v>
+        <v>268811</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>39</v>
@@ -7887,7 +7896,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>232514</v>
+        <v>233613</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7904,7 +7913,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>235964</v>
+        <v>237063</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -7921,7 +7930,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-34097</v>
+        <v>-35198</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -7956,7 +7965,7 @@
       </c>
       <c r="B10" s="52">
         <f>PartnerShares!H8</f>
-        <v>1567.6666666666715</v>
+        <v>2334.3333333333285</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -7966,7 +7975,7 @@
       </c>
       <c r="B11" s="53">
         <f>PartnerShares!H9</f>
-        <v>-1260.993333333332</v>
+        <v>-1994.326666666675</v>
       </c>
       <c r="C11" s="7"/>
     </row>
@@ -7976,7 +7985,7 @@
       </c>
       <c r="B12" s="52">
         <f>PartnerShares!H10</f>
-        <v>-306.67333333332499</v>
+        <v>-340.00666666666802</v>
       </c>
       <c r="C12" s="6"/>
     </row>
@@ -8015,15 +8024,15 @@
       </c>
       <c r="B18" s="6">
         <f>PartnerShares!B8</f>
-        <v>103752</v>
+        <v>105252</v>
       </c>
       <c r="C18" s="6">
         <f>PartnerShares!C8</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D18" s="6">
         <f>PartnerShares!D8</f>
-        <v>14881.666666666672</v>
+        <v>15648.333333333328</v>
       </c>
       <c r="E18" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8031,10 +8040,10 @@
       </c>
       <c r="F18" s="8">
         <f>D18-E18</f>
-        <v>1567.6666666666715</v>
+        <v>2334.3333333333285</v>
       </c>
       <c r="G18" s="73" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8048,11 +8057,11 @@
       </c>
       <c r="C19" s="7">
         <f>PartnerShares!C9</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D19" s="7">
         <f>PartnerShares!D9</f>
-        <v>45311.666666666672</v>
+        <v>44578.333333333328</v>
       </c>
       <c r="E19" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8060,10 +8069,10 @@
       </c>
       <c r="F19" s="9">
         <f>D19-E19</f>
-        <v>-1260.993333333332</v>
+        <v>-1994.326666666675</v>
       </c>
       <c r="G19" s="71" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -8073,15 +8082,15 @@
       </c>
       <c r="B20" s="6">
         <f>PartnerShares!B10</f>
-        <v>28677</v>
+        <v>29377</v>
       </c>
       <c r="C20" s="6">
         <f>PartnerShares!C10</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D20" s="6">
         <f>PartnerShares!D10</f>
-        <v>-60193.333333333328</v>
+        <v>-60226.666666666672</v>
       </c>
       <c r="E20" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8089,10 +8098,10 @@
       </c>
       <c r="F20" s="8">
         <f>D20-E20</f>
-        <v>-306.67333333332499</v>
+        <v>-340.00666666666802</v>
       </c>
       <c r="G20" s="71" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1">
@@ -8130,15 +8139,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>213365</v>
+        <v>214464</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>77520.167600000001</v>
+        <v>77886.574199999988</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>135844.83240000001</v>
+        <v>136577.42580000003</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8146,10 +8155,10 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>11791.356400000019</v>
+        <v>12523.949800000031</v>
       </c>
       <c r="G26" s="71" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -8163,11 +8172,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>77473.664799999999</v>
+        <v>77839.851599999995</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-70854.664799999999</v>
+        <v>-71220.851599999995</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8175,10 +8184,10 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-5893.7127999999939</v>
+        <v>-6259.8995999999897</v>
       </c>
       <c r="G27" s="72" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -8192,11 +8201,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>77520.167600000001</v>
+        <v>77886.574199999988</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-64990.167600000001</v>
+        <v>-65356.574199999988</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8204,10 +8213,10 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-5897.6435999999958</v>
+        <v>-6264.0501999999833</v>
       </c>
       <c r="G28" s="73" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1">
@@ -8304,7 +8313,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46090</v>
+        <v>46091</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8313,14 +8322,14 @@
       </c>
       <c r="B5" s="15">
         <f>Summary!B3</f>
-        <v>266611</v>
+        <v>268811</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>232514</v>
+        <v>233613</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8329,7 +8338,7 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-34097</v>
+        <v>-35198</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
@@ -8413,15 +8422,15 @@
       </c>
       <c r="B12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A12)*Purchases!$C$2:$C$998),0)</f>
-        <v>9492</v>
+        <v>11692</v>
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>5400</v>
+        <v>6499</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-4092</v>
+        <v>-5193</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -9395,7 +9404,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9410,7 +9419,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -9424,7 +9433,7 @@
         <v>6328</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -9438,26 +9447,50 @@
         <v>3164</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="52" spans="1:4">
-      <c r="A52" s="41"/>
-      <c r="B52" s="39"/>
-      <c r="C52" s="40"/>
-      <c r="D52" s="39"/>
+      <c r="A52" s="41">
+        <v>46090</v>
+      </c>
+      <c r="B52" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="C52" s="40">
+        <v>100</v>
+      </c>
+      <c r="D52" s="39" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="53" spans="1:4">
-      <c r="A53" s="36"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="38"/>
-      <c r="D53" s="37"/>
+      <c r="A53" s="36">
+        <v>46091</v>
+      </c>
+      <c r="B53" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="C53" s="38">
+        <v>1400</v>
+      </c>
+      <c r="D53" s="37" t="s">
+        <v>614</v>
+      </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="41"/>
-      <c r="B54" s="39"/>
-      <c r="C54" s="40"/>
-      <c r="D54" s="39"/>
+      <c r="A54" s="41">
+        <v>46091</v>
+      </c>
+      <c r="B54" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C54" s="40">
+        <v>700</v>
+      </c>
+      <c r="D54" s="39" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="36"/>
@@ -14293,7 +14326,7 @@
         <v>46046</v>
       </c>
       <c r="B102" s="50" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C102" s="51">
         <v>950</v>
@@ -14307,7 +14340,7 @@
       <c r="F102" s="50"/>
       <c r="G102" s="50"/>
       <c r="H102" s="69" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="I102" s="50" t="s">
         <v>276</v>
@@ -14318,7 +14351,7 @@
         <v>46048</v>
       </c>
       <c r="B103" s="47" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="C103" s="48">
         <v>1380</v>
@@ -14343,7 +14376,7 @@
         <v>46048</v>
       </c>
       <c r="B104" s="50" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C104" s="51">
         <v>2700</v>
@@ -14357,7 +14390,7 @@
       <c r="F104" s="50"/>
       <c r="G104" s="50"/>
       <c r="H104" s="69" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="I104" s="50" t="s">
         <v>276</v>
@@ -14368,7 +14401,7 @@
         <v>46049</v>
       </c>
       <c r="B105" s="47" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C105" s="48">
         <v>1380</v>
@@ -14393,7 +14426,7 @@
         <v>46049</v>
       </c>
       <c r="B106" s="50" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="C106" s="51">
         <v>1380</v>
@@ -14407,7 +14440,7 @@
       <c r="F106" s="50"/>
       <c r="G106" s="50"/>
       <c r="H106" s="69" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="I106" s="50" t="s">
         <v>276</v>
@@ -14418,7 +14451,7 @@
         <v>46049</v>
       </c>
       <c r="B107" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C107" s="48">
         <v>1200</v>
@@ -14432,7 +14465,7 @@
       <c r="F107" s="49"/>
       <c r="G107" s="49"/>
       <c r="H107" s="68" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="I107" s="47" t="s">
         <v>276</v>
@@ -14443,7 +14476,7 @@
         <v>46050</v>
       </c>
       <c r="B108" s="50" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C108" s="51">
         <v>1250</v>
@@ -14457,7 +14490,7 @@
       <c r="F108" s="50"/>
       <c r="G108" s="50"/>
       <c r="H108" s="69" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="I108" s="50" t="s">
         <v>276</v>
@@ -14468,7 +14501,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14493,7 +14526,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14524,7 +14557,7 @@
         <v>580</v>
       </c>
       <c r="D111" s="47" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E111" s="47" t="s">
         <v>48</v>
@@ -14532,7 +14565,7 @@
       <c r="F111" s="49"/>
       <c r="G111" s="49"/>
       <c r="H111" s="68" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="I111" s="47" t="s">
         <v>276</v>
@@ -14543,7 +14576,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14557,7 +14590,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14568,7 +14601,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14632,7 +14665,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14643,7 +14676,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14657,7 +14690,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14668,7 +14701,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14693,7 +14726,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14718,7 +14751,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14743,13 +14776,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14782,7 +14815,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14793,7 +14826,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14807,7 +14840,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14818,7 +14851,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -14843,7 +14876,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -14857,7 +14890,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -14882,7 +14915,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -14893,7 +14926,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -14907,7 +14940,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -14918,7 +14951,7 @@
         <v>46090</v>
       </c>
       <c r="B127" s="47" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C127" s="48">
         <v>850</v>
@@ -14932,7 +14965,7 @@
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
       <c r="H127" s="28" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="I127" s="47" t="s">
         <v>276</v>
@@ -14943,7 +14976,7 @@
         <v>46090</v>
       </c>
       <c r="B128" s="50" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C128" s="51">
         <v>1100</v>
@@ -14957,7 +14990,7 @@
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
       <c r="H128" s="69" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="I128" s="50" t="s">
         <v>276</v>
@@ -14968,7 +15001,7 @@
         <v>46090</v>
       </c>
       <c r="B129" s="47" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C129" s="48">
         <v>1200</v>
@@ -14982,7 +15015,7 @@
       <c r="F129" s="49"/>
       <c r="G129" s="49"/>
       <c r="H129" s="68" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="I129" s="47" t="s">
         <v>191</v>
@@ -14993,7 +15026,7 @@
         <v>46090</v>
       </c>
       <c r="B130" s="50" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C130" s="51">
         <v>2250</v>
@@ -15007,22 +15040,36 @@
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
       <c r="H130" s="69" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="I130" s="50" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="131" spans="1:9">
-      <c r="A131" s="46"/>
-      <c r="B131" s="47"/>
-      <c r="C131" s="48"/>
-      <c r="D131" s="47"/>
-      <c r="E131" s="47"/>
+    <row r="131" spans="1:9" ht="16">
+      <c r="A131" s="46">
+        <v>46091</v>
+      </c>
+      <c r="B131" s="47" t="s">
+        <v>717</v>
+      </c>
+      <c r="C131" s="48">
+        <v>1099</v>
+      </c>
+      <c r="D131" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E131" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="F131" s="49"/>
       <c r="G131" s="49"/>
-      <c r="H131" s="68"/>
-      <c r="I131" s="47"/>
+      <c r="H131" s="68" t="s">
+        <v>718</v>
+      </c>
+      <c r="I131" s="47" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="132" spans="1:9">
       <c r="A132" s="43"/>
@@ -19308,7 +19355,7 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
@@ -19364,7 +19411,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19374,7 +19421,7 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
@@ -19476,7 +19523,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19748,7 +19795,7 @@
         <v>1080</v>
       </c>
       <c r="L60" s="30" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="M60" s="30" t="s">
         <v>46</v>
@@ -19858,7 +19905,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -20270,7 +20317,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -20920,7 +20967,7 @@
         <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
@@ -21080,7 +21127,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21134,7 +21181,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21396,7 +21443,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21448,7 +21495,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -22192,7 +22239,7 @@
         <v>0</v>
       </c>
       <c r="L106" s="30" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
@@ -22674,7 +22721,7 @@
         <v>3764.2799999999997</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22682,7 +22729,7 @@
       </c>
       <c r="O115" s="28"/>
       <c r="P115" s="89" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="Q115" s="28"/>
       <c r="R115" s="28"/>
@@ -22728,7 +22775,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -22736,7 +22783,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -23050,14 +23097,14 @@
         <v>2350</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -23104,7 +23151,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23486,7 +23533,7 @@
         <v>472</v>
       </c>
       <c r="B131" s="28" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C131" s="28" t="s">
         <v>120</v>
@@ -23570,7 +23617,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -23588,7 +23635,7 @@
         <v>474</v>
       </c>
       <c r="B133" s="28" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>120</v>
@@ -23638,7 +23685,7 @@
         <v>475</v>
       </c>
       <c r="B134" s="30" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C134" s="30" t="s">
         <v>120</v>
@@ -23688,7 +23735,7 @@
         <v>476</v>
       </c>
       <c r="B135" s="28" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C135" s="28" t="s">
         <v>120</v>
@@ -23722,7 +23769,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="28" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
@@ -23774,7 +23821,7 @@
         <v>1816</v>
       </c>
       <c r="L136" s="30" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="M136" s="30"/>
       <c r="N136" s="30" t="s">
@@ -23782,7 +23829,7 @@
       </c>
       <c r="O136" s="30"/>
       <c r="P136" s="30" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="Q136" s="30"/>
       <c r="R136" s="30"/>
@@ -23930,7 +23977,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -23982,7 +24029,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="30" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
@@ -24084,7 +24131,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -24154,7 +24201,7 @@
         <v>601</v>
       </c>
       <c r="B144" s="30" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="C144" s="30" t="s">
         <v>120</v>
@@ -24238,7 +24285,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24251,12 +24298,12 @@
       <c r="S145" s="28"/>
       <c r="T145" s="28"/>
     </row>
-    <row r="146" spans="1:20" ht="30">
+    <row r="146" spans="1:20" ht="15">
       <c r="A146" s="30" t="s">
         <v>617</v>
       </c>
       <c r="B146" s="30" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C146" s="30" t="s">
         <v>120</v>
@@ -24306,7 +24353,7 @@
         <v>618</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24356,7 +24403,7 @@
         <v>619</v>
       </c>
       <c r="B148" s="30" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="C148" s="30" t="s">
         <v>120</v>
@@ -24408,7 +24455,7 @@
         <v>620</v>
       </c>
       <c r="B149" s="28" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C149" s="28" t="s">
         <v>120</v>
@@ -24458,7 +24505,7 @@
         <v>621</v>
       </c>
       <c r="B150" s="30" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C150" s="30" t="s">
         <v>120</v>
@@ -24541,13 +24588,15 @@
         <f t="shared" ref="K151:K152" si="32">IF(LEN(G151)=0,0,G151)*I151</f>
         <v>2580</v>
       </c>
-      <c r="L151" s="28"/>
+      <c r="L151" s="28" t="s">
+        <v>719</v>
+      </c>
       <c r="M151" s="28"/>
       <c r="N151" s="28" t="s">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>625</v>
+        <v>720</v>
       </c>
       <c r="P151" s="28" t="s">
         <v>624</v>
@@ -24559,10 +24608,10 @@
     </row>
     <row r="152" spans="1:20" ht="15">
       <c r="A152" s="30" t="s">
+        <v>625</v>
+      </c>
+      <c r="B152" s="30" t="s">
         <v>626</v>
-      </c>
-      <c r="B152" s="30" t="s">
-        <v>627</v>
       </c>
       <c r="C152" s="30" t="s">
         <v>248</v>
@@ -24596,17 +24645,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="M152" s="30"/>
       <c r="N152" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O152" s="30" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="P152" s="30" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="Q152" s="30"/>
       <c r="R152" s="30"/>
@@ -24615,10 +24664,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="28" t="s">
+        <v>648</v>
+      </c>
+      <c r="B153" s="28" t="s">
         <v>649</v>
-      </c>
-      <c r="B153" s="28" t="s">
-        <v>650</v>
       </c>
       <c r="C153" s="28" t="s">
         <v>120</v>
@@ -24658,7 +24707,7 @@
       </c>
       <c r="O153" s="28"/>
       <c r="P153" s="28" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="Q153" s="28"/>
       <c r="R153" s="28"/>
@@ -25269,15 +25318,15 @@
       </c>
       <c r="B8" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>103752</v>
+        <v>105252</v>
       </c>
       <c r="C8" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D8" s="6">
         <f>B8-C8</f>
-        <v>14881.666666666672</v>
+        <v>15648.333333333328</v>
       </c>
       <c r="E8" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE),0)</f>
@@ -25285,7 +25334,7 @@
       </c>
       <c r="F8" s="6">
         <f>D8+E8</f>
-        <v>14881.666666666672</v>
+        <v>15648.333333333328</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -25293,7 +25342,7 @@
       </c>
       <c r="H8" s="8">
         <f>F8-G8</f>
-        <v>1567.6666666666715</v>
+        <v>2334.3333333333285</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -25306,11 +25355,11 @@
       </c>
       <c r="C9" s="7">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D9" s="7">
         <f>B9-C9</f>
-        <v>45311.666666666672</v>
+        <v>44578.333333333328</v>
       </c>
       <c r="E9" s="7">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE),0)</f>
@@ -25318,7 +25367,7 @@
       </c>
       <c r="F9" s="7">
         <f>D9+E9</f>
-        <v>45311.666666666672</v>
+        <v>44578.333333333328</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -25326,7 +25375,7 @@
       </c>
       <c r="H9" s="9">
         <f>F9-G9</f>
-        <v>-1260.993333333332</v>
+        <v>-1994.326666666675</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -25335,15 +25384,15 @@
       </c>
       <c r="B10" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A10,Purchases!$C:$C),0)</f>
-        <v>28677</v>
+        <v>29377</v>
       </c>
       <c r="C10" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>88870.333333333328</v>
+        <v>89603.666666666672</v>
       </c>
       <c r="D10" s="6">
         <f>B10-C10</f>
-        <v>-60193.333333333328</v>
+        <v>-60226.666666666672</v>
       </c>
       <c r="E10" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE),0)</f>
@@ -25351,7 +25400,7 @@
       </c>
       <c r="F10" s="6">
         <f>D10+E10</f>
-        <v>-60193.333333333328</v>
+        <v>-60226.666666666672</v>
       </c>
       <c r="G10" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -25359,7 +25408,7 @@
       </c>
       <c r="H10" s="8">
         <f>F10-G10</f>
-        <v>-306.67333333332499</v>
+        <v>-340.00666666666802</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="22" customFormat="1" ht="16" customHeight="1">
@@ -25712,7 +25761,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>213365</v>
+        <v>214464</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -25720,11 +25769,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>77520.167600000001</v>
+        <v>77886.574199999988</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>135844.83240000001</v>
+        <v>136577.42580000003</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25732,7 +25781,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>11791.356400000019</v>
+        <v>12523.949800000031</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -25749,11 +25798,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>77473.664799999999</v>
+        <v>77839.851599999995</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-70854.664799999999</v>
+        <v>-71220.851599999995</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25761,7 +25810,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-5893.7127999999939</v>
+        <v>-6259.8995999999897</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -25778,11 +25827,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>77520.167600000001</v>
+        <v>77886.574199999988</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-64990.167600000001</v>
+        <v>-65356.574199999988</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25790,7 +25839,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-5897.6435999999958</v>
+        <v>-6264.0501999999833</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
3/11 sales and purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AECEB8D-E683-1B4D-8BEA-726641C37BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CCAAC73-E0F3-BB4E-9AE5-871784BABD2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1808" uniqueCount="725">
   <si>
     <t>Notes:</t>
   </si>
@@ -1997,9 +1997,6 @@
   </si>
   <si>
     <t>Soft Cotton Saree (with butterfly design on Pallu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linen Saree (Mustard/gree, Blue/Green, Blue/Red) </t>
   </si>
   <si>
     <t>Linen Saree with Check (Maroon with golden checks, Green with golden checks, Rust Orange with golden checks)</t>
@@ -2244,10 +2241,25 @@
     <t>Chikkankari(L)</t>
   </si>
   <si>
-    <t>Praneetha (L)</t>
-  </si>
-  <si>
     <t>M,Xl,XXL</t>
+  </si>
+  <si>
+    <t>Matka silk - Blue (500 transferred)</t>
+  </si>
+  <si>
+    <t>Rameez Cousin</t>
+  </si>
+  <si>
+    <t>Chikkankari(M)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matka Silk Saree (Mustard/gree, Blue/Green, Blue/Red) </t>
+  </si>
+  <si>
+    <t>Blue - Sarany Hyd (Adv-500)</t>
+  </si>
+  <si>
+    <t>Praneetha (L), Rameez Cousin (M)</t>
   </si>
 </sst>
 </file>
@@ -3010,7 +3022,7 @@
                   <c:v>4790</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11692</c:v>
+                  <c:v>20082</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3128,7 +3140,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6499</c:v>
+                  <c:v>8798</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3383,7 +3395,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-5193</c:v>
+                  <c:v>-11284</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3706,10 +3718,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>182</c:v>
+                  <c:v>185</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>103</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4018,10 +4030,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>108</c:v>
+                  <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>72</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4141,10 +4153,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>50</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>48</c:v>
+                  <c:v>46</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4571,10 +4583,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>53077</c:v>
+                  <c:v>51787</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>42425.18</c:v>
+                  <c:v>41706.18</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -7881,7 +7893,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(Purchases!C:C)</f>
-        <v>268811</v>
+        <v>277201</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>39</v>
@@ -7896,7 +7908,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>233613</v>
+        <v>234712</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7913,7 +7925,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>237063</v>
+        <v>239362</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -7930,7 +7942,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-35198</v>
+        <v>-42489</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -7965,7 +7977,7 @@
       </c>
       <c r="B10" s="52">
         <f>PartnerShares!H8</f>
-        <v>2334.3333333333285</v>
+        <v>5131.6666666666715</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -7975,7 +7987,7 @@
       </c>
       <c r="B11" s="53">
         <f>PartnerShares!H9</f>
-        <v>-1994.326666666675</v>
+        <v>-4790.993333333332</v>
       </c>
       <c r="C11" s="7"/>
     </row>
@@ -7985,7 +7997,7 @@
       </c>
       <c r="B12" s="52">
         <f>PartnerShares!H10</f>
-        <v>-340.00666666666802</v>
+        <v>-340.67333333332499</v>
       </c>
       <c r="C12" s="6"/>
     </row>
@@ -8024,15 +8036,15 @@
       </c>
       <c r="B18" s="6">
         <f>PartnerShares!B8</f>
-        <v>105252</v>
+        <v>110846</v>
       </c>
       <c r="C18" s="6">
         <f>PartnerShares!C8</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D18" s="6">
         <f>PartnerShares!D8</f>
-        <v>15648.333333333328</v>
+        <v>18445.666666666672</v>
       </c>
       <c r="E18" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8040,10 +8052,10 @@
       </c>
       <c r="F18" s="8">
         <f>D18-E18</f>
-        <v>2334.3333333333285</v>
+        <v>5131.6666666666715</v>
       </c>
       <c r="G18" s="73" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8057,11 +8069,11 @@
       </c>
       <c r="C19" s="7">
         <f>PartnerShares!C9</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D19" s="7">
         <f>PartnerShares!D9</f>
-        <v>44578.333333333328</v>
+        <v>41781.666666666672</v>
       </c>
       <c r="E19" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8069,10 +8081,10 @@
       </c>
       <c r="F19" s="9">
         <f>D19-E19</f>
-        <v>-1994.326666666675</v>
+        <v>-4790.993333333332</v>
       </c>
       <c r="G19" s="71" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -8082,15 +8094,15 @@
       </c>
       <c r="B20" s="6">
         <f>PartnerShares!B10</f>
-        <v>29377</v>
+        <v>32173</v>
       </c>
       <c r="C20" s="6">
         <f>PartnerShares!C10</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D20" s="6">
         <f>PartnerShares!D10</f>
-        <v>-60226.666666666672</v>
+        <v>-60227.333333333328</v>
       </c>
       <c r="E20" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8098,10 +8110,10 @@
       </c>
       <c r="F20" s="8">
         <f>D20-E20</f>
-        <v>-340.00666666666802</v>
+        <v>-340.67333333332499</v>
       </c>
       <c r="G20" s="71" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" customHeight="1">
@@ -8139,15 +8151,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>214464</v>
+        <v>215563</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>77886.574199999988</v>
+        <v>78252.98079999999</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>136577.42580000003</v>
+        <v>137310.01920000001</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8155,10 +8167,10 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>12523.949800000031</v>
+        <v>13256.543200000015</v>
       </c>
       <c r="G26" s="71" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -8172,11 +8184,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>77839.851599999995</v>
+        <v>78206.038400000005</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-71220.851599999995</v>
+        <v>-71587.038400000005</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8184,10 +8196,10 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-6259.8995999999897</v>
+        <v>-6626.0864000000001</v>
       </c>
       <c r="G27" s="72" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -8201,11 +8213,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>77886.574199999988</v>
+        <v>78252.98079999999</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-65356.574199999988</v>
+        <v>-65722.98079999999</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8213,10 +8225,10 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-6264.0501999999833</v>
+        <v>-6630.4567999999854</v>
       </c>
       <c r="G28" s="73" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" customHeight="1">
@@ -8313,7 +8325,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46091</v>
+        <v>46092</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8322,14 +8334,14 @@
       </c>
       <c r="B5" s="15">
         <f>Summary!B3</f>
-        <v>268811</v>
+        <v>277201</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>233613</v>
+        <v>234712</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8338,14 +8350,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-35198</v>
+        <v>-42489</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>94434.68</v>
+        <v>92425.68</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8389,7 +8401,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8413,7 +8425,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8422,15 +8434,15 @@
       </c>
       <c r="B12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A12)*Purchases!$C$2:$C$998),0)</f>
-        <v>11692</v>
+        <v>20082</v>
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>6499</v>
+        <v>8798</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-5193</v>
+        <v>-11284</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8609,18 +8621,18 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
       </c>
       <c r="K47" s="77" cm="1">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$479=J47)*(INVENTORY!$D$2:$D$479)*(INVENTORY!$G$2:$G$479))</f>
-        <v>53077</v>
+        <v>51787</v>
       </c>
     </row>
     <row r="48" spans="6:11">
@@ -8629,18 +8641,18 @@
       </c>
       <c r="G48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J48" s="76" t="s">
         <v>120</v>
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$479=J48)*(INVENTORY!$D$2:$D$479)*(INVENTORY!$G$2:$G$479))</f>
-        <v>42425.18</v>
+        <v>41706.18</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9404,7 +9416,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9419,7 +9431,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -9433,7 +9445,7 @@
         <v>6328</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -9447,7 +9459,7 @@
         <v>3164</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -9489,20 +9501,36 @@
         <v>700</v>
       </c>
       <c r="D54" s="39" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="36">
+        <v>46092</v>
+      </c>
+      <c r="B55" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="C55" s="38">
+        <v>5594</v>
+      </c>
+      <c r="D55" s="37" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="41">
+        <v>46092</v>
+      </c>
+      <c r="B56" s="39" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="36"/>
-      <c r="B55" s="37"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="37"/>
-    </row>
-    <row r="56" spans="1:4">
-      <c r="A56" s="41"/>
-      <c r="B56" s="39"/>
-      <c r="C56" s="40"/>
-      <c r="D56" s="39"/>
+      <c r="C56" s="40">
+        <v>2796</v>
+      </c>
+      <c r="D56" s="39" t="s">
+        <v>700</v>
+      </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="36"/>
@@ -14401,7 +14429,7 @@
         <v>46049</v>
       </c>
       <c r="B105" s="47" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C105" s="48">
         <v>1380</v>
@@ -14426,7 +14454,7 @@
         <v>46049</v>
       </c>
       <c r="B106" s="50" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C106" s="51">
         <v>1380</v>
@@ -14440,7 +14468,7 @@
       <c r="F106" s="50"/>
       <c r="G106" s="50"/>
       <c r="H106" s="69" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I106" s="50" t="s">
         <v>276</v>
@@ -14451,7 +14479,7 @@
         <v>46049</v>
       </c>
       <c r="B107" s="47" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="C107" s="48">
         <v>1200</v>
@@ -14465,7 +14493,7 @@
       <c r="F107" s="49"/>
       <c r="G107" s="49"/>
       <c r="H107" s="68" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="I107" s="47" t="s">
         <v>276</v>
@@ -14476,7 +14504,7 @@
         <v>46050</v>
       </c>
       <c r="B108" s="50" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="C108" s="51">
         <v>1250</v>
@@ -14490,7 +14518,7 @@
       <c r="F108" s="50"/>
       <c r="G108" s="50"/>
       <c r="H108" s="69" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="I108" s="50" t="s">
         <v>276</v>
@@ -14501,7 +14529,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14526,7 +14554,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14557,7 +14585,7 @@
         <v>580</v>
       </c>
       <c r="D111" s="47" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E111" s="47" t="s">
         <v>48</v>
@@ -14565,7 +14593,7 @@
       <c r="F111" s="49"/>
       <c r="G111" s="49"/>
       <c r="H111" s="68" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="I111" s="47" t="s">
         <v>276</v>
@@ -14576,7 +14604,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14590,7 +14618,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14601,7 +14629,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14665,7 +14693,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14676,7 +14704,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14690,7 +14718,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14701,7 +14729,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14726,7 +14754,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14751,7 +14779,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14776,13 +14804,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14815,7 +14843,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14826,7 +14854,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14840,7 +14868,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14851,7 +14879,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -14876,7 +14904,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -14890,7 +14918,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -14915,7 +14943,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -14926,7 +14954,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -14940,7 +14968,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -14951,7 +14979,7 @@
         <v>46090</v>
       </c>
       <c r="B127" s="47" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C127" s="48">
         <v>850</v>
@@ -14965,7 +14993,7 @@
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
       <c r="H127" s="28" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="I127" s="47" t="s">
         <v>276</v>
@@ -14976,7 +15004,7 @@
         <v>46090</v>
       </c>
       <c r="B128" s="50" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C128" s="51">
         <v>1100</v>
@@ -14990,7 +15018,7 @@
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
       <c r="H128" s="69" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="I128" s="50" t="s">
         <v>276</v>
@@ -15001,7 +15029,7 @@
         <v>46090</v>
       </c>
       <c r="B129" s="47" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C129" s="48">
         <v>1200</v>
@@ -15015,7 +15043,7 @@
       <c r="F129" s="49"/>
       <c r="G129" s="49"/>
       <c r="H129" s="68" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="I129" s="47" t="s">
         <v>191</v>
@@ -15026,7 +15054,7 @@
         <v>46090</v>
       </c>
       <c r="B130" s="50" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C130" s="51">
         <v>2250</v>
@@ -15040,7 +15068,7 @@
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
       <c r="H130" s="69" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="I130" s="50" t="s">
         <v>191</v>
@@ -15051,7 +15079,7 @@
         <v>46091</v>
       </c>
       <c r="B131" s="47" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="C131" s="48">
         <v>1099</v>
@@ -15065,33 +15093,61 @@
       <c r="F131" s="49"/>
       <c r="G131" s="49"/>
       <c r="H131" s="68" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="I131" s="47" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="132" spans="1:9">
-      <c r="A132" s="43"/>
-      <c r="B132" s="50"/>
-      <c r="C132" s="51"/>
-      <c r="D132" s="50"/>
-      <c r="E132" s="50"/>
+      <c r="A132" s="43">
+        <v>46092</v>
+      </c>
+      <c r="B132" s="50" t="s">
+        <v>704</v>
+      </c>
+      <c r="C132" s="51">
+        <v>1200</v>
+      </c>
+      <c r="D132" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E132" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F132" s="50"/>
       <c r="G132" s="50"/>
-      <c r="H132" s="69"/>
-      <c r="I132" s="50"/>
-    </row>
-    <row r="133" spans="1:9">
-      <c r="A133" s="46"/>
-      <c r="B133" s="47"/>
-      <c r="C133" s="48"/>
-      <c r="D133" s="47"/>
-      <c r="E133" s="47"/>
+      <c r="H132" s="69" t="s">
+        <v>719</v>
+      </c>
+      <c r="I132" s="50" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" ht="16">
+      <c r="A133" s="46">
+        <v>46092</v>
+      </c>
+      <c r="B133" s="47" t="s">
+        <v>720</v>
+      </c>
+      <c r="C133" s="48">
+        <v>1099</v>
+      </c>
+      <c r="D133" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E133" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="F133" s="49"/>
       <c r="G133" s="49"/>
-      <c r="H133" s="68"/>
-      <c r="I133" s="47"/>
+      <c r="H133" s="68" t="s">
+        <v>721</v>
+      </c>
+      <c r="I133" s="47" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="134" spans="1:9">
       <c r="A134" s="43"/>
@@ -16539,7 +16595,7 @@
     <col min="11" max="11" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="43.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13" style="2" customWidth="1"/>
     <col min="15" max="15" width="13.83203125" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="41" style="2" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" style="2" bestFit="1" customWidth="1"/>
@@ -19355,7 +19411,7 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
@@ -19411,7 +19467,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19421,7 +19477,7 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
@@ -19523,7 +19579,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19795,7 +19851,7 @@
         <v>1080</v>
       </c>
       <c r="L60" s="30" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="M60" s="30" t="s">
         <v>46</v>
@@ -19905,7 +19961,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -20317,7 +20373,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -20967,7 +21023,7 @@
         <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
@@ -21127,7 +21183,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21181,7 +21237,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21443,7 +21499,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21495,7 +21551,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -22239,7 +22295,7 @@
         <v>0</v>
       </c>
       <c r="L106" s="30" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
@@ -22721,7 +22777,7 @@
         <v>3764.2799999999997</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22729,7 +22785,7 @@
       </c>
       <c r="O115" s="28"/>
       <c r="P115" s="89" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="Q115" s="28"/>
       <c r="R115" s="28"/>
@@ -22775,7 +22831,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -22783,7 +22839,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -23097,14 +23153,14 @@
         <v>2350</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -23151,7 +23207,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23617,7 +23673,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -23769,7 +23825,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="28" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
@@ -23821,7 +23877,7 @@
         <v>1816</v>
       </c>
       <c r="L136" s="30" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="M136" s="30"/>
       <c r="N136" s="30" t="s">
@@ -23829,7 +23885,7 @@
       </c>
       <c r="O136" s="30"/>
       <c r="P136" s="30" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="Q136" s="30"/>
       <c r="R136" s="30"/>
@@ -23977,7 +24033,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -24029,7 +24085,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="30" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
@@ -24131,7 +24187,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -24285,7 +24341,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24298,12 +24354,12 @@
       <c r="S145" s="28"/>
       <c r="T145" s="28"/>
     </row>
-    <row r="146" spans="1:20" ht="15">
+    <row r="146" spans="1:20" ht="30">
       <c r="A146" s="30" t="s">
         <v>617</v>
       </c>
       <c r="B146" s="30" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="C146" s="30" t="s">
         <v>120</v>
@@ -24353,7 +24409,7 @@
         <v>618</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>641</v>
+        <v>722</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24365,10 +24421,10 @@
         <v>1200</v>
       </c>
       <c r="F147" s="82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G147" s="82">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H147" s="80">
         <f t="shared" si="27"/>
@@ -24380,16 +24436,18 @@
       </c>
       <c r="J147" s="81">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>719</v>
       </c>
       <c r="K147" s="81">
         <f t="shared" si="29"/>
-        <v>2157</v>
-      </c>
-      <c r="L147" s="28"/>
+        <v>1438</v>
+      </c>
+      <c r="L147" s="28" t="s">
+        <v>723</v>
+      </c>
       <c r="M147" s="28"/>
       <c r="N147" s="28" t="s">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="O147" s="28"/>
       <c r="P147" s="28"/>
@@ -24567,10 +24625,10 @@
         <v>1099</v>
       </c>
       <c r="F151" s="85">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G151" s="85">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H151" s="86">
         <f t="shared" ref="H151:H152" si="30">F151+IF(LEN(G151)=0,0,G151)</f>
@@ -24582,21 +24640,21 @@
       </c>
       <c r="J151" s="84">
         <f t="shared" ref="J151:J152" si="31">F151*I151</f>
-        <v>0</v>
+        <v>1290</v>
       </c>
       <c r="K151" s="84">
         <f t="shared" ref="K151:K152" si="32">IF(LEN(G151)=0,0,G151)*I151</f>
-        <v>2580</v>
+        <v>1290</v>
       </c>
       <c r="L151" s="28" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="M151" s="28"/>
       <c r="N151" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="P151" s="28" t="s">
         <v>624</v>
@@ -24645,14 +24703,14 @@
         <v>885</v>
       </c>
       <c r="L152" s="30" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="M152" s="30"/>
       <c r="N152" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O152" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="P152" s="30" t="s">
         <v>627</v>
@@ -24664,10 +24722,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="28" t="s">
+        <v>647</v>
+      </c>
+      <c r="B153" s="28" t="s">
         <v>648</v>
-      </c>
-      <c r="B153" s="28" t="s">
-        <v>649</v>
       </c>
       <c r="C153" s="28" t="s">
         <v>120</v>
@@ -24707,7 +24765,7 @@
       </c>
       <c r="O153" s="28"/>
       <c r="P153" s="28" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="Q153" s="28"/>
       <c r="R153" s="28"/>
@@ -25318,15 +25376,15 @@
       </c>
       <c r="B8" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>105252</v>
+        <v>110846</v>
       </c>
       <c r="C8" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D8" s="6">
         <f>B8-C8</f>
-        <v>15648.333333333328</v>
+        <v>18445.666666666672</v>
       </c>
       <c r="E8" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE),0)</f>
@@ -25334,7 +25392,7 @@
       </c>
       <c r="F8" s="6">
         <f>D8+E8</f>
-        <v>15648.333333333328</v>
+        <v>18445.666666666672</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -25342,7 +25400,7 @@
       </c>
       <c r="H8" s="8">
         <f>F8-G8</f>
-        <v>2334.3333333333285</v>
+        <v>5131.6666666666715</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -25355,11 +25413,11 @@
       </c>
       <c r="C9" s="7">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D9" s="7">
         <f>B9-C9</f>
-        <v>44578.333333333328</v>
+        <v>41781.666666666672</v>
       </c>
       <c r="E9" s="7">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE),0)</f>
@@ -25367,7 +25425,7 @@
       </c>
       <c r="F9" s="7">
         <f>D9+E9</f>
-        <v>44578.333333333328</v>
+        <v>41781.666666666672</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -25375,7 +25433,7 @@
       </c>
       <c r="H9" s="9">
         <f>F9-G9</f>
-        <v>-1994.326666666675</v>
+        <v>-4790.993333333332</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -25384,15 +25442,15 @@
       </c>
       <c r="B10" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A10,Purchases!$C:$C),0)</f>
-        <v>29377</v>
+        <v>32173</v>
       </c>
       <c r="C10" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>89603.666666666672</v>
+        <v>92400.333333333328</v>
       </c>
       <c r="D10" s="6">
         <f>B10-C10</f>
-        <v>-60226.666666666672</v>
+        <v>-60227.333333333328</v>
       </c>
       <c r="E10" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE),0)</f>
@@ -25400,7 +25458,7 @@
       </c>
       <c r="F10" s="6">
         <f>D10+E10</f>
-        <v>-60226.666666666672</v>
+        <v>-60227.333333333328</v>
       </c>
       <c r="G10" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -25408,7 +25466,7 @@
       </c>
       <c r="H10" s="8">
         <f>F10-G10</f>
-        <v>-340.00666666666802</v>
+        <v>-340.67333333332499</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="22" customFormat="1" ht="16" customHeight="1">
@@ -25761,7 +25819,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>214464</v>
+        <v>215563</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -25769,11 +25827,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>77886.574199999988</v>
+        <v>78252.98079999999</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>136577.42580000003</v>
+        <v>137310.01920000001</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25781,7 +25839,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>12523.949800000031</v>
+        <v>13256.543200000015</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -25798,11 +25856,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>77839.851599999995</v>
+        <v>78206.038400000005</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-71220.851599999995</v>
+        <v>-71587.038400000005</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25810,7 +25868,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-6259.8995999999897</v>
+        <v>-6626.0864000000001</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -25827,11 +25885,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>77886.574199999988</v>
+        <v>78252.98079999999</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-65356.574199999988</v>
+        <v>-65722.98079999999</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -25839,7 +25897,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-6264.0501999999833</v>
+        <v>-6630.4567999999854</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
Chokda update to soldout
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF3647C-CA9A-8843-87D1-5AB0B5FB9B92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AA9778-23E5-484A-B8D7-2686AEC96D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1824,9 +1824,6 @@
     <t>Size: L, XL</t>
   </si>
   <si>
-    <t>⁠​Maheswari cotton Silk saree (Red &amp; Pink)</t>
-  </si>
-  <si>
     <t>Rinsha</t>
   </si>
   <si>
@@ -2026,10 +2023,6 @@
   </si>
   <si>
     <t>Short Kurta - M</t>
-  </si>
-  <si>
-    <t>Rust orange - 1
-Biscuit - 1</t>
   </si>
   <si>
     <t>Jisha (XL), Rameez Relative(L): 900</t>
@@ -2222,12 +2215,6 @@
     <t>Chikkankari(M)</t>
   </si>
   <si>
-    <t xml:space="preserve">Matka Silk Saree (Mustard/gree, Blue/Green, Blue/Red) </t>
-  </si>
-  <si>
-    <t>Blue - Sarany Hyd (Adv-500)</t>
-  </si>
-  <si>
     <t>Praneetha (L), Rameez Cousin (M)</t>
   </si>
   <si>
@@ -2311,6 +2298,18 @@
   </si>
   <si>
     <t>CHR-158</t>
+  </si>
+  <si>
+    <t>Rust orange - 1</t>
+  </si>
+  <si>
+    <t>Matka Silk Saree</t>
+  </si>
+  <si>
+    <t>Blue - Sarany Hyd (Adv-500), Yellow Sudhisha ordered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⁠​Maheswari cotton Silk saree </t>
   </si>
 </sst>
 </file>
@@ -3769,10 +3768,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>188</c:v>
+                  <c:v>189</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>121</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4081,7 +4080,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>109</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>77</c:v>
@@ -4204,7 +4203,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>49</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>67</c:v>
@@ -4637,7 +4636,7 @@
                   <c:v>69555</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>41706.18</c:v>
+                  <c:v>40608.68</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -8364,7 +8363,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46094</v>
+        <v>46095</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8396,7 +8395,7 @@
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>110193.68</v>
+        <v>110912.68</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8440,7 +8439,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8464,7 +8463,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8660,11 +8659,11 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
@@ -8691,7 +8690,7 @@
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$478=J48)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>41706.18</v>
+        <v>40608.68</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9385,7 +9384,7 @@
         <v>1370</v>
       </c>
       <c r="D43" s="37" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -9413,7 +9412,7 @@
         <v>106</v>
       </c>
       <c r="D45" s="37" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -9455,7 +9454,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9470,7 +9469,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -9484,7 +9483,7 @@
         <v>6328</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -9498,7 +9497,7 @@
         <v>3164</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -9526,7 +9525,7 @@
         <v>1400</v>
       </c>
       <c r="D53" s="37" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -9540,7 +9539,7 @@
         <v>700</v>
       </c>
       <c r="D54" s="39" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -9554,7 +9553,7 @@
         <v>5594</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -9568,7 +9567,7 @@
         <v>2796</v>
       </c>
       <c r="D56" s="39" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -14226,7 +14225,7 @@
         <v>46038</v>
       </c>
       <c r="B95" s="47" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C95" s="48">
         <v>1100</v>
@@ -14276,7 +14275,7 @@
         <v>46039</v>
       </c>
       <c r="B97" s="47" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C97" s="48">
         <v>2300</v>
@@ -14290,7 +14289,7 @@
       <c r="F97" s="49"/>
       <c r="G97" s="49"/>
       <c r="H97" s="68" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="I97" s="47" t="s">
         <v>276</v>
@@ -14301,7 +14300,7 @@
         <v>46040</v>
       </c>
       <c r="B98" s="50" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C98" s="51">
         <v>1399</v>
@@ -14315,7 +14314,7 @@
       <c r="F98" s="50"/>
       <c r="G98" s="50"/>
       <c r="H98" s="69" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="I98" s="50" t="s">
         <v>276</v>
@@ -14326,7 +14325,7 @@
         <v>46041</v>
       </c>
       <c r="B99" s="47" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C99" s="48">
         <v>1100</v>
@@ -14351,7 +14350,7 @@
         <v>46042</v>
       </c>
       <c r="B100" s="50" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C100" s="51">
         <v>1250</v>
@@ -14365,7 +14364,7 @@
       <c r="F100" s="50"/>
       <c r="G100" s="50"/>
       <c r="H100" s="69" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="I100" s="50" t="s">
         <v>276</v>
@@ -14376,7 +14375,7 @@
         <v>46043</v>
       </c>
       <c r="B101" s="47" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C101" s="48">
         <v>1380</v>
@@ -14390,7 +14389,7 @@
       <c r="F101" s="49"/>
       <c r="G101" s="49"/>
       <c r="H101" s="68" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="I101" s="47" t="s">
         <v>276</v>
@@ -14401,7 +14400,7 @@
         <v>46046</v>
       </c>
       <c r="B102" s="50" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C102" s="51">
         <v>950</v>
@@ -14415,7 +14414,7 @@
       <c r="F102" s="50"/>
       <c r="G102" s="50"/>
       <c r="H102" s="69" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="I102" s="50" t="s">
         <v>276</v>
@@ -14426,7 +14425,7 @@
         <v>46048</v>
       </c>
       <c r="B103" s="47" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="C103" s="48">
         <v>1380</v>
@@ -14451,7 +14450,7 @@
         <v>46048</v>
       </c>
       <c r="B104" s="50" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C104" s="51">
         <v>2700</v>
@@ -14465,7 +14464,7 @@
       <c r="F104" s="50"/>
       <c r="G104" s="50"/>
       <c r="H104" s="69" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="I104" s="50" t="s">
         <v>276</v>
@@ -14476,7 +14475,7 @@
         <v>46049</v>
       </c>
       <c r="B105" s="47" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="C105" s="48">
         <v>1380</v>
@@ -14501,7 +14500,7 @@
         <v>46049</v>
       </c>
       <c r="B106" s="50" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C106" s="51">
         <v>1380</v>
@@ -14515,7 +14514,7 @@
       <c r="F106" s="50"/>
       <c r="G106" s="50"/>
       <c r="H106" s="69" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="I106" s="50" t="s">
         <v>276</v>
@@ -14526,7 +14525,7 @@
         <v>46049</v>
       </c>
       <c r="B107" s="47" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C107" s="48">
         <v>1200</v>
@@ -14540,7 +14539,7 @@
       <c r="F107" s="49"/>
       <c r="G107" s="49"/>
       <c r="H107" s="68" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="I107" s="47" t="s">
         <v>276</v>
@@ -14551,7 +14550,7 @@
         <v>46050</v>
       </c>
       <c r="B108" s="50" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C108" s="51">
         <v>1250</v>
@@ -14565,7 +14564,7 @@
       <c r="F108" s="50"/>
       <c r="G108" s="50"/>
       <c r="H108" s="69" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="I108" s="50" t="s">
         <v>276</v>
@@ -14576,7 +14575,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14601,7 +14600,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14626,13 +14625,13 @@
         <v>46051</v>
       </c>
       <c r="B111" s="47" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C111" s="48">
         <v>580</v>
       </c>
       <c r="D111" s="47" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E111" s="47" t="s">
         <v>48</v>
@@ -14640,7 +14639,7 @@
       <c r="F111" s="49"/>
       <c r="G111" s="49"/>
       <c r="H111" s="68" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="I111" s="47" t="s">
         <v>276</v>
@@ -14651,7 +14650,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14665,7 +14664,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14676,7 +14675,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14740,7 +14739,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14751,7 +14750,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14765,7 +14764,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14776,7 +14775,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14801,7 +14800,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14826,7 +14825,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14851,13 +14850,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14865,7 +14864,7 @@
       <c r="F120" s="50"/>
       <c r="G120" s="50"/>
       <c r="H120" s="69" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="I120" s="50" t="s">
         <v>276</v>
@@ -14890,7 +14889,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14901,7 +14900,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14915,7 +14914,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14926,7 +14925,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -14951,7 +14950,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -14965,7 +14964,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -14990,7 +14989,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -15001,7 +15000,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -15015,7 +15014,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -15026,7 +15025,7 @@
         <v>46090</v>
       </c>
       <c r="B127" s="47" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C127" s="48">
         <v>850</v>
@@ -15040,7 +15039,7 @@
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
       <c r="H127" s="28" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="I127" s="47" t="s">
         <v>276</v>
@@ -15051,7 +15050,7 @@
         <v>46090</v>
       </c>
       <c r="B128" s="50" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C128" s="51">
         <v>1100</v>
@@ -15065,7 +15064,7 @@
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
       <c r="H128" s="69" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="I128" s="50" t="s">
         <v>276</v>
@@ -15076,7 +15075,7 @@
         <v>46090</v>
       </c>
       <c r="B129" s="47" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C129" s="48">
         <v>1200</v>
@@ -15090,7 +15089,7 @@
       <c r="F129" s="49"/>
       <c r="G129" s="49"/>
       <c r="H129" s="68" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="I129" s="47" t="s">
         <v>191</v>
@@ -15101,7 +15100,7 @@
         <v>46090</v>
       </c>
       <c r="B130" s="50" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C130" s="51">
         <v>2250</v>
@@ -15115,7 +15114,7 @@
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
       <c r="H130" s="69" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="I130" s="50" t="s">
         <v>191</v>
@@ -15126,7 +15125,7 @@
         <v>46091</v>
       </c>
       <c r="B131" s="47" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C131" s="48">
         <v>1099</v>
@@ -15140,7 +15139,7 @@
       <c r="F131" s="49"/>
       <c r="G131" s="49"/>
       <c r="H131" s="68" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="I131" s="47" t="s">
         <v>276</v>
@@ -15151,7 +15150,7 @@
         <v>46092</v>
       </c>
       <c r="B132" s="50" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C132" s="51">
         <v>1200</v>
@@ -15165,7 +15164,7 @@
       <c r="F132" s="50"/>
       <c r="G132" s="50"/>
       <c r="H132" s="69" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="I132" s="50" t="s">
         <v>191</v>
@@ -15176,7 +15175,7 @@
         <v>46092</v>
       </c>
       <c r="B133" s="47" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="C133" s="48">
         <v>1099</v>
@@ -15190,7 +15189,7 @@
       <c r="F133" s="49"/>
       <c r="G133" s="49"/>
       <c r="H133" s="68" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="I133" s="47" t="s">
         <v>276</v>
@@ -15215,7 +15214,7 @@
       <c r="F134" s="50"/>
       <c r="G134" s="50"/>
       <c r="H134" s="69" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="I134" s="50" t="s">
         <v>191</v>
@@ -15240,7 +15239,7 @@
       <c r="F135" s="49"/>
       <c r="G135" s="49"/>
       <c r="H135" s="68" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="I135" s="47" t="s">
         <v>191</v>
@@ -16654,6 +16653,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:T175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7" defaultRowHeight="14"/>
   <cols>
@@ -16668,7 +16668,7 @@
     <col min="9" max="9" width="15.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.83203125" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="43.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="59" style="2" customWidth="1"/>
     <col min="13" max="13" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13" style="2" customWidth="1"/>
     <col min="15" max="15" width="22.33203125" style="2" customWidth="1"/>
@@ -17119,7 +17119,7 @@
       <c r="S8" s="30"/>
       <c r="T8" s="30"/>
     </row>
-    <row r="9" spans="1:20" ht="15" customHeight="1">
+    <row r="9" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A9" s="28" t="s">
         <v>349</v>
       </c>
@@ -17281,7 +17281,7 @@
       <c r="S11" s="28"/>
       <c r="T11" s="28"/>
     </row>
-    <row r="12" spans="1:20" ht="15" customHeight="1">
+    <row r="12" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A12" s="26" t="s">
         <v>352</v>
       </c>
@@ -17335,7 +17335,7 @@
       <c r="S12" s="30"/>
       <c r="T12" s="30"/>
     </row>
-    <row r="13" spans="1:20" ht="15" customHeight="1">
+    <row r="13" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>353</v>
       </c>
@@ -17389,7 +17389,7 @@
       <c r="S13" s="28"/>
       <c r="T13" s="28"/>
     </row>
-    <row r="14" spans="1:20" ht="15" customHeight="1">
+    <row r="14" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A14" s="26" t="s">
         <v>354</v>
       </c>
@@ -17443,7 +17443,7 @@
       <c r="S14" s="30"/>
       <c r="T14" s="30"/>
     </row>
-    <row r="15" spans="1:20" ht="15" customHeight="1">
+    <row r="15" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A15" s="28" t="s">
         <v>355</v>
       </c>
@@ -17497,7 +17497,7 @@
       <c r="S15" s="28"/>
       <c r="T15" s="28"/>
     </row>
-    <row r="16" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="16" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A16" s="26" t="s">
         <v>356</v>
       </c>
@@ -17659,7 +17659,7 @@
       <c r="S18" s="30"/>
       <c r="T18" s="30"/>
     </row>
-    <row r="19" spans="1:20" ht="15" customHeight="1">
+    <row r="19" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A19" s="28" t="s">
         <v>359</v>
       </c>
@@ -17713,7 +17713,7 @@
       <c r="S19" s="28"/>
       <c r="T19" s="28"/>
     </row>
-    <row r="20" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="20" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A20" s="26" t="s">
         <v>360</v>
       </c>
@@ -17767,7 +17767,7 @@
       <c r="S20" s="30"/>
       <c r="T20" s="30"/>
     </row>
-    <row r="21" spans="1:20" ht="15" customHeight="1">
+    <row r="21" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A21" s="28" t="s">
         <v>361</v>
       </c>
@@ -18199,7 +18199,7 @@
       <c r="S28" s="30"/>
       <c r="T28" s="30"/>
     </row>
-    <row r="29" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="29" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A29" s="28" t="s">
         <v>369</v>
       </c>
@@ -18307,7 +18307,7 @@
       <c r="S30" s="30"/>
       <c r="T30" s="30"/>
     </row>
-    <row r="31" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="31" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A31" s="28" t="s">
         <v>371</v>
       </c>
@@ -18361,7 +18361,7 @@
       <c r="S31" s="28"/>
       <c r="T31" s="28"/>
     </row>
-    <row r="32" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="32" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A32" s="26" t="s">
         <v>372</v>
       </c>
@@ -18415,7 +18415,7 @@
       <c r="S32" s="30"/>
       <c r="T32" s="30"/>
     </row>
-    <row r="33" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
+    <row r="33" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A33" s="28" t="s">
         <v>373</v>
       </c>
@@ -18631,7 +18631,7 @@
       <c r="S36" s="30"/>
       <c r="T36" s="30"/>
     </row>
-    <row r="37" spans="1:20" ht="15" customHeight="1">
+    <row r="37" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A37" s="28" t="s">
         <v>377</v>
       </c>
@@ -18739,7 +18739,7 @@
       <c r="S38" s="30"/>
       <c r="T38" s="30"/>
     </row>
-    <row r="39" spans="1:20" ht="15" customHeight="1">
+    <row r="39" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A39" s="28" t="s">
         <v>379</v>
       </c>
@@ -18793,7 +18793,7 @@
       <c r="S39" s="28"/>
       <c r="T39" s="28"/>
     </row>
-    <row r="40" spans="1:20" ht="15" customHeight="1">
+    <row r="40" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A40" s="26" t="s">
         <v>380</v>
       </c>
@@ -18901,7 +18901,7 @@
       <c r="S41" s="28"/>
       <c r="T41" s="28"/>
     </row>
-    <row r="42" spans="1:20" ht="15" customHeight="1">
+    <row r="42" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A42" s="26" t="s">
         <v>382</v>
       </c>
@@ -18955,7 +18955,7 @@
       <c r="S42" s="30"/>
       <c r="T42" s="30"/>
     </row>
-    <row r="43" spans="1:20" ht="15" customHeight="1">
+    <row r="43" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A43" s="28" t="s">
         <v>383</v>
       </c>
@@ -19009,7 +19009,7 @@
       <c r="S43" s="28"/>
       <c r="T43" s="28"/>
     </row>
-    <row r="44" spans="1:20" ht="15" customHeight="1">
+    <row r="44" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A44" s="26" t="s">
         <v>384</v>
       </c>
@@ -19339,7 +19339,7 @@
       <c r="S49" s="28"/>
       <c r="T49" s="28"/>
     </row>
-    <row r="50" spans="1:20" ht="15" customHeight="1">
+    <row r="50" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A50" s="26" t="s">
         <v>390</v>
       </c>
@@ -19393,7 +19393,7 @@
       <c r="S50" s="30"/>
       <c r="T50" s="30"/>
     </row>
-    <row r="51" spans="1:20" ht="15" customHeight="1">
+    <row r="51" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A51" s="28" t="s">
         <v>391</v>
       </c>
@@ -19447,7 +19447,7 @@
       <c r="S51" s="28"/>
       <c r="T51" s="28"/>
     </row>
-    <row r="52" spans="1:20" ht="15" customHeight="1">
+    <row r="52" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A52" s="26" t="s">
         <v>392</v>
       </c>
@@ -19486,7 +19486,7 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
@@ -19503,7 +19503,7 @@
       <c r="S52" s="30"/>
       <c r="T52" s="30"/>
     </row>
-    <row r="53" spans="1:20" ht="15" customHeight="1">
+    <row r="53" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A53" s="28" t="s">
         <v>393</v>
       </c>
@@ -19542,7 +19542,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19552,14 +19552,14 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
       <c r="S53" s="28"/>
       <c r="T53" s="28"/>
     </row>
-    <row r="54" spans="1:20" s="64" customFormat="1" ht="15" customHeight="1">
+    <row r="54" spans="1:20" s="64" customFormat="1" ht="15" hidden="1" customHeight="1">
       <c r="A54" s="26" t="s">
         <v>394</v>
       </c>
@@ -19615,7 +19615,7 @@
       <c r="S54" s="62"/>
       <c r="T54" s="62"/>
     </row>
-    <row r="55" spans="1:20" ht="15" customHeight="1">
+    <row r="55" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A55" s="28" t="s">
         <v>395</v>
       </c>
@@ -19654,7 +19654,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19671,7 +19671,7 @@
       <c r="S55" s="28"/>
       <c r="T55" s="28"/>
     </row>
-    <row r="56" spans="1:20" ht="15" customHeight="1">
+    <row r="56" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A56" s="26" t="s">
         <v>396</v>
       </c>
@@ -19727,7 +19727,7 @@
       <c r="S56" s="30"/>
       <c r="T56" s="30"/>
     </row>
-    <row r="57" spans="1:20" ht="15" customHeight="1">
+    <row r="57" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A57" s="28" t="s">
         <v>397</v>
       </c>
@@ -19779,7 +19779,7 @@
       <c r="S57" s="28"/>
       <c r="T57" s="28"/>
     </row>
-    <row r="58" spans="1:20" ht="15" customHeight="1">
+    <row r="58" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A58" s="26" t="s">
         <v>398</v>
       </c>
@@ -19831,7 +19831,7 @@
       <c r="S58" s="30"/>
       <c r="T58" s="30"/>
     </row>
-    <row r="59" spans="1:20" ht="15" customHeight="1">
+    <row r="59" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A59" s="28" t="s">
         <v>399</v>
       </c>
@@ -19877,7 +19877,7 @@
         <v>180</v>
       </c>
       <c r="O59" s="28" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="P59" s="28" t="s">
         <v>203</v>
@@ -19887,7 +19887,7 @@
       <c r="S59" s="28"/>
       <c r="T59" s="28"/>
     </row>
-    <row r="60" spans="1:20" ht="15">
+    <row r="60" spans="1:20" ht="15" hidden="1">
       <c r="A60" s="26" t="s">
         <v>400</v>
       </c>
@@ -19926,7 +19926,7 @@
         <v>1080</v>
       </c>
       <c r="L60" s="30" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="M60" s="30" t="s">
         <v>46</v>
@@ -19943,7 +19943,7 @@
       <c r="S60" s="30"/>
       <c r="T60" s="30"/>
     </row>
-    <row r="61" spans="1:20" ht="45">
+    <row r="61" spans="1:20" ht="45" hidden="1">
       <c r="A61" s="28" t="s">
         <v>401</v>
       </c>
@@ -19982,17 +19982,17 @@
         <v>4384</v>
       </c>
       <c r="L61" s="28" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
       <c r="M61" s="28"/>
       <c r="N61" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O61" s="28" t="s">
-        <v>725</v>
+        <v>721</v>
       </c>
       <c r="P61" s="28" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="Q61" s="28" t="s">
         <v>478</v>
@@ -20040,7 +20040,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -20246,7 +20246,7 @@
         <v>1558</v>
       </c>
       <c r="L66" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="M66" s="30"/>
       <c r="N66" s="30" t="s">
@@ -20361,7 +20361,7 @@
       <c r="S68" s="30"/>
       <c r="T68" s="30"/>
     </row>
-    <row r="69" spans="1:20" ht="15" customHeight="1">
+    <row r="69" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A69" s="28" t="s">
         <v>409</v>
       </c>
@@ -20418,7 +20418,7 @@
         <v>410</v>
       </c>
       <c r="B70" s="30" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C70" s="30" t="s">
         <v>120</v>
@@ -20452,7 +20452,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -20573,7 +20573,7 @@
       <c r="S72" s="30"/>
       <c r="T72" s="30"/>
     </row>
-    <row r="73" spans="1:20" ht="15" customHeight="1">
+    <row r="73" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A73" s="28" t="s">
         <v>413</v>
       </c>
@@ -20679,7 +20679,7 @@
       <c r="S74" s="30"/>
       <c r="T74" s="30"/>
     </row>
-    <row r="75" spans="1:20" ht="15" customHeight="1">
+    <row r="75" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A75" s="28" t="s">
         <v>415</v>
       </c>
@@ -20787,7 +20787,7 @@
       <c r="S76" s="30"/>
       <c r="T76" s="30"/>
     </row>
-    <row r="77" spans="1:20" ht="15" customHeight="1">
+    <row r="77" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A77" s="28" t="s">
         <v>417</v>
       </c>
@@ -20841,7 +20841,7 @@
       <c r="S77" s="28"/>
       <c r="T77" s="28"/>
     </row>
-    <row r="78" spans="1:20" ht="15" customHeight="1">
+    <row r="78" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A78" s="26" t="s">
         <v>418</v>
       </c>
@@ -20895,7 +20895,7 @@
       <c r="S78" s="30"/>
       <c r="T78" s="30"/>
     </row>
-    <row r="79" spans="1:20" ht="15" customHeight="1">
+    <row r="79" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A79" s="28" t="s">
         <v>419</v>
       </c>
@@ -20947,7 +20947,7 @@
       <c r="S79" s="28"/>
       <c r="T79" s="28"/>
     </row>
-    <row r="80" spans="1:20" ht="15" customHeight="1">
+    <row r="80" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A80" s="26" t="s">
         <v>420</v>
       </c>
@@ -21001,7 +21001,7 @@
       <c r="S80" s="30"/>
       <c r="T80" s="30"/>
     </row>
-    <row r="81" spans="1:20" ht="37" customHeight="1">
+    <row r="81" spans="1:20" ht="37" hidden="1" customHeight="1">
       <c r="A81" s="28" t="s">
         <v>421</v>
       </c>
@@ -21040,7 +21040,7 @@
         <v>0</v>
       </c>
       <c r="L81" s="28" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="M81" s="28"/>
       <c r="N81" s="28" t="s">
@@ -21053,7 +21053,7 @@
       <c r="S81" s="28"/>
       <c r="T81" s="28"/>
     </row>
-    <row r="82" spans="1:20" ht="30">
+    <row r="82" spans="1:20" ht="30" hidden="1">
       <c r="A82" s="26" t="s">
         <v>422</v>
       </c>
@@ -21092,7 +21092,7 @@
         <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
@@ -21105,7 +21105,7 @@
       <c r="S82" s="30"/>
       <c r="T82" s="30"/>
     </row>
-    <row r="83" spans="1:20" ht="45" customHeight="1">
+    <row r="83" spans="1:20" ht="45" hidden="1" customHeight="1">
       <c r="A83" s="28" t="s">
         <v>423</v>
       </c>
@@ -21159,7 +21159,7 @@
       <c r="S83" s="28"/>
       <c r="T83" s="28"/>
     </row>
-    <row r="84" spans="1:20" ht="15" customHeight="1">
+    <row r="84" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A84" s="26" t="s">
         <v>424</v>
       </c>
@@ -21213,7 +21213,7 @@
       <c r="S84" s="30"/>
       <c r="T84" s="30"/>
     </row>
-    <row r="85" spans="1:20" ht="30" customHeight="1">
+    <row r="85" spans="1:20" ht="30" hidden="1" customHeight="1">
       <c r="A85" s="28" t="s">
         <v>425</v>
       </c>
@@ -21252,7 +21252,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21267,7 +21267,7 @@
       <c r="S85" s="28"/>
       <c r="T85" s="28"/>
     </row>
-    <row r="86" spans="1:20" ht="15" customHeight="1">
+    <row r="86" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A86" s="26" t="s">
         <v>426</v>
       </c>
@@ -21306,7 +21306,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21321,7 +21321,7 @@
       <c r="S86" s="30"/>
       <c r="T86" s="30"/>
     </row>
-    <row r="87" spans="1:20" ht="15" customHeight="1">
+    <row r="87" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A87" s="28" t="s">
         <v>427</v>
       </c>
@@ -21373,7 +21373,7 @@
       <c r="S87" s="28"/>
       <c r="T87" s="28"/>
     </row>
-    <row r="88" spans="1:20" ht="30">
+    <row r="88" spans="1:20" ht="30" hidden="1">
       <c r="A88" s="26" t="s">
         <v>428</v>
       </c>
@@ -21479,7 +21479,7 @@
     </row>
     <row r="90" spans="1:20" ht="15" customHeight="1">
       <c r="A90" s="26" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B90" s="30" t="s">
         <v>244</v>
@@ -21516,7 +21516,7 @@
         <v>0</v>
       </c>
       <c r="L90" s="30" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="M90" s="30"/>
       <c r="N90" s="30" t="s">
@@ -21568,7 +21568,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21620,7 +21620,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -21633,7 +21633,7 @@
       <c r="S92" s="30"/>
       <c r="T92" s="30"/>
     </row>
-    <row r="93" spans="1:20" ht="15" customHeight="1">
+    <row r="93" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A93" s="28" t="s">
         <v>432</v>
       </c>
@@ -21893,7 +21893,7 @@
       <c r="S97" s="28"/>
       <c r="T97" s="28"/>
     </row>
-    <row r="98" spans="1:20" ht="15" customHeight="1">
+    <row r="98" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A98" s="26" t="s">
         <v>437</v>
       </c>
@@ -21947,7 +21947,7 @@
       <c r="S98" s="30"/>
       <c r="T98" s="30"/>
     </row>
-    <row r="99" spans="1:20" ht="15" customHeight="1">
+    <row r="99" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A99" s="28" t="s">
         <v>438</v>
       </c>
@@ -22001,7 +22001,7 @@
       <c r="S99" s="28"/>
       <c r="T99" s="28"/>
     </row>
-    <row r="100" spans="1:20" ht="15" customHeight="1">
+    <row r="100" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A100" s="26" t="s">
         <v>439</v>
       </c>
@@ -22055,7 +22055,7 @@
       <c r="S100" s="30"/>
       <c r="T100" s="30"/>
     </row>
-    <row r="101" spans="1:20" ht="15" customHeight="1">
+    <row r="101" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A101" s="28" t="s">
         <v>440</v>
       </c>
@@ -22109,7 +22109,7 @@
       <c r="S101" s="28"/>
       <c r="T101" s="28"/>
     </row>
-    <row r="102" spans="1:20" ht="15" customHeight="1">
+    <row r="102" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A102" s="26" t="s">
         <v>441</v>
       </c>
@@ -22163,7 +22163,7 @@
       <c r="S102" s="30"/>
       <c r="T102" s="30"/>
     </row>
-    <row r="103" spans="1:20" ht="15" customHeight="1">
+    <row r="103" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A103" s="28" t="s">
         <v>442</v>
       </c>
@@ -22217,7 +22217,7 @@
       <c r="S103" s="28"/>
       <c r="T103" s="28"/>
     </row>
-    <row r="104" spans="1:20" ht="15" customHeight="1">
+    <row r="104" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A104" s="26" t="s">
         <v>443</v>
       </c>
@@ -22271,7 +22271,7 @@
       <c r="S104" s="30"/>
       <c r="T104" s="30"/>
     </row>
-    <row r="105" spans="1:20" ht="15" customHeight="1">
+    <row r="105" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A105" s="28" t="s">
         <v>444</v>
       </c>
@@ -22325,7 +22325,7 @@
       <c r="S105" s="28"/>
       <c r="T105" s="28"/>
     </row>
-    <row r="106" spans="1:20" ht="15" customHeight="1">
+    <row r="106" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A106" s="26" t="s">
         <v>445</v>
       </c>
@@ -22364,7 +22364,7 @@
         <v>0</v>
       </c>
       <c r="L106" s="30" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
@@ -22379,7 +22379,7 @@
       <c r="S106" s="30"/>
       <c r="T106" s="30"/>
     </row>
-    <row r="107" spans="1:20" ht="15" customHeight="1">
+    <row r="107" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A107" s="28" t="s">
         <v>446</v>
       </c>
@@ -22433,7 +22433,7 @@
       <c r="S107" s="28"/>
       <c r="T107" s="28"/>
     </row>
-    <row r="108" spans="1:20" ht="15" customHeight="1">
+    <row r="108" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A108" s="26" t="s">
         <v>447</v>
       </c>
@@ -22487,7 +22487,7 @@
       <c r="S108" s="30"/>
       <c r="T108" s="30"/>
     </row>
-    <row r="109" spans="1:20" ht="15" customHeight="1">
+    <row r="109" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A109" s="28" t="s">
         <v>448</v>
       </c>
@@ -22541,7 +22541,7 @@
       <c r="S109" s="28"/>
       <c r="T109" s="28"/>
     </row>
-    <row r="110" spans="1:20" ht="15" customHeight="1">
+    <row r="110" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A110" s="26" t="s">
         <v>449</v>
       </c>
@@ -22595,7 +22595,7 @@
       <c r="S110" s="30"/>
       <c r="T110" s="30"/>
     </row>
-    <row r="111" spans="1:20" ht="15" customHeight="1">
+    <row r="111" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A111" s="28" t="s">
         <v>450</v>
       </c>
@@ -22649,7 +22649,7 @@
       <c r="S111" s="28"/>
       <c r="T111" s="28"/>
     </row>
-    <row r="112" spans="1:20" ht="15" customHeight="1">
+    <row r="112" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A112" s="26" t="s">
         <v>451</v>
       </c>
@@ -22701,7 +22701,7 @@
       <c r="S112" s="30"/>
       <c r="T112" s="30"/>
     </row>
-    <row r="113" spans="1:20" ht="15" customHeight="1">
+    <row r="113" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A113" s="28" t="s">
         <v>452</v>
       </c>
@@ -22846,7 +22846,7 @@
         <v>3764.2799999999997</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22854,14 +22854,14 @@
       </c>
       <c r="O115" s="28"/>
       <c r="P115" s="89" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="Q115" s="28"/>
       <c r="R115" s="28"/>
       <c r="S115" s="28"/>
       <c r="T115" s="28"/>
     </row>
-    <row r="116" spans="1:20" ht="181" customHeight="1">
+    <row r="116" spans="1:20" ht="135">
       <c r="A116" s="26" t="s">
         <v>455</v>
       </c>
@@ -22900,7 +22900,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -22908,7 +22908,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>652</v>
+        <v>739</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -23122,7 +23122,7 @@
       </c>
       <c r="O120" s="30"/>
       <c r="P120" s="30" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="Q120" s="30"/>
       <c r="R120" s="30"/>
@@ -23176,14 +23176,14 @@
       </c>
       <c r="O121" s="28"/>
       <c r="P121" s="28" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="Q121" s="28"/>
       <c r="R121" s="28"/>
       <c r="S121" s="28"/>
       <c r="T121" s="28"/>
     </row>
-    <row r="122" spans="1:20" ht="15">
+    <row r="122" spans="1:20" ht="15" hidden="1">
       <c r="A122" s="26" t="s">
         <v>461</v>
       </c>
@@ -23222,14 +23222,14 @@
         <v>2350</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -23276,7 +23276,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23328,7 +23328,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="84" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M124" s="84"/>
       <c r="N124" s="84" t="s">
@@ -23360,10 +23360,10 @@
         <v>1450</v>
       </c>
       <c r="F125" s="82">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G125" s="82">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H125" s="80">
         <f t="shared" si="9"/>
@@ -23375,14 +23375,14 @@
       </c>
       <c r="J125" s="81">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1816.5</v>
       </c>
       <c r="K125" s="81">
         <f t="shared" si="11"/>
-        <v>1816.5</v>
+        <v>0</v>
       </c>
       <c r="L125" s="81" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="M125" s="81"/>
       <c r="N125" s="81" t="s">
@@ -23397,7 +23397,7 @@
       <c r="S125" s="81"/>
       <c r="T125" s="81"/>
     </row>
-    <row r="126" spans="1:20" ht="15" customHeight="1">
+    <row r="126" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A126" s="83" t="s">
         <v>465</v>
       </c>
@@ -23449,7 +23449,7 @@
       <c r="S126" s="30"/>
       <c r="T126" s="30"/>
     </row>
-    <row r="127" spans="1:20" ht="15" customHeight="1">
+    <row r="127" spans="1:20" ht="15" hidden="1" customHeight="1">
       <c r="A127" s="80" t="s">
         <v>466</v>
       </c>
@@ -23608,7 +23608,7 @@
         <v>469</v>
       </c>
       <c r="B130" s="30" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="C130" s="30" t="s">
         <v>120</v>
@@ -23658,7 +23658,7 @@
         <v>470</v>
       </c>
       <c r="B131" s="28" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C131" s="28" t="s">
         <v>120</v>
@@ -23742,7 +23742,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -23760,7 +23760,7 @@
         <v>472</v>
       </c>
       <c r="B133" s="28" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>120</v>
@@ -23810,7 +23810,7 @@
         <v>473</v>
       </c>
       <c r="B134" s="30" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C134" s="30" t="s">
         <v>120</v>
@@ -23860,7 +23860,7 @@
         <v>474</v>
       </c>
       <c r="B135" s="28" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C135" s="28" t="s">
         <v>120</v>
@@ -23894,7 +23894,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="28" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
@@ -23912,7 +23912,7 @@
         <v>576</v>
       </c>
       <c r="B136" s="30" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C136" s="30" t="s">
         <v>120</v>
@@ -23946,15 +23946,15 @@
         <v>1816</v>
       </c>
       <c r="L136" s="30" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="M136" s="30"/>
       <c r="N136" s="30" t="s">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="O136" s="30"/>
       <c r="P136" s="30" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="Q136" s="30"/>
       <c r="R136" s="30"/>
@@ -24102,7 +24102,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -24120,7 +24120,7 @@
         <v>580</v>
       </c>
       <c r="B140" s="30" t="s">
-        <v>584</v>
+        <v>742</v>
       </c>
       <c r="C140" s="30" t="s">
         <v>120</v>
@@ -24154,7 +24154,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="30" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
@@ -24219,10 +24219,10 @@
     </row>
     <row r="142" spans="1:20" ht="30">
       <c r="A142" s="30" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B142" s="30" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C142" s="30" t="s">
         <v>120</v>
@@ -24256,7 +24256,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -24273,10 +24273,10 @@
     </row>
     <row r="143" spans="1:20" ht="15">
       <c r="A143" s="28" t="s">
+        <v>593</v>
+      </c>
+      <c r="B143" s="28" t="s">
         <v>594</v>
-      </c>
-      <c r="B143" s="28" t="s">
-        <v>595</v>
       </c>
       <c r="C143" s="28" t="s">
         <v>120</v>
@@ -24323,10 +24323,10 @@
     </row>
     <row r="144" spans="1:20" ht="15">
       <c r="A144" s="30" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B144" s="30" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C144" s="30" t="s">
         <v>120</v>
@@ -24373,10 +24373,10 @@
     </row>
     <row r="145" spans="1:20" ht="15">
       <c r="A145" s="28" t="s">
+        <v>596</v>
+      </c>
+      <c r="B145" s="28" t="s">
         <v>597</v>
-      </c>
-      <c r="B145" s="28" t="s">
-        <v>598</v>
       </c>
       <c r="C145" s="28" t="s">
         <v>120</v>
@@ -24410,7 +24410,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24425,10 +24425,10 @@
     </row>
     <row r="146" spans="1:20" ht="30">
       <c r="A146" s="30" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B146" s="30" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C146" s="30" t="s">
         <v>120</v>
@@ -24473,12 +24473,12 @@
       <c r="S146" s="30"/>
       <c r="T146" s="30"/>
     </row>
-    <row r="147" spans="1:20" ht="15">
+    <row r="147" spans="1:20" ht="30">
       <c r="A147" s="28" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>713</v>
+        <v>740</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24490,10 +24490,10 @@
         <v>1200</v>
       </c>
       <c r="F147" s="82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G147" s="82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H147" s="80">
         <f t="shared" si="27"/>
@@ -24505,14 +24505,14 @@
       </c>
       <c r="J147" s="81">
         <f t="shared" si="28"/>
-        <v>719</v>
+        <v>0</v>
       </c>
       <c r="K147" s="81">
         <f t="shared" si="29"/>
-        <v>1438</v>
+        <v>2157</v>
       </c>
       <c r="L147" s="28" t="s">
-        <v>714</v>
+        <v>741</v>
       </c>
       <c r="M147" s="28"/>
       <c r="N147" s="28" t="s">
@@ -24527,10 +24527,10 @@
     </row>
     <row r="148" spans="1:20" ht="15">
       <c r="A148" s="30" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B148" s="30" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="C148" s="30" t="s">
         <v>120</v>
@@ -24579,10 +24579,10 @@
     </row>
     <row r="149" spans="1:20" ht="15">
       <c r="A149" s="28" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B149" s="28" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C149" s="28" t="s">
         <v>120</v>
@@ -24629,10 +24629,10 @@
     </row>
     <row r="150" spans="1:20" ht="15">
       <c r="A150" s="30" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B150" s="30" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C150" s="30" t="s">
         <v>120</v>
@@ -24677,12 +24677,12 @@
       <c r="S150" s="30"/>
       <c r="T150" s="30"/>
     </row>
-    <row r="151" spans="1:20" ht="15">
+    <row r="151" spans="1:20" ht="15" hidden="1">
       <c r="A151" s="28" t="s">
+        <v>615</v>
+      </c>
+      <c r="B151" s="28" t="s">
         <v>616</v>
-      </c>
-      <c r="B151" s="28" t="s">
-        <v>617</v>
       </c>
       <c r="C151" s="28" t="s">
         <v>135</v>
@@ -24716,29 +24716,29 @@
         <v>1290</v>
       </c>
       <c r="L151" s="28" t="s">
-        <v>715</v>
+        <v>711</v>
       </c>
       <c r="M151" s="28"/>
       <c r="N151" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>724</v>
+        <v>720</v>
       </c>
       <c r="P151" s="28" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="Q151" s="28"/>
       <c r="R151" s="28"/>
       <c r="S151" s="28"/>
       <c r="T151" s="28"/>
     </row>
-    <row r="152" spans="1:20" ht="15">
+    <row r="152" spans="1:20" ht="15" hidden="1">
       <c r="A152" s="30" t="s">
+        <v>618</v>
+      </c>
+      <c r="B152" s="30" t="s">
         <v>619</v>
-      </c>
-      <c r="B152" s="30" t="s">
-        <v>620</v>
       </c>
       <c r="C152" s="30" t="s">
         <v>248</v>
@@ -24772,17 +24772,17 @@
         <v>885</v>
       </c>
       <c r="L152" s="30" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="M152" s="30"/>
       <c r="N152" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O152" s="30" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="P152" s="30" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="Q152" s="30"/>
       <c r="R152" s="30"/>
@@ -24791,10 +24791,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="28" t="s">
+        <v>640</v>
+      </c>
+      <c r="B153" s="28" t="s">
         <v>641</v>
-      </c>
-      <c r="B153" s="28" t="s">
-        <v>642</v>
       </c>
       <c r="C153" s="28" t="s">
         <v>120</v>
@@ -24834,19 +24834,19 @@
       </c>
       <c r="O153" s="28"/>
       <c r="P153" s="28" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="Q153" s="28"/>
       <c r="R153" s="28"/>
       <c r="S153" s="28"/>
       <c r="T153" s="28"/>
     </row>
-    <row r="154" spans="1:20" ht="15">
+    <row r="154" spans="1:20" ht="15" hidden="1">
       <c r="A154" s="30" t="s">
-        <v>716</v>
+        <v>712</v>
       </c>
       <c r="B154" s="30" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="C154" s="30" t="s">
         <v>135</v>
@@ -24885,7 +24885,7 @@
         <v>222</v>
       </c>
       <c r="O154" s="30" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="P154" s="30"/>
       <c r="Q154" s="30"/>
@@ -24893,12 +24893,12 @@
       <c r="S154" s="30"/>
       <c r="T154" s="30"/>
     </row>
-    <row r="155" spans="1:20" ht="15">
+    <row r="155" spans="1:20" ht="15" hidden="1">
       <c r="A155" s="28" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="B155" s="28" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="C155" s="28" t="s">
         <v>135</v>
@@ -24937,7 +24937,7 @@
         <v>222</v>
       </c>
       <c r="O155" s="28" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="P155" s="28"/>
       <c r="Q155" s="28"/>
@@ -24945,12 +24945,12 @@
       <c r="S155" s="28"/>
       <c r="T155" s="28"/>
     </row>
-    <row r="156" spans="1:20" ht="15">
+    <row r="156" spans="1:20" ht="15" hidden="1">
       <c r="A156" s="30" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="B156" s="30" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="C156" s="30" t="s">
         <v>135</v>
@@ -24989,7 +24989,7 @@
         <v>222</v>
       </c>
       <c r="O156" s="30" t="s">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="P156" s="30"/>
       <c r="Q156" s="30"/>
@@ -24997,12 +24997,12 @@
       <c r="S156" s="30"/>
       <c r="T156" s="30"/>
     </row>
-    <row r="157" spans="1:20" ht="15">
+    <row r="157" spans="1:20" ht="15" hidden="1">
       <c r="A157" s="28" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="B157" s="28" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="C157" s="28" t="s">
         <v>135</v>
@@ -25036,14 +25036,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="28" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="M157" s="28"/>
       <c r="N157" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O157" s="28" t="s">
-        <v>721</v>
+        <v>717</v>
       </c>
       <c r="P157" s="28"/>
       <c r="Q157" s="28"/>
@@ -25051,12 +25051,12 @@
       <c r="S157" s="28"/>
       <c r="T157" s="28"/>
     </row>
-    <row r="158" spans="1:20" ht="15">
+    <row r="158" spans="1:20" ht="15" hidden="1">
       <c r="A158" s="30" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="B158" s="30" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="C158" s="30" t="s">
         <v>135</v>
@@ -25095,7 +25095,7 @@
         <v>222</v>
       </c>
       <c r="O158" s="30" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="P158" s="30"/>
       <c r="Q158" s="30"/>
@@ -25103,12 +25103,12 @@
       <c r="S158" s="30"/>
       <c r="T158" s="30"/>
     </row>
-    <row r="159" spans="1:20" ht="15">
+    <row r="159" spans="1:20" ht="15" hidden="1">
       <c r="A159" s="28" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="B159" s="28" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="C159" s="28" t="s">
         <v>135</v>
@@ -25147,7 +25147,7 @@
         <v>222</v>
       </c>
       <c r="O159" s="28" t="s">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="P159" s="28"/>
       <c r="Q159" s="28"/>
@@ -25508,6 +25508,13 @@
       <c r="T175" s="30"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:T159" xr:uid="{00000000-0001-0000-0400-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Saree"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N989" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>

<commit_message>
Updated returns & sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AA9778-23E5-484A-B8D7-2686AEC96D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7232C90C-9EC3-7642-858E-61F193828792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="747">
   <si>
     <t>Notes:</t>
   </si>
@@ -2029,9 +2029,6 @@
   </si>
   <si>
     <t>black/purple -1, black/yellow-1, maroon -1</t>
-  </si>
-  <si>
-    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550</t>
   </si>
   <si>
     <t>Rameez Relative</t>
@@ -2146,9 +2143,6 @@
     <t>Tissue silk floral</t>
   </si>
   <si>
-    <t>Rainbow saree &amp; Golden yello with Butterfly on pallu</t>
-  </si>
-  <si>
     <t>Saranya Gopalakrishnan(1300 pending)</t>
   </si>
   <si>
@@ -2191,15 +2185,6 @@
     <t>Sheeja mol maid(1200)</t>
   </si>
   <si>
-    <t>Sushitha (XL-1600), Sheeja Mol (1400)</t>
-  </si>
-  <si>
-    <t>M, L</t>
-  </si>
-  <si>
-    <t>Roman Silk(XXL), Coral Pink (XXL)</t>
-  </si>
-  <si>
     <t>Praneetha (Kochi)</t>
   </si>
   <si>
@@ -2243,15 +2228,6 @@
   </si>
   <si>
     <t>XL, XXL</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Prema(XL)</t>
-  </si>
-  <si>
-    <t>Violet, Mustard, Pink, Grey</t>
   </si>
   <si>
     <t>Prema(XXL)</t>
@@ -2285,9 +2261,6 @@
     <t>Olive green cotton 2-piece kurti set with floral prints</t>
   </si>
   <si>
-    <t>Imported Rayon Violet(XL), Off-white cotton 2-piece set with blue floral prints (XXL)</t>
-  </si>
-  <si>
     <t>Violet, navy blue, rani pink</t>
   </si>
   <si>
@@ -2310,6 +2283,45 @@
   </si>
   <si>
     <t xml:space="preserve">⁠​Maheswari cotton Silk saree </t>
+  </si>
+  <si>
+    <t>Vineet (External)</t>
+  </si>
+  <si>
+    <t>Georgette maroon</t>
+  </si>
+  <si>
+    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550, Vineet(Maroon): 1550</t>
+  </si>
+  <si>
+    <t>Latha(Yellow), Sari(Peach)</t>
+  </si>
+  <si>
+    <t>Rainbow saree &amp; Golden yellow with Butterfly on pallu</t>
+  </si>
+  <si>
+    <t>Sari</t>
+  </si>
+  <si>
+    <t>Soft Cotton Peach with butterfly design</t>
+  </si>
+  <si>
+    <t>Coral Pink Salwar (XXL)</t>
+  </si>
+  <si>
+    <t>Sushitha (XL-1600)</t>
+  </si>
+  <si>
+    <t>Off-white cotton 2-piece set with blue floral prints (XXL)</t>
+  </si>
+  <si>
+    <t>M/XL</t>
+  </si>
+  <si>
+    <t>Deepthi - Mustard for Hokoba return</t>
+  </si>
+  <si>
+    <t>Violet(M&amp;XL), Pink</t>
   </si>
 </sst>
 </file>
@@ -3190,7 +3202,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11498</c:v>
+                  <c:v>11248</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3445,7 +3457,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-9011</c:v>
+                  <c:v>-9261</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3768,10 +3780,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>189</c:v>
+                  <c:v>190</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>120</c:v>
+                  <c:v>119</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4080,10 +4092,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>110</c:v>
+                  <c:v>112</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77</c:v>
+                  <c:v>76</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4203,10 +4215,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>48</c:v>
+                  <c:v>46</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>67</c:v>
+                  <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4633,10 +4645,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>69555</c:v>
+                  <c:v>70730</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>40608.68</c:v>
+                  <c:v>38851.919999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -7958,7 +7970,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>234712</v>
+        <v>237912</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7975,7 +7987,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>242062</v>
+        <v>241812</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -7992,7 +8004,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-42916</v>
+        <v>-39716</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -8195,15 +8207,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>215563</v>
+        <v>218763</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>78252.98079999999</v>
+        <v>79319.860799999995</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>137310.01920000001</v>
+        <v>139443.13920000001</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8211,7 +8223,7 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>-6.8000000028405339E-3</v>
+        <v>2133.1131999999925</v>
       </c>
       <c r="G26" s="71"/>
     </row>
@@ -8226,11 +8238,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>78206.038400000005</v>
+        <v>79272.278399999996</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-71587.038400000005</v>
+        <v>-72653.278399999996</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8238,7 +8250,7 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>3.599999996367842E-3</v>
+        <v>-1066.2363999999943</v>
       </c>
       <c r="G27" s="72"/>
     </row>
@@ -8253,11 +8265,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>78252.98079999999</v>
+        <v>79319.860799999995</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-65722.98079999999</v>
+        <v>-66789.860799999995</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8265,7 +8277,7 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>3.2000000210246071E-3</v>
+        <v>-1066.8767999999836</v>
       </c>
       <c r="G28" s="73"/>
     </row>
@@ -8363,7 +8375,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46095</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8379,7 +8391,7 @@
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>234712</v>
+        <v>237912</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8388,14 +8400,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-42916</v>
+        <v>-39716</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>110912.68</v>
+        <v>110330.92</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8439,7 +8451,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8463,7 +8475,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8476,11 +8488,11 @@
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>11498</v>
+        <v>11248</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-9011</v>
+        <v>-9261</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8659,18 +8671,18 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
       </c>
       <c r="K47" s="77" cm="1">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$478=J47)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>69555</v>
+        <v>70730</v>
       </c>
     </row>
     <row r="48" spans="6:11">
@@ -8679,18 +8691,18 @@
       </c>
       <c r="G48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J48" s="76" t="s">
         <v>120</v>
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$478=J48)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>40608.68</v>
+        <v>38851.919999999998</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9454,7 +9466,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9469,7 +9481,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -9483,7 +9495,7 @@
         <v>6328</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -9497,7 +9509,7 @@
         <v>3164</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -9553,7 +9565,7 @@
         <v>5594</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -9567,7 +9579,7 @@
         <v>2796</v>
       </c>
       <c r="D56" s="39" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -14575,7 +14587,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14600,7 +14612,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14650,7 +14662,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14664,7 +14676,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14675,7 +14687,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14739,7 +14751,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14750,7 +14762,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14764,7 +14776,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14775,7 +14787,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14800,7 +14812,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14825,7 +14837,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14850,13 +14862,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14889,7 +14901,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14900,7 +14912,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14914,7 +14926,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14925,7 +14937,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -14950,7 +14962,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -14964,7 +14976,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -14989,7 +15001,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>688</v>
+        <v>738</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -15000,7 +15012,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -15014,7 +15026,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -15025,7 +15037,7 @@
         <v>46090</v>
       </c>
       <c r="B127" s="47" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C127" s="48">
         <v>850</v>
@@ -15039,7 +15051,7 @@
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
       <c r="H127" s="28" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="I127" s="47" t="s">
         <v>276</v>
@@ -15050,7 +15062,7 @@
         <v>46090</v>
       </c>
       <c r="B128" s="50" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C128" s="51">
         <v>1100</v>
@@ -15064,7 +15076,7 @@
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
       <c r="H128" s="69" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="I128" s="50" t="s">
         <v>276</v>
@@ -15075,7 +15087,7 @@
         <v>46090</v>
       </c>
       <c r="B129" s="47" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C129" s="48">
         <v>1200</v>
@@ -15089,7 +15101,7 @@
       <c r="F129" s="49"/>
       <c r="G129" s="49"/>
       <c r="H129" s="68" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="I129" s="47" t="s">
         <v>191</v>
@@ -15100,10 +15112,10 @@
         <v>46090</v>
       </c>
       <c r="B130" s="50" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C130" s="51">
-        <v>2250</v>
+        <v>800</v>
       </c>
       <c r="D130" s="50" t="s">
         <v>281</v>
@@ -15114,10 +15126,10 @@
       <c r="F130" s="50"/>
       <c r="G130" s="50"/>
       <c r="H130" s="69" t="s">
-        <v>705</v>
+        <v>741</v>
       </c>
       <c r="I130" s="50" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
     </row>
     <row r="131" spans="1:9" ht="16">
@@ -15125,7 +15137,7 @@
         <v>46091</v>
       </c>
       <c r="B131" s="47" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="C131" s="48">
         <v>1099</v>
@@ -15139,7 +15151,7 @@
       <c r="F131" s="49"/>
       <c r="G131" s="49"/>
       <c r="H131" s="68" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="I131" s="47" t="s">
         <v>276</v>
@@ -15150,7 +15162,7 @@
         <v>46092</v>
       </c>
       <c r="B132" s="50" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C132" s="51">
         <v>1200</v>
@@ -15164,7 +15176,7 @@
       <c r="F132" s="50"/>
       <c r="G132" s="50"/>
       <c r="H132" s="69" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="I132" s="50" t="s">
         <v>191</v>
@@ -15175,7 +15187,7 @@
         <v>46092</v>
       </c>
       <c r="B133" s="47" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="C133" s="48">
         <v>1099</v>
@@ -15189,13 +15201,13 @@
       <c r="F133" s="49"/>
       <c r="G133" s="49"/>
       <c r="H133" s="68" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="I133" s="47" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="28">
+    <row r="134" spans="1:9">
       <c r="A134" s="43">
         <v>46093</v>
       </c>
@@ -15203,7 +15215,7 @@
         <v>508</v>
       </c>
       <c r="C134" s="51">
-        <v>2050</v>
+        <v>850</v>
       </c>
       <c r="D134" s="50" t="s">
         <v>281</v>
@@ -15214,7 +15226,7 @@
       <c r="F134" s="50"/>
       <c r="G134" s="50"/>
       <c r="H134" s="69" t="s">
-        <v>734</v>
+        <v>743</v>
       </c>
       <c r="I134" s="50" t="s">
         <v>191</v>
@@ -15239,33 +15251,61 @@
       <c r="F135" s="49"/>
       <c r="G135" s="49"/>
       <c r="H135" s="68" t="s">
-        <v>737</v>
+        <v>728</v>
       </c>
       <c r="I135" s="47" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="136" spans="1:9">
-      <c r="A136" s="43"/>
-      <c r="B136" s="50"/>
-      <c r="C136" s="51"/>
-      <c r="D136" s="50"/>
-      <c r="E136" s="50"/>
+      <c r="A136" s="43">
+        <v>46097</v>
+      </c>
+      <c r="B136" s="50" t="s">
+        <v>734</v>
+      </c>
+      <c r="C136" s="51">
+        <v>1550</v>
+      </c>
+      <c r="D136" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E136" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F136" s="50"/>
       <c r="G136" s="50"/>
-      <c r="H136" s="69"/>
-      <c r="I136" s="50"/>
-    </row>
-    <row r="137" spans="1:9">
-      <c r="A137" s="46"/>
-      <c r="B137" s="47"/>
-      <c r="C137" s="48"/>
-      <c r="D137" s="47"/>
-      <c r="E137" s="47"/>
+      <c r="H136" s="69" t="s">
+        <v>735</v>
+      </c>
+      <c r="I136" s="50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" ht="16">
+      <c r="A137" s="46">
+        <v>46097</v>
+      </c>
+      <c r="B137" s="47" t="s">
+        <v>739</v>
+      </c>
+      <c r="C137" s="48">
+        <v>850</v>
+      </c>
+      <c r="D137" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E137" s="47" t="s">
+        <v>46</v>
+      </c>
       <c r="F137" s="49"/>
       <c r="G137" s="49"/>
-      <c r="H137" s="68"/>
-      <c r="I137" s="47"/>
+      <c r="H137" s="68" t="s">
+        <v>740</v>
+      </c>
+      <c r="I137" s="47" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="138" spans="1:9">
       <c r="A138" s="43"/>
@@ -16653,7 +16693,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:T175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7" defaultRowHeight="14"/>
   <cols>
@@ -17119,7 +17158,7 @@
       <c r="S8" s="30"/>
       <c r="T8" s="30"/>
     </row>
-    <row r="9" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="9" spans="1:20" ht="15" customHeight="1">
       <c r="A9" s="28" t="s">
         <v>349</v>
       </c>
@@ -17281,7 +17320,7 @@
       <c r="S11" s="28"/>
       <c r="T11" s="28"/>
     </row>
-    <row r="12" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="12" spans="1:20" ht="15" customHeight="1">
       <c r="A12" s="26" t="s">
         <v>352</v>
       </c>
@@ -17335,7 +17374,7 @@
       <c r="S12" s="30"/>
       <c r="T12" s="30"/>
     </row>
-    <row r="13" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="13" spans="1:20" ht="15" customHeight="1">
       <c r="A13" s="28" t="s">
         <v>353</v>
       </c>
@@ -17389,7 +17428,7 @@
       <c r="S13" s="28"/>
       <c r="T13" s="28"/>
     </row>
-    <row r="14" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="14" spans="1:20" ht="15" customHeight="1">
       <c r="A14" s="26" t="s">
         <v>354</v>
       </c>
@@ -17443,7 +17482,7 @@
       <c r="S14" s="30"/>
       <c r="T14" s="30"/>
     </row>
-    <row r="15" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="15" spans="1:20" ht="15" customHeight="1">
       <c r="A15" s="28" t="s">
         <v>355</v>
       </c>
@@ -17497,7 +17536,7 @@
       <c r="S15" s="28"/>
       <c r="T15" s="28"/>
     </row>
-    <row r="16" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="16" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A16" s="26" t="s">
         <v>356</v>
       </c>
@@ -17659,7 +17698,7 @@
       <c r="S18" s="30"/>
       <c r="T18" s="30"/>
     </row>
-    <row r="19" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="19" spans="1:20" ht="15" customHeight="1">
       <c r="A19" s="28" t="s">
         <v>359</v>
       </c>
@@ -17713,7 +17752,7 @@
       <c r="S19" s="28"/>
       <c r="T19" s="28"/>
     </row>
-    <row r="20" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="20" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A20" s="26" t="s">
         <v>360</v>
       </c>
@@ -17767,7 +17806,7 @@
       <c r="S20" s="30"/>
       <c r="T20" s="30"/>
     </row>
-    <row r="21" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="21" spans="1:20" ht="15" customHeight="1">
       <c r="A21" s="28" t="s">
         <v>361</v>
       </c>
@@ -18199,7 +18238,7 @@
       <c r="S28" s="30"/>
       <c r="T28" s="30"/>
     </row>
-    <row r="29" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="29" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A29" s="28" t="s">
         <v>369</v>
       </c>
@@ -18307,7 +18346,7 @@
       <c r="S30" s="30"/>
       <c r="T30" s="30"/>
     </row>
-    <row r="31" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="31" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A31" s="28" t="s">
         <v>371</v>
       </c>
@@ -18361,7 +18400,7 @@
       <c r="S31" s="28"/>
       <c r="T31" s="28"/>
     </row>
-    <row r="32" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="32" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A32" s="26" t="s">
         <v>372</v>
       </c>
@@ -18415,7 +18454,7 @@
       <c r="S32" s="30"/>
       <c r="T32" s="30"/>
     </row>
-    <row r="33" spans="1:20" s="3" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="33" spans="1:20" s="3" customFormat="1" ht="15" customHeight="1">
       <c r="A33" s="28" t="s">
         <v>373</v>
       </c>
@@ -18631,7 +18670,7 @@
       <c r="S36" s="30"/>
       <c r="T36" s="30"/>
     </row>
-    <row r="37" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="37" spans="1:20" ht="15" customHeight="1">
       <c r="A37" s="28" t="s">
         <v>377</v>
       </c>
@@ -18739,7 +18778,7 @@
       <c r="S38" s="30"/>
       <c r="T38" s="30"/>
     </row>
-    <row r="39" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="39" spans="1:20" ht="15" customHeight="1">
       <c r="A39" s="28" t="s">
         <v>379</v>
       </c>
@@ -18793,7 +18832,7 @@
       <c r="S39" s="28"/>
       <c r="T39" s="28"/>
     </row>
-    <row r="40" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="40" spans="1:20" ht="15" customHeight="1">
       <c r="A40" s="26" t="s">
         <v>380</v>
       </c>
@@ -18901,7 +18940,7 @@
       <c r="S41" s="28"/>
       <c r="T41" s="28"/>
     </row>
-    <row r="42" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="42" spans="1:20" ht="15" customHeight="1">
       <c r="A42" s="26" t="s">
         <v>382</v>
       </c>
@@ -18955,7 +18994,7 @@
       <c r="S42" s="30"/>
       <c r="T42" s="30"/>
     </row>
-    <row r="43" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="43" spans="1:20" ht="15" customHeight="1">
       <c r="A43" s="28" t="s">
         <v>383</v>
       </c>
@@ -19009,7 +19048,7 @@
       <c r="S43" s="28"/>
       <c r="T43" s="28"/>
     </row>
-    <row r="44" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="44" spans="1:20" ht="15" customHeight="1">
       <c r="A44" s="26" t="s">
         <v>384</v>
       </c>
@@ -19339,7 +19378,7 @@
       <c r="S49" s="28"/>
       <c r="T49" s="28"/>
     </row>
-    <row r="50" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="50" spans="1:20" ht="15" customHeight="1">
       <c r="A50" s="26" t="s">
         <v>390</v>
       </c>
@@ -19393,7 +19432,7 @@
       <c r="S50" s="30"/>
       <c r="T50" s="30"/>
     </row>
-    <row r="51" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="51" spans="1:20" ht="15" customHeight="1">
       <c r="A51" s="28" t="s">
         <v>391</v>
       </c>
@@ -19447,7 +19486,7 @@
       <c r="S51" s="28"/>
       <c r="T51" s="28"/>
     </row>
-    <row r="52" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="52" spans="1:20" ht="15" customHeight="1">
       <c r="A52" s="26" t="s">
         <v>392</v>
       </c>
@@ -19486,7 +19525,7 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
@@ -19503,7 +19542,7 @@
       <c r="S52" s="30"/>
       <c r="T52" s="30"/>
     </row>
-    <row r="53" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="53" spans="1:20" ht="15" customHeight="1">
       <c r="A53" s="28" t="s">
         <v>393</v>
       </c>
@@ -19542,7 +19581,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19552,14 +19591,14 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
       <c r="S53" s="28"/>
       <c r="T53" s="28"/>
     </row>
-    <row r="54" spans="1:20" s="64" customFormat="1" ht="15" hidden="1" customHeight="1">
+    <row r="54" spans="1:20" s="64" customFormat="1" ht="15" customHeight="1">
       <c r="A54" s="26" t="s">
         <v>394</v>
       </c>
@@ -19615,7 +19654,7 @@
       <c r="S54" s="62"/>
       <c r="T54" s="62"/>
     </row>
-    <row r="55" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="55" spans="1:20" ht="15" customHeight="1">
       <c r="A55" s="28" t="s">
         <v>395</v>
       </c>
@@ -19654,7 +19693,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19671,7 +19710,7 @@
       <c r="S55" s="28"/>
       <c r="T55" s="28"/>
     </row>
-    <row r="56" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="56" spans="1:20" ht="15" customHeight="1">
       <c r="A56" s="26" t="s">
         <v>396</v>
       </c>
@@ -19727,7 +19766,7 @@
       <c r="S56" s="30"/>
       <c r="T56" s="30"/>
     </row>
-    <row r="57" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="57" spans="1:20" ht="15" customHeight="1">
       <c r="A57" s="28" t="s">
         <v>397</v>
       </c>
@@ -19779,7 +19818,7 @@
       <c r="S57" s="28"/>
       <c r="T57" s="28"/>
     </row>
-    <row r="58" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="58" spans="1:20" ht="15" customHeight="1">
       <c r="A58" s="26" t="s">
         <v>398</v>
       </c>
@@ -19831,7 +19870,7 @@
       <c r="S58" s="30"/>
       <c r="T58" s="30"/>
     </row>
-    <row r="59" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="59" spans="1:20" ht="15" customHeight="1">
       <c r="A59" s="28" t="s">
         <v>399</v>
       </c>
@@ -19877,7 +19916,7 @@
         <v>180</v>
       </c>
       <c r="O59" s="28" t="s">
-        <v>726</v>
+        <v>718</v>
       </c>
       <c r="P59" s="28" t="s">
         <v>203</v>
@@ -19887,7 +19926,7 @@
       <c r="S59" s="28"/>
       <c r="T59" s="28"/>
     </row>
-    <row r="60" spans="1:20" ht="15" hidden="1">
+    <row r="60" spans="1:20" ht="15">
       <c r="A60" s="26" t="s">
         <v>400</v>
       </c>
@@ -19943,7 +19982,7 @@
       <c r="S60" s="30"/>
       <c r="T60" s="30"/>
     </row>
-    <row r="61" spans="1:20" ht="45" hidden="1">
+    <row r="61" spans="1:20" ht="45">
       <c r="A61" s="28" t="s">
         <v>401</v>
       </c>
@@ -19982,17 +20021,17 @@
         <v>4384</v>
       </c>
       <c r="L61" s="28" t="s">
-        <v>722</v>
+        <v>745</v>
       </c>
       <c r="M61" s="28"/>
       <c r="N61" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O61" s="28" t="s">
-        <v>721</v>
+        <v>744</v>
       </c>
       <c r="P61" s="28" t="s">
-        <v>723</v>
+        <v>746</v>
       </c>
       <c r="Q61" s="28" t="s">
         <v>478</v>
@@ -20040,7 +20079,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -20207,7 +20246,7 @@
       <c r="S65" s="28"/>
       <c r="T65" s="28"/>
     </row>
-    <row r="66" spans="1:20" ht="30">
+    <row r="66" spans="1:20" ht="15">
       <c r="A66" s="26" t="s">
         <v>406</v>
       </c>
@@ -20361,7 +20400,7 @@
       <c r="S68" s="30"/>
       <c r="T68" s="30"/>
     </row>
-    <row r="69" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="69" spans="1:20" ht="15" customHeight="1">
       <c r="A69" s="28" t="s">
         <v>409</v>
       </c>
@@ -20452,7 +20491,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -20573,7 +20612,7 @@
       <c r="S72" s="30"/>
       <c r="T72" s="30"/>
     </row>
-    <row r="73" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="73" spans="1:20" ht="15" customHeight="1">
       <c r="A73" s="28" t="s">
         <v>413</v>
       </c>
@@ -20679,7 +20718,7 @@
       <c r="S74" s="30"/>
       <c r="T74" s="30"/>
     </row>
-    <row r="75" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="75" spans="1:20" ht="15" customHeight="1">
       <c r="A75" s="28" t="s">
         <v>415</v>
       </c>
@@ -20787,7 +20826,7 @@
       <c r="S76" s="30"/>
       <c r="T76" s="30"/>
     </row>
-    <row r="77" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="77" spans="1:20" ht="15" customHeight="1">
       <c r="A77" s="28" t="s">
         <v>417</v>
       </c>
@@ -20841,7 +20880,7 @@
       <c r="S77" s="28"/>
       <c r="T77" s="28"/>
     </row>
-    <row r="78" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="78" spans="1:20" ht="15" customHeight="1">
       <c r="A78" s="26" t="s">
         <v>418</v>
       </c>
@@ -20895,7 +20934,7 @@
       <c r="S78" s="30"/>
       <c r="T78" s="30"/>
     </row>
-    <row r="79" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="79" spans="1:20" ht="15" customHeight="1">
       <c r="A79" s="28" t="s">
         <v>419</v>
       </c>
@@ -20947,7 +20986,7 @@
       <c r="S79" s="28"/>
       <c r="T79" s="28"/>
     </row>
-    <row r="80" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="80" spans="1:20" ht="15" customHeight="1">
       <c r="A80" s="26" t="s">
         <v>420</v>
       </c>
@@ -21001,7 +21040,7 @@
       <c r="S80" s="30"/>
       <c r="T80" s="30"/>
     </row>
-    <row r="81" spans="1:20" ht="37" hidden="1" customHeight="1">
+    <row r="81" spans="1:20" ht="37" customHeight="1">
       <c r="A81" s="28" t="s">
         <v>421</v>
       </c>
@@ -21040,7 +21079,7 @@
         <v>0</v>
       </c>
       <c r="L81" s="28" t="s">
-        <v>727</v>
+        <v>719</v>
       </c>
       <c r="M81" s="28"/>
       <c r="N81" s="28" t="s">
@@ -21053,7 +21092,7 @@
       <c r="S81" s="28"/>
       <c r="T81" s="28"/>
     </row>
-    <row r="82" spans="1:20" ht="30" hidden="1">
+    <row r="82" spans="1:20" ht="15">
       <c r="A82" s="26" t="s">
         <v>422</v>
       </c>
@@ -21092,7 +21131,7 @@
         <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
@@ -21105,7 +21144,7 @@
       <c r="S82" s="30"/>
       <c r="T82" s="30"/>
     </row>
-    <row r="83" spans="1:20" ht="45" hidden="1" customHeight="1">
+    <row r="83" spans="1:20" ht="45" customHeight="1">
       <c r="A83" s="28" t="s">
         <v>423</v>
       </c>
@@ -21159,7 +21198,7 @@
       <c r="S83" s="28"/>
       <c r="T83" s="28"/>
     </row>
-    <row r="84" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="84" spans="1:20" ht="15" customHeight="1">
       <c r="A84" s="26" t="s">
         <v>424</v>
       </c>
@@ -21213,7 +21252,7 @@
       <c r="S84" s="30"/>
       <c r="T84" s="30"/>
     </row>
-    <row r="85" spans="1:20" ht="30" hidden="1" customHeight="1">
+    <row r="85" spans="1:20" ht="30" customHeight="1">
       <c r="A85" s="28" t="s">
         <v>425</v>
       </c>
@@ -21252,7 +21291,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21267,7 +21306,7 @@
       <c r="S85" s="28"/>
       <c r="T85" s="28"/>
     </row>
-    <row r="86" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="86" spans="1:20" ht="15" customHeight="1">
       <c r="A86" s="26" t="s">
         <v>426</v>
       </c>
@@ -21306,7 +21345,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21321,7 +21360,7 @@
       <c r="S86" s="30"/>
       <c r="T86" s="30"/>
     </row>
-    <row r="87" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="87" spans="1:20" ht="15" customHeight="1">
       <c r="A87" s="28" t="s">
         <v>427</v>
       </c>
@@ -21373,7 +21412,7 @@
       <c r="S87" s="28"/>
       <c r="T87" s="28"/>
     </row>
-    <row r="88" spans="1:20" ht="30" hidden="1">
+    <row r="88" spans="1:20" ht="30">
       <c r="A88" s="26" t="s">
         <v>428</v>
       </c>
@@ -21568,7 +21607,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21620,7 +21659,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -21633,7 +21672,7 @@
       <c r="S92" s="30"/>
       <c r="T92" s="30"/>
     </row>
-    <row r="93" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="93" spans="1:20" ht="15" customHeight="1">
       <c r="A93" s="28" t="s">
         <v>432</v>
       </c>
@@ -21893,7 +21932,7 @@
       <c r="S97" s="28"/>
       <c r="T97" s="28"/>
     </row>
-    <row r="98" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="98" spans="1:20" ht="15" customHeight="1">
       <c r="A98" s="26" t="s">
         <v>437</v>
       </c>
@@ -21947,7 +21986,7 @@
       <c r="S98" s="30"/>
       <c r="T98" s="30"/>
     </row>
-    <row r="99" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="99" spans="1:20" ht="15" customHeight="1">
       <c r="A99" s="28" t="s">
         <v>438</v>
       </c>
@@ -22001,7 +22040,7 @@
       <c r="S99" s="28"/>
       <c r="T99" s="28"/>
     </row>
-    <row r="100" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="100" spans="1:20" ht="15" customHeight="1">
       <c r="A100" s="26" t="s">
         <v>439</v>
       </c>
@@ -22055,7 +22094,7 @@
       <c r="S100" s="30"/>
       <c r="T100" s="30"/>
     </row>
-    <row r="101" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="101" spans="1:20" ht="15" customHeight="1">
       <c r="A101" s="28" t="s">
         <v>440</v>
       </c>
@@ -22109,7 +22148,7 @@
       <c r="S101" s="28"/>
       <c r="T101" s="28"/>
     </row>
-    <row r="102" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="102" spans="1:20" ht="15" customHeight="1">
       <c r="A102" s="26" t="s">
         <v>441</v>
       </c>
@@ -22163,7 +22202,7 @@
       <c r="S102" s="30"/>
       <c r="T102" s="30"/>
     </row>
-    <row r="103" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="103" spans="1:20" ht="15" customHeight="1">
       <c r="A103" s="28" t="s">
         <v>442</v>
       </c>
@@ -22217,7 +22256,7 @@
       <c r="S103" s="28"/>
       <c r="T103" s="28"/>
     </row>
-    <row r="104" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="104" spans="1:20" ht="15" customHeight="1">
       <c r="A104" s="26" t="s">
         <v>443</v>
       </c>
@@ -22271,7 +22310,7 @@
       <c r="S104" s="30"/>
       <c r="T104" s="30"/>
     </row>
-    <row r="105" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="105" spans="1:20" ht="15" customHeight="1">
       <c r="A105" s="28" t="s">
         <v>444</v>
       </c>
@@ -22325,7 +22364,7 @@
       <c r="S105" s="28"/>
       <c r="T105" s="28"/>
     </row>
-    <row r="106" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="106" spans="1:20" ht="15" customHeight="1">
       <c r="A106" s="26" t="s">
         <v>445</v>
       </c>
@@ -22364,7 +22403,7 @@
         <v>0</v>
       </c>
       <c r="L106" s="30" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
@@ -22379,7 +22418,7 @@
       <c r="S106" s="30"/>
       <c r="T106" s="30"/>
     </row>
-    <row r="107" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="107" spans="1:20" ht="15" customHeight="1">
       <c r="A107" s="28" t="s">
         <v>446</v>
       </c>
@@ -22433,7 +22472,7 @@
       <c r="S107" s="28"/>
       <c r="T107" s="28"/>
     </row>
-    <row r="108" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="108" spans="1:20" ht="15" customHeight="1">
       <c r="A108" s="26" t="s">
         <v>447</v>
       </c>
@@ -22487,7 +22526,7 @@
       <c r="S108" s="30"/>
       <c r="T108" s="30"/>
     </row>
-    <row r="109" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="109" spans="1:20" ht="15" customHeight="1">
       <c r="A109" s="28" t="s">
         <v>448</v>
       </c>
@@ -22541,7 +22580,7 @@
       <c r="S109" s="28"/>
       <c r="T109" s="28"/>
     </row>
-    <row r="110" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="110" spans="1:20" ht="15" customHeight="1">
       <c r="A110" s="26" t="s">
         <v>449</v>
       </c>
@@ -22595,7 +22634,7 @@
       <c r="S110" s="30"/>
       <c r="T110" s="30"/>
     </row>
-    <row r="111" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="111" spans="1:20" ht="15" customHeight="1">
       <c r="A111" s="28" t="s">
         <v>450</v>
       </c>
@@ -22649,7 +22688,7 @@
       <c r="S111" s="28"/>
       <c r="T111" s="28"/>
     </row>
-    <row r="112" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="112" spans="1:20" ht="15" customHeight="1">
       <c r="A112" s="26" t="s">
         <v>451</v>
       </c>
@@ -22701,7 +22740,7 @@
       <c r="S112" s="30"/>
       <c r="T112" s="30"/>
     </row>
-    <row r="113" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="113" spans="1:20" ht="15" customHeight="1">
       <c r="A113" s="28" t="s">
         <v>452</v>
       </c>
@@ -22824,10 +22863,10 @@
         <v>1599</v>
       </c>
       <c r="F115" s="29">
+        <v>3</v>
+      </c>
+      <c r="G115" s="29">
         <v>2</v>
-      </c>
-      <c r="G115" s="29">
-        <v>3</v>
       </c>
       <c r="H115" s="28">
         <f t="shared" si="9"/>
@@ -22839,14 +22878,14 @@
       </c>
       <c r="J115" s="28">
         <f t="shared" si="10"/>
-        <v>2509.52</v>
+        <v>3764.2799999999997</v>
       </c>
       <c r="K115" s="28">
         <f t="shared" si="11"/>
-        <v>3764.2799999999997</v>
+        <v>2509.52</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>653</v>
+        <v>736</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22900,7 +22939,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -22908,7 +22947,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>739</v>
+        <v>730</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -23122,7 +23161,7 @@
       </c>
       <c r="O120" s="30"/>
       <c r="P120" s="30" t="s">
-        <v>735</v>
+        <v>726</v>
       </c>
       <c r="Q120" s="30"/>
       <c r="R120" s="30"/>
@@ -23176,14 +23215,14 @@
       </c>
       <c r="O121" s="28"/>
       <c r="P121" s="28" t="s">
-        <v>736</v>
+        <v>727</v>
       </c>
       <c r="Q121" s="28"/>
       <c r="R121" s="28"/>
       <c r="S121" s="28"/>
       <c r="T121" s="28"/>
     </row>
-    <row r="122" spans="1:20" ht="15" hidden="1">
+    <row r="122" spans="1:20" ht="15">
       <c r="A122" s="26" t="s">
         <v>461</v>
       </c>
@@ -23200,10 +23239,10 @@
         <v>1600</v>
       </c>
       <c r="F122" s="31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G122" s="31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H122" s="30">
         <f t="shared" si="9"/>
@@ -23215,21 +23254,21 @@
       </c>
       <c r="J122" s="30">
         <f t="shared" si="10"/>
-        <v>2350</v>
+        <v>1175</v>
       </c>
       <c r="K122" s="30">
         <f t="shared" si="11"/>
-        <v>2350</v>
+        <v>3525</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>703</v>
+        <v>742</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>704</v>
+        <v>531</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -23276,7 +23315,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23289,7 +23328,7 @@
       <c r="S123" s="81"/>
       <c r="T123" s="81"/>
     </row>
-    <row r="124" spans="1:20" s="87" customFormat="1" ht="45">
+    <row r="124" spans="1:20" s="87" customFormat="1" ht="30">
       <c r="A124" s="83" t="s">
         <v>463</v>
       </c>
@@ -23397,7 +23436,7 @@
       <c r="S125" s="81"/>
       <c r="T125" s="81"/>
     </row>
-    <row r="126" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="126" spans="1:20" ht="15" customHeight="1">
       <c r="A126" s="83" t="s">
         <v>465</v>
       </c>
@@ -23449,7 +23488,7 @@
       <c r="S126" s="30"/>
       <c r="T126" s="30"/>
     </row>
-    <row r="127" spans="1:20" ht="15" hidden="1" customHeight="1">
+    <row r="127" spans="1:20" ht="15" customHeight="1">
       <c r="A127" s="80" t="s">
         <v>466</v>
       </c>
@@ -23742,7 +23781,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -23894,7 +23933,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="28" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
@@ -24102,7 +24141,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -24120,7 +24159,7 @@
         <v>580</v>
       </c>
       <c r="B140" s="30" t="s">
-        <v>742</v>
+        <v>733</v>
       </c>
       <c r="C140" s="30" t="s">
         <v>120</v>
@@ -24154,7 +24193,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="30" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
@@ -24217,7 +24256,7 @@
       <c r="S141" s="28"/>
       <c r="T141" s="28"/>
     </row>
-    <row r="142" spans="1:20" ht="30">
+    <row r="142" spans="1:20" ht="15">
       <c r="A142" s="30" t="s">
         <v>592</v>
       </c>
@@ -24256,7 +24295,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -24410,7 +24449,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24473,12 +24512,12 @@
       <c r="S146" s="30"/>
       <c r="T146" s="30"/>
     </row>
-    <row r="147" spans="1:20" ht="30">
+    <row r="147" spans="1:20" ht="15">
       <c r="A147" s="28" t="s">
         <v>611</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>740</v>
+        <v>731</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24512,7 +24551,7 @@
         <v>2157</v>
       </c>
       <c r="L147" s="28" t="s">
-        <v>741</v>
+        <v>732</v>
       </c>
       <c r="M147" s="28"/>
       <c r="N147" s="28" t="s">
@@ -24542,10 +24581,10 @@
         <v>850</v>
       </c>
       <c r="F148" s="85">
+        <v>2</v>
+      </c>
+      <c r="G148" s="85">
         <v>1</v>
-      </c>
-      <c r="G148" s="85">
-        <v>2</v>
       </c>
       <c r="H148" s="86">
         <f t="shared" si="27"/>
@@ -24557,14 +24596,14 @@
       </c>
       <c r="J148" s="84">
         <f t="shared" si="28"/>
-        <v>502</v>
+        <v>1004</v>
       </c>
       <c r="K148" s="84">
         <f t="shared" si="29"/>
-        <v>1004</v>
+        <v>502</v>
       </c>
       <c r="L148" s="30" t="s">
-        <v>128</v>
+        <v>737</v>
       </c>
       <c r="M148" s="30"/>
       <c r="N148" s="30" t="s">
@@ -24677,7 +24716,7 @@
       <c r="S150" s="30"/>
       <c r="T150" s="30"/>
     </row>
-    <row r="151" spans="1:20" ht="15" hidden="1">
+    <row r="151" spans="1:20" ht="15">
       <c r="A151" s="28" t="s">
         <v>615</v>
       </c>
@@ -24716,14 +24755,14 @@
         <v>1290</v>
       </c>
       <c r="L151" s="28" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="M151" s="28"/>
       <c r="N151" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="P151" s="28" t="s">
         <v>617</v>
@@ -24733,7 +24772,7 @@
       <c r="S151" s="28"/>
       <c r="T151" s="28"/>
     </row>
-    <row r="152" spans="1:20" ht="15" hidden="1">
+    <row r="152" spans="1:20" ht="15">
       <c r="A152" s="30" t="s">
         <v>618</v>
       </c>
@@ -24841,12 +24880,12 @@
       <c r="S153" s="28"/>
       <c r="T153" s="28"/>
     </row>
-    <row r="154" spans="1:20" ht="15" hidden="1">
+    <row r="154" spans="1:20" ht="15">
       <c r="A154" s="30" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="B154" s="30" t="s">
-        <v>728</v>
+        <v>720</v>
       </c>
       <c r="C154" s="30" t="s">
         <v>135</v>
@@ -24885,7 +24924,7 @@
         <v>222</v>
       </c>
       <c r="O154" s="30" t="s">
-        <v>725</v>
+        <v>717</v>
       </c>
       <c r="P154" s="30"/>
       <c r="Q154" s="30"/>
@@ -24893,12 +24932,12 @@
       <c r="S154" s="30"/>
       <c r="T154" s="30"/>
     </row>
-    <row r="155" spans="1:20" ht="15" hidden="1">
+    <row r="155" spans="1:20" ht="15">
       <c r="A155" s="28" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
       <c r="B155" s="28" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="C155" s="28" t="s">
         <v>135</v>
@@ -24937,7 +24976,7 @@
         <v>222</v>
       </c>
       <c r="O155" s="28" t="s">
-        <v>725</v>
+        <v>717</v>
       </c>
       <c r="P155" s="28"/>
       <c r="Q155" s="28"/>
@@ -24945,12 +24984,12 @@
       <c r="S155" s="28"/>
       <c r="T155" s="28"/>
     </row>
-    <row r="156" spans="1:20" ht="15" hidden="1">
+    <row r="156" spans="1:20" ht="15">
       <c r="A156" s="30" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="B156" s="30" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="C156" s="30" t="s">
         <v>135</v>
@@ -24989,7 +25028,7 @@
         <v>222</v>
       </c>
       <c r="O156" s="30" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="P156" s="30"/>
       <c r="Q156" s="30"/>
@@ -24997,12 +25036,12 @@
       <c r="S156" s="30"/>
       <c r="T156" s="30"/>
     </row>
-    <row r="157" spans="1:20" ht="15" hidden="1">
+    <row r="157" spans="1:20" ht="15">
       <c r="A157" s="28" t="s">
-        <v>715</v>
+        <v>710</v>
       </c>
       <c r="B157" s="28" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="C157" s="28" t="s">
         <v>135</v>
@@ -25036,14 +25075,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="28" t="s">
-        <v>724</v>
+        <v>716</v>
       </c>
       <c r="M157" s="28"/>
       <c r="N157" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O157" s="28" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="P157" s="28"/>
       <c r="Q157" s="28"/>
@@ -25051,12 +25090,12 @@
       <c r="S157" s="28"/>
       <c r="T157" s="28"/>
     </row>
-    <row r="158" spans="1:20" ht="15" hidden="1">
+    <row r="158" spans="1:20" ht="15">
       <c r="A158" s="30" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="B158" s="30" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
       <c r="C158" s="30" t="s">
         <v>135</v>
@@ -25095,7 +25134,7 @@
         <v>222</v>
       </c>
       <c r="O158" s="30" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="P158" s="30"/>
       <c r="Q158" s="30"/>
@@ -25103,12 +25142,12 @@
       <c r="S158" s="30"/>
       <c r="T158" s="30"/>
     </row>
-    <row r="159" spans="1:20" ht="15" hidden="1">
+    <row r="159" spans="1:20" ht="15">
       <c r="A159" s="28" t="s">
-        <v>738</v>
+        <v>729</v>
       </c>
       <c r="B159" s="28" t="s">
-        <v>733</v>
+        <v>725</v>
       </c>
       <c r="C159" s="28" t="s">
         <v>135</v>
@@ -25147,7 +25186,7 @@
         <v>222</v>
       </c>
       <c r="O159" s="28" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="P159" s="28"/>
       <c r="Q159" s="28"/>
@@ -25508,13 +25547,6 @@
       <c r="T175" s="30"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T159" xr:uid="{00000000-0001-0000-0400-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Saree"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N989" xr:uid="{00000000-0002-0000-0400-000000000000}">
@@ -26119,7 +26151,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>215563</v>
+        <v>218763</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -26127,11 +26159,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>78252.98079999999</v>
+        <v>79319.860799999995</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>137310.01920000001</v>
+        <v>139443.13920000001</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26139,7 +26171,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>-6.8000000028405339E-3</v>
+        <v>2133.1131999999925</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -26156,11 +26188,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>78206.038400000005</v>
+        <v>79272.278399999996</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-71587.038400000005</v>
+        <v>-72653.278399999996</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26168,7 +26200,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>3.599999996367842E-3</v>
+        <v>-1066.2363999999943</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -26185,11 +26217,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>78252.98079999999</v>
+        <v>79319.860799999995</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-65722.98079999999</v>
+        <v>-66789.860799999995</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26197,7 +26229,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>3.2000000210246071E-3</v>
+        <v>-1066.8767999999836</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
New meesho purchases & Khadee sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7232C90C-9EC3-7642-858E-61F193828792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4523930-D614-BB4C-BA3B-78B1E56F58DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1889" uniqueCount="757">
   <si>
     <t>Notes:</t>
   </si>
@@ -2309,9 +2309,6 @@
     <t>Coral Pink Salwar (XXL)</t>
   </si>
   <si>
-    <t>Sushitha (XL-1600)</t>
-  </si>
-  <si>
     <t>Off-white cotton 2-piece set with blue floral prints (XXL)</t>
   </si>
   <si>
@@ -2322,6 +2319,39 @@
   </si>
   <si>
     <t>Violet(M&amp;XL), Pink</t>
+  </si>
+  <si>
+    <t>Khadee and Cotton Silk Sarees</t>
+  </si>
+  <si>
+    <t>CHR-159</t>
+  </si>
+  <si>
+    <t>CHR-160</t>
+  </si>
+  <si>
+    <t>CHR-161</t>
+  </si>
+  <si>
+    <t>CHR-162</t>
+  </si>
+  <si>
+    <t>Black &amp; Beige Leaf Print Cotton Silk Saree</t>
+  </si>
+  <si>
+    <t>Teal &amp; Coral Abstract Print Cotton Silk Saree</t>
+  </si>
+  <si>
+    <t>Khadee Saree - Navy Blue and Olive Green</t>
+  </si>
+  <si>
+    <t>Khadee Saree - Brown &amp; Black</t>
+  </si>
+  <si>
+    <t>Neethu</t>
+  </si>
+  <si>
+    <t>Sushitha (XXL-1600)</t>
   </si>
 </sst>
 </file>
@@ -3084,7 +3114,7 @@
                   <c:v>4790</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20509</c:v>
+                  <c:v>22172</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3202,7 +3232,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11248</c:v>
+                  <c:v>12448</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3457,7 +3487,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-9261</c:v>
+                  <c:v>-9724</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3780,10 +3810,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>190</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>119</c:v>
+                  <c:v>121</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4092,7 +4122,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>112</c:v>
+                  <c:v>114</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>76</c:v>
@@ -4215,7 +4245,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>46</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>68</c:v>
@@ -4648,7 +4678,7 @@
                   <c:v>70730</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>38851.919999999998</c:v>
+                  <c:v>39825.919999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -7955,7 +7985,7 @@
       </c>
       <c r="B3" s="1">
         <f>SUM(Purchases!C:C)</f>
-        <v>277628</v>
+        <v>279291</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>39</v>
@@ -7970,7 +8000,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>237912</v>
+        <v>239112</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -7987,7 +8017,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>241812</v>
+        <v>243012</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -8004,7 +8034,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-39716</v>
+        <v>-40179</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -8039,7 +8069,7 @@
       </c>
       <c r="B10" s="52">
         <f>PartnerShares!H8</f>
-        <v>-6.6666666716628242E-3</v>
+        <v>1108.6599999999999</v>
       </c>
       <c r="C10" s="6"/>
     </row>
@@ -8049,7 +8079,7 @@
       </c>
       <c r="B11" s="53">
         <f>PartnerShares!H9</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
       <c r="C11" s="7"/>
     </row>
@@ -8059,7 +8089,7 @@
       </c>
       <c r="B12" s="52">
         <f>PartnerShares!H10</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
       <c r="C12" s="6"/>
     </row>
@@ -8098,15 +8128,15 @@
       </c>
       <c r="B18" s="6">
         <f>PartnerShares!B8</f>
-        <v>110846</v>
+        <v>112509</v>
       </c>
       <c r="C18" s="6">
         <f>PartnerShares!C8</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D18" s="6">
         <f>PartnerShares!D8</f>
-        <v>18303.333333333328</v>
+        <v>19412</v>
       </c>
       <c r="E18" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8114,7 +8144,7 @@
       </c>
       <c r="F18" s="8">
         <f>D18-E18</f>
-        <v>-6.6666666716628242E-3</v>
+        <v>1108.6599999999999</v>
       </c>
       <c r="G18" s="73"/>
     </row>
@@ -8129,11 +8159,11 @@
       </c>
       <c r="C19" s="7">
         <f>PartnerShares!C9</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D19" s="7">
         <f>PartnerShares!D9</f>
-        <v>41639.333333333328</v>
+        <v>41085</v>
       </c>
       <c r="E19" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8141,7 +8171,7 @@
       </c>
       <c r="F19" s="9">
         <f>D19-E19</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
       <c r="G19" s="71"/>
     </row>
@@ -8156,11 +8186,11 @@
       </c>
       <c r="C20" s="6">
         <f>PartnerShares!C10</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D20" s="6">
         <f>PartnerShares!D10</f>
-        <v>-59942.666666666672</v>
+        <v>-60497</v>
       </c>
       <c r="E20" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8168,7 +8198,7 @@
       </c>
       <c r="F20" s="8">
         <f>D20-E20</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
       <c r="G20" s="71"/>
     </row>
@@ -8207,15 +8237,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>218763</v>
+        <v>219963</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>79319.860799999995</v>
+        <v>79719.940799999997</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>139443.13920000001</v>
+        <v>140243.05920000002</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8223,7 +8253,7 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>2133.1131999999925</v>
+        <v>2933.0332000000053</v>
       </c>
       <c r="G26" s="71"/>
     </row>
@@ -8238,11 +8268,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>79272.278399999996</v>
+        <v>79672.118399999992</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-72653.278399999996</v>
+        <v>-73053.118399999992</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8250,7 +8280,7 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-1066.2363999999943</v>
+        <v>-1466.0763999999908</v>
       </c>
       <c r="G27" s="72"/>
     </row>
@@ -8265,11 +8295,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>79319.860799999995</v>
+        <v>79719.940799999997</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-66789.860799999995</v>
+        <v>-67189.940799999997</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8277,7 +8307,7 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-1066.8767999999836</v>
+        <v>-1466.9567999999854</v>
       </c>
       <c r="G28" s="73"/>
     </row>
@@ -8375,7 +8405,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46098</v>
+        <v>46100</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8384,14 +8414,14 @@
       </c>
       <c r="B5" s="15">
         <f>Summary!B3</f>
-        <v>277628</v>
+        <v>279291</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>237912</v>
+        <v>239112</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8400,14 +8430,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-39716</v>
+        <v>-40179</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>110330.92</v>
+        <v>111304.92</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8451,7 +8481,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8475,7 +8505,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8484,15 +8514,15 @@
       </c>
       <c r="B12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A12)*Purchases!$C$2:$C$998),0)</f>
-        <v>20509</v>
+        <v>22172</v>
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>11248</v>
+        <v>12448</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-9261</v>
+        <v>-9724</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8671,11 +8701,11 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
@@ -8702,7 +8732,7 @@
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$478=J48)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>38851.919999999998</v>
+        <v>39825.919999999998</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9597,10 +9627,18 @@
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="41"/>
-      <c r="B58" s="39"/>
-      <c r="C58" s="40"/>
-      <c r="D58" s="39"/>
+      <c r="A58" s="41">
+        <v>46100</v>
+      </c>
+      <c r="B58" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="C58" s="40">
+        <v>1663</v>
+      </c>
+      <c r="D58" s="39" t="s">
+        <v>746</v>
+      </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="36"/>
@@ -15226,7 +15264,7 @@
       <c r="F134" s="50"/>
       <c r="G134" s="50"/>
       <c r="H134" s="69" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="I134" s="50" t="s">
         <v>191</v>
@@ -15308,15 +15346,29 @@
       </c>
     </row>
     <row r="138" spans="1:9">
-      <c r="A138" s="43"/>
-      <c r="B138" s="50"/>
-      <c r="C138" s="51"/>
-      <c r="D138" s="50"/>
-      <c r="E138" s="50"/>
+      <c r="A138" s="43">
+        <v>46100</v>
+      </c>
+      <c r="B138" s="50" t="s">
+        <v>755</v>
+      </c>
+      <c r="C138" s="51">
+        <v>1200</v>
+      </c>
+      <c r="D138" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E138" s="50" t="s">
+        <v>46</v>
+      </c>
       <c r="F138" s="50"/>
       <c r="G138" s="50"/>
-      <c r="H138" s="69"/>
-      <c r="I138" s="50"/>
+      <c r="H138" s="69" t="s">
+        <v>99</v>
+      </c>
+      <c r="I138" s="50" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="139" spans="1:9">
       <c r="A139" s="46"/>
@@ -20021,17 +20073,17 @@
         <v>4384</v>
       </c>
       <c r="L61" s="28" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="M61" s="28"/>
       <c r="N61" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O61" s="28" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="P61" s="28" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="Q61" s="28" t="s">
         <v>478</v>
@@ -23261,14 +23313,14 @@
         <v>3525</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>742</v>
+        <v>756</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>531</v>
+        <v>712</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -25194,21 +25246,51 @@
       <c r="S159" s="28"/>
       <c r="T159" s="28"/>
     </row>
-    <row r="160" spans="1:20">
-      <c r="A160" s="30"/>
-      <c r="B160" s="30"/>
-      <c r="C160" s="30"/>
-      <c r="D160" s="31"/>
-      <c r="E160" s="31"/>
-      <c r="F160" s="31"/>
-      <c r="G160" s="31"/>
-      <c r="H160" s="30"/>
-      <c r="I160" s="30"/>
-      <c r="J160" s="30"/>
-      <c r="K160" s="30"/>
-      <c r="L160" s="30"/>
+    <row r="160" spans="1:20" ht="15">
+      <c r="A160" s="30" t="s">
+        <v>747</v>
+      </c>
+      <c r="B160" s="30" t="s">
+        <v>753</v>
+      </c>
+      <c r="C160" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="D160" s="31">
+        <v>336</v>
+      </c>
+      <c r="E160" s="31">
+        <v>600</v>
+      </c>
+      <c r="F160" s="85">
+        <v>1</v>
+      </c>
+      <c r="G160" s="85">
+        <v>0</v>
+      </c>
+      <c r="H160" s="86">
+        <f t="shared" ref="H160:H161" si="39">F160+IF(LEN(G160)=0,0,G160)</f>
+        <v>1</v>
+      </c>
+      <c r="I160" s="84">
+        <f>IF(D160&lt;&gt;"",D160,IFERROR(E160/(IFERROR(SUM([1]Sales!C:C),0))*(IFERROR(SUM([1]Purchases!C:C),0)),0))</f>
+        <v>336</v>
+      </c>
+      <c r="J160" s="84">
+        <f t="shared" ref="J160:J161" si="40">F160*I160</f>
+        <v>336</v>
+      </c>
+      <c r="K160" s="84">
+        <f t="shared" ref="K160:K161" si="41">IF(LEN(G160)=0,0,G160)*I160</f>
+        <v>0</v>
+      </c>
+      <c r="L160" s="30" t="s">
+        <v>755</v>
+      </c>
       <c r="M160" s="30"/>
-      <c r="N160" s="30"/>
+      <c r="N160" s="30" t="s">
+        <v>122</v>
+      </c>
       <c r="O160" s="30"/>
       <c r="P160" s="30"/>
       <c r="Q160" s="30"/>
@@ -25216,21 +25298,51 @@
       <c r="S160" s="30"/>
       <c r="T160" s="30"/>
     </row>
-    <row r="161" spans="1:20">
-      <c r="A161" s="28"/>
-      <c r="B161" s="28"/>
-      <c r="C161" s="28"/>
-      <c r="D161" s="29"/>
-      <c r="E161" s="29"/>
-      <c r="F161" s="29"/>
-      <c r="G161" s="29"/>
-      <c r="H161" s="28"/>
-      <c r="I161" s="28"/>
-      <c r="J161" s="28"/>
-      <c r="K161" s="28"/>
-      <c r="L161" s="28"/>
+    <row r="161" spans="1:20" ht="15">
+      <c r="A161" s="28" t="s">
+        <v>748</v>
+      </c>
+      <c r="B161" s="28" t="s">
+        <v>754</v>
+      </c>
+      <c r="C161" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="D161" s="29">
+        <v>353</v>
+      </c>
+      <c r="E161" s="29">
+        <v>600</v>
+      </c>
+      <c r="F161" s="90">
+        <v>1</v>
+      </c>
+      <c r="G161" s="90">
+        <v>0</v>
+      </c>
+      <c r="H161" s="81">
+        <f t="shared" si="39"/>
+        <v>1</v>
+      </c>
+      <c r="I161" s="80">
+        <f>IF(D161&lt;&gt;"",D161,IFERROR(E161/(IFERROR(SUM([1]Sales!C:C),0))*(IFERROR(SUM([1]Purchases!C:C),0)),0))</f>
+        <v>353</v>
+      </c>
+      <c r="J161" s="80">
+        <f t="shared" si="40"/>
+        <v>353</v>
+      </c>
+      <c r="K161" s="80">
+        <f t="shared" si="41"/>
+        <v>0</v>
+      </c>
+      <c r="L161" s="28" t="s">
+        <v>755</v>
+      </c>
       <c r="M161" s="28"/>
-      <c r="N161" s="28"/>
+      <c r="N161" s="28" t="s">
+        <v>122</v>
+      </c>
       <c r="O161" s="28"/>
       <c r="P161" s="28"/>
       <c r="Q161" s="28"/>
@@ -25238,21 +25350,49 @@
       <c r="S161" s="28"/>
       <c r="T161" s="28"/>
     </row>
-    <row r="162" spans="1:20">
-      <c r="A162" s="30"/>
-      <c r="B162" s="30"/>
-      <c r="C162" s="30"/>
-      <c r="D162" s="31"/>
-      <c r="E162" s="31"/>
-      <c r="F162" s="31"/>
-      <c r="G162" s="31"/>
-      <c r="H162" s="30"/>
-      <c r="I162" s="30"/>
-      <c r="J162" s="30"/>
-      <c r="K162" s="30"/>
+    <row r="162" spans="1:20" ht="15">
+      <c r="A162" s="30" t="s">
+        <v>749</v>
+      </c>
+      <c r="B162" s="30" t="s">
+        <v>751</v>
+      </c>
+      <c r="C162" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="D162" s="31">
+        <v>533</v>
+      </c>
+      <c r="E162" s="31">
+        <v>750</v>
+      </c>
+      <c r="F162" s="85">
+        <v>0</v>
+      </c>
+      <c r="G162" s="85">
+        <v>1</v>
+      </c>
+      <c r="H162" s="86">
+        <f t="shared" ref="H162:H163" si="42">F162+IF(LEN(G162)=0,0,G162)</f>
+        <v>1</v>
+      </c>
+      <c r="I162" s="84">
+        <f>IF(D162&lt;&gt;"",D162,IFERROR(E162/(IFERROR(SUM([1]Sales!C:C),0))*(IFERROR(SUM([1]Purchases!C:C),0)),0))</f>
+        <v>533</v>
+      </c>
+      <c r="J162" s="84">
+        <f t="shared" ref="J162:J163" si="43">F162*I162</f>
+        <v>0</v>
+      </c>
+      <c r="K162" s="84">
+        <f t="shared" ref="K162:K163" si="44">IF(LEN(G162)=0,0,G162)*I162</f>
+        <v>533</v>
+      </c>
       <c r="L162" s="30"/>
       <c r="M162" s="30"/>
-      <c r="N162" s="30"/>
+      <c r="N162" s="30" t="s">
+        <v>222</v>
+      </c>
       <c r="O162" s="30"/>
       <c r="P162" s="30"/>
       <c r="Q162" s="30"/>
@@ -25260,21 +25400,49 @@
       <c r="S162" s="30"/>
       <c r="T162" s="30"/>
     </row>
-    <row r="163" spans="1:20">
-      <c r="A163" s="28"/>
-      <c r="B163" s="28"/>
-      <c r="C163" s="28"/>
-      <c r="D163" s="29"/>
-      <c r="E163" s="29"/>
-      <c r="F163" s="29"/>
-      <c r="G163" s="29"/>
-      <c r="H163" s="28"/>
-      <c r="I163" s="28"/>
-      <c r="J163" s="28"/>
-      <c r="K163" s="28"/>
+    <row r="163" spans="1:20" ht="15">
+      <c r="A163" s="28" t="s">
+        <v>750</v>
+      </c>
+      <c r="B163" s="28" t="s">
+        <v>752</v>
+      </c>
+      <c r="C163" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="D163" s="29">
+        <v>441</v>
+      </c>
+      <c r="E163" s="29">
+        <v>750</v>
+      </c>
+      <c r="F163" s="90">
+        <v>0</v>
+      </c>
+      <c r="G163" s="90">
+        <v>1</v>
+      </c>
+      <c r="H163" s="81">
+        <f t="shared" si="42"/>
+        <v>1</v>
+      </c>
+      <c r="I163" s="80">
+        <f>IF(D163&lt;&gt;"",D163,IFERROR(E163/(IFERROR(SUM([1]Sales!C:C),0))*(IFERROR(SUM([1]Purchases!C:C),0)),0))</f>
+        <v>441</v>
+      </c>
+      <c r="J163" s="80">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="K163" s="80">
+        <f t="shared" si="44"/>
+        <v>441</v>
+      </c>
       <c r="L163" s="28"/>
       <c r="M163" s="28"/>
-      <c r="N163" s="28"/>
+      <c r="N163" s="28" t="s">
+        <v>222</v>
+      </c>
       <c r="O163" s="28"/>
       <c r="P163" s="28"/>
       <c r="Q163" s="28"/>
@@ -25644,15 +25812,15 @@
       </c>
       <c r="B8" s="6">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>110846</v>
+        <v>112509</v>
       </c>
       <c r="C8" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D8" s="6">
         <f>B8-C8</f>
-        <v>18303.333333333328</v>
+        <v>19412</v>
       </c>
       <c r="E8" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE),0)</f>
@@ -25660,7 +25828,7 @@
       </c>
       <c r="F8" s="6">
         <f>D8+E8</f>
-        <v>18303.333333333328</v>
+        <v>19412</v>
       </c>
       <c r="G8" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -25668,7 +25836,7 @@
       </c>
       <c r="H8" s="8">
         <f>F8-G8</f>
-        <v>-6.6666666716628242E-3</v>
+        <v>1108.6599999999999</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -25681,11 +25849,11 @@
       </c>
       <c r="C9" s="7">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D9" s="7">
         <f>B9-C9</f>
-        <v>41639.333333333328</v>
+        <v>41085</v>
       </c>
       <c r="E9" s="7">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE),0)</f>
@@ -25693,7 +25861,7 @@
       </c>
       <c r="F9" s="7">
         <f>D9+E9</f>
-        <v>41639.333333333328</v>
+        <v>41085</v>
       </c>
       <c r="G9" s="7">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -25701,7 +25869,7 @@
       </c>
       <c r="H9" s="9">
         <f>F9-G9</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -25714,11 +25882,11 @@
       </c>
       <c r="C10" s="6">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>92542.666666666672</v>
+        <v>93097</v>
       </c>
       <c r="D10" s="6">
         <f>B10-C10</f>
-        <v>-59942.666666666672</v>
+        <v>-60497</v>
       </c>
       <c r="E10" s="6">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE),0)</f>
@@ -25726,7 +25894,7 @@
       </c>
       <c r="F10" s="6">
         <f>D10+E10</f>
-        <v>-59942.666666666672</v>
+        <v>-60497</v>
       </c>
       <c r="G10" s="6">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -25734,7 +25902,7 @@
       </c>
       <c r="H10" s="8">
         <f>F10-G10</f>
-        <v>3.3333333267364651E-3</v>
+        <v>-554.33000000000175</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="22" customFormat="1" ht="16" customHeight="1">
@@ -26151,7 +26319,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>218763</v>
+        <v>219963</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -26159,11 +26327,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>79319.860799999995</v>
+        <v>79719.940799999997</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>139443.13920000001</v>
+        <v>140243.05920000002</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26171,7 +26339,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>2133.1131999999925</v>
+        <v>2933.0332000000053</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -26188,11 +26356,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>79272.278399999996</v>
+        <v>79672.118399999992</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-72653.278399999996</v>
+        <v>-73053.118399999992</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26200,7 +26368,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-1066.2363999999943</v>
+        <v>-1466.0763999999908</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -26217,11 +26385,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>79319.860799999995</v>
+        <v>79719.940799999997</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-66789.860799999995</v>
+        <v>-67189.940799999997</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26229,7 +26397,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-1066.8767999999836</v>
+        <v>-1466.9567999999854</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
Malu Salwar and Aruna Salwar sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4523930-D614-BB4C-BA3B-78B1E56F58DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8E1FFA-A4FA-7841-90CC-24CEA5B6BEF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1889" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1895" uniqueCount="759">
   <si>
     <t>Notes:</t>
   </si>
@@ -2352,6 +2352,12 @@
   </si>
   <si>
     <t>Sushitha (XXL-1600)</t>
+  </si>
+  <si>
+    <t>Aanchal Maroon XXXL Salwar</t>
+  </si>
+  <si>
+    <t>Malu (1800)</t>
   </si>
 </sst>
 </file>
@@ -3232,7 +3238,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12448</c:v>
+                  <c:v>14248</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3487,7 +3493,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-9724</c:v>
+                  <c:v>-7924</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3810,10 +3816,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>192</c:v>
+                  <c:v>193</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>121</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4125,7 +4131,7 @@
                   <c:v>114</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4248,7 +4254,7 @@
                   <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>68</c:v>
+                  <c:v>67</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4675,7 +4681,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>70730</c:v>
+                  <c:v>68970</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>39825.919999999998</c:v>
@@ -8000,7 +8006,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>239112</v>
+        <v>241562</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -8017,7 +8023,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>243012</v>
+        <v>244812</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -8034,7 +8040,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-40179</v>
+        <v>-37729</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -8237,15 +8243,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>219963</v>
+        <v>220613</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>79719.940799999997</v>
+        <v>80536.770799999998</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>140243.05920000002</v>
+        <v>140076.2292</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8253,7 +8259,7 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>2933.0332000000053</v>
+        <v>2766.203199999989</v>
       </c>
       <c r="G26" s="71"/>
     </row>
@@ -8264,15 +8270,15 @@
       </c>
       <c r="B27" s="7">
         <f>'Cash Pool'!B5</f>
-        <v>6619</v>
+        <v>8419</v>
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>79672.118399999992</v>
+        <v>80488.458400000003</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-73053.118399999992</v>
+        <v>-72069.458400000003</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8280,7 +8286,7 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-1466.0763999999908</v>
+        <v>-482.41640000000189</v>
       </c>
       <c r="G27" s="72"/>
     </row>
@@ -8295,11 +8301,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>79719.940799999997</v>
+        <v>80536.770799999998</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-67189.940799999997</v>
+        <v>-68006.770799999998</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8307,7 +8313,7 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-1466.9567999999854</v>
+        <v>-2283.7867999999871</v>
       </c>
       <c r="G28" s="73"/>
     </row>
@@ -8405,7 +8411,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46103</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8421,7 +8427,7 @@
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>239112</v>
+        <v>241562</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8430,14 +8436,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-40179</v>
+        <v>-37729</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>111304.92</v>
+        <v>109544.92</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8481,7 +8487,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8505,7 +8511,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8518,11 +8524,11 @@
       </c>
       <c r="C12" s="15">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>12448</v>
+        <v>14248</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-9724</v>
+        <v>-7924</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8712,7 +8718,7 @@
       </c>
       <c r="K47" s="77" cm="1">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$478=J47)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>70730</v>
+        <v>68970</v>
       </c>
     </row>
     <row r="48" spans="6:11">
@@ -8721,11 +8727,11 @@
       </c>
       <c r="G48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J48" s="76" t="s">
         <v>120</v>
@@ -15292,7 +15298,7 @@
         <v>728</v>
       </c>
       <c r="I135" s="47" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -15370,16 +15376,30 @@
         <v>276</v>
       </c>
     </row>
-    <row r="139" spans="1:9">
-      <c r="A139" s="46"/>
-      <c r="B139" s="47"/>
-      <c r="C139" s="48"/>
-      <c r="D139" s="47"/>
-      <c r="E139" s="47"/>
+    <row r="139" spans="1:9" ht="16">
+      <c r="A139" s="46">
+        <v>46104</v>
+      </c>
+      <c r="B139" s="47" t="s">
+        <v>485</v>
+      </c>
+      <c r="C139" s="48">
+        <v>1800</v>
+      </c>
+      <c r="D139" s="47" t="s">
+        <v>277</v>
+      </c>
+      <c r="E139" s="47" t="s">
+        <v>47</v>
+      </c>
       <c r="F139" s="49"/>
       <c r="G139" s="49"/>
-      <c r="H139" s="68"/>
-      <c r="I139" s="47"/>
+      <c r="H139" s="68" t="s">
+        <v>757</v>
+      </c>
+      <c r="I139" s="47" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="140" spans="1:9">
       <c r="A140" s="43"/>
@@ -23502,13 +23522,13 @@
         <v>1760</v>
       </c>
       <c r="E126" s="31">
-        <v>2100</v>
+        <v>1800</v>
       </c>
       <c r="F126" s="85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G126" s="85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H126" s="86">
         <f t="shared" ref="H126:H127" si="12">F126+IF(LEN(G126)=0,0,G126)</f>
@@ -23520,16 +23540,18 @@
       </c>
       <c r="J126" s="84">
         <f t="shared" ref="J126:J127" si="13">F126*I126</f>
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="K126" s="84">
         <f t="shared" ref="K126:K127" si="14">IF(LEN(G126)=0,0,G126)*I126</f>
-        <v>1760</v>
-      </c>
-      <c r="L126" s="30"/>
+        <v>0</v>
+      </c>
+      <c r="L126" s="30" t="s">
+        <v>758</v>
+      </c>
       <c r="M126" s="30"/>
       <c r="N126" s="30" t="s">
-        <v>191</v>
+        <v>122</v>
       </c>
       <c r="O126" s="30" t="s">
         <v>544</v>
@@ -26319,7 +26341,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>219963</v>
+        <v>220613</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -26327,11 +26349,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>79719.940799999997</v>
+        <v>80536.770799999998</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>140243.05920000002</v>
+        <v>140076.2292</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26339,7 +26361,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>2933.0332000000053</v>
+        <v>2766.203199999989</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -26348,7 +26370,7 @@
       </c>
       <c r="B5" s="7">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A5,Sales!$I:$I,"Completed"),0)</f>
-        <v>6619</v>
+        <v>8419</v>
       </c>
       <c r="C5" s="7">
         <f>VLOOKUP($A5,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -26356,11 +26378,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>79672.118399999992</v>
+        <v>80488.458400000003</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-73053.118399999992</v>
+        <v>-72069.458400000003</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26368,7 +26390,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-1466.0763999999908</v>
+        <v>-482.41640000000189</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -26385,11 +26407,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>79719.940799999997</v>
+        <v>80536.770799999998</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-67189.940799999997</v>
+        <v>-68006.770799999998</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26397,7 +26419,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-1466.9567999999854</v>
+        <v>-2283.7867999999871</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>

<commit_message>
Chris sales & sheeja mol maid returns
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Business-Summary-Latest.xlsx
+++ b/docs/Chiraath-Business-Summary-Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8E1FFA-A4FA-7841-90CC-24CEA5B6BEF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF2D1E0-6187-7F49-A4CF-3B03697B1CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1895" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1896" uniqueCount="759">
   <si>
     <t>Notes:</t>
   </si>
@@ -1972,9 +1972,6 @@
   </si>
   <si>
     <t>Soft Cotton Saree (with butterfly design on Pallu)</t>
-  </si>
-  <si>
-    <t>Linen Saree with Check (Maroon with golden checks, Green with golden checks, Rust Orange with golden checks)</t>
   </si>
   <si>
     <t>Nisha Sajith (Chengannur)</t>
@@ -2143,9 +2140,6 @@
     <t>Tissue silk floral</t>
   </si>
   <si>
-    <t>Saranya Gopalakrishnan(1300 pending)</t>
-  </si>
-  <si>
     <t>Aanchal cotton salwars</t>
   </si>
   <si>
@@ -2164,9 +2158,6 @@
     <t>Haris (EKM)</t>
   </si>
   <si>
-    <t>Sheeja mol maid</t>
-  </si>
-  <si>
     <t>Sheeja mol</t>
   </si>
   <si>
@@ -2177,12 +2168,6 @@
   </si>
   <si>
     <t>Jisha (1545-XL), Shiji(1370-L), Sheejamol(XXL)-850</t>
-  </si>
-  <si>
-    <t>Aanchal Blue - 1200</t>
-  </si>
-  <si>
-    <t>Sheeja mol maid(1200)</t>
   </si>
   <si>
     <t>Praneetha (Kochi)</t>
@@ -2291,9 +2276,6 @@
     <t>Georgette maroon</t>
   </si>
   <si>
-    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550, Vineet(Maroon): 1550</t>
-  </si>
-  <si>
     <t>Latha(Yellow), Sari(Peach)</t>
   </si>
   <si>
@@ -2358,6 +2340,24 @@
   </si>
   <si>
     <t>Malu (1800)</t>
+  </si>
+  <si>
+    <t>Viscose Georgette(Black Yellow), Net Kota Arrow, Linen Green with Golden Checks</t>
+  </si>
+  <si>
+    <t>Chris (1000 - Green)</t>
+  </si>
+  <si>
+    <t>Linen Saree with Check (Maroon with golden checks, Rust Orange with golden checks)</t>
+  </si>
+  <si>
+    <t>Chris (1250)</t>
+  </si>
+  <si>
+    <t>Amalu(black/maroon), Lethy(Thiruvalla):1550, Vineet(Maroon): 1550, Chris(Yellow) - 1250</t>
+  </si>
+  <si>
+    <t>Saranya Gopalakrishnan(1300)</t>
   </si>
 </sst>
 </file>
@@ -3238,7 +3238,7 @@
                   <c:v>19089</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14248</c:v>
+                  <c:v>16548</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3493,7 +3493,7 @@
                   <c:v>14299</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-7924</c:v>
+                  <c:v>-5624</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3816,10 +3816,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>193</c:v>
+                  <c:v>195</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>120</c:v>
+                  <c:v>118</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4128,10 +4128,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>114</c:v>
+                  <c:v>117</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77</c:v>
+                  <c:v>76</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4251,10 +4251,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>48</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>67</c:v>
+                  <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4681,10 +4681,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>68970</c:v>
+                  <c:v>69946</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39825.919999999998</c:v>
+                  <c:v>36655.160000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1829</c:v>
@@ -8006,7 +8006,7 @@
       </c>
       <c r="B4" s="52">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>241562</v>
+        <v>245062</v>
       </c>
       <c r="E4" s="6" t="str">
         <f>PartnerShares!A3</f>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="B5" s="53">
         <f>SUM(Sales!C:C)</f>
-        <v>244812</v>
+        <v>247112</v>
       </c>
       <c r="E5" s="7" t="str">
         <f>PartnerShares!A4</f>
@@ -8040,7 +8040,7 @@
       </c>
       <c r="B6" s="52">
         <f>B4-B3</f>
-        <v>-37729</v>
+        <v>-34229</v>
       </c>
       <c r="E6" s="6" t="str">
         <f>PartnerShares!A5</f>
@@ -8243,15 +8243,15 @@
       </c>
       <c r="B26" s="6">
         <f>'Cash Pool'!B4</f>
-        <v>220613</v>
+        <v>224113</v>
       </c>
       <c r="C26" s="6">
         <f>'Cash Pool'!D4</f>
-        <v>80536.770799999998</v>
+        <v>81703.670799999993</v>
       </c>
       <c r="D26" s="6">
         <f>'Cash Pool'!E4</f>
-        <v>140076.2292</v>
+        <v>142409.32920000001</v>
       </c>
       <c r="E26" s="6">
         <f>'Cash Pool'!F4</f>
@@ -8259,7 +8259,7 @@
       </c>
       <c r="F26" s="8">
         <f>'Cash Pool'!G4</f>
-        <v>2766.203199999989</v>
+        <v>5099.3031999999948</v>
       </c>
       <c r="G26" s="71"/>
     </row>
@@ -8274,11 +8274,11 @@
       </c>
       <c r="C27" s="7">
         <f>'Cash Pool'!D5</f>
-        <v>80488.458400000003</v>
+        <v>81654.6584</v>
       </c>
       <c r="D27" s="7">
         <f>'Cash Pool'!E5</f>
-        <v>-72069.458400000003</v>
+        <v>-73235.6584</v>
       </c>
       <c r="E27" s="7">
         <f>'Cash Pool'!F5</f>
@@ -8286,7 +8286,7 @@
       </c>
       <c r="F27" s="9">
         <f>'Cash Pool'!G5</f>
-        <v>-482.41640000000189</v>
+        <v>-1648.616399999999</v>
       </c>
       <c r="G27" s="72"/>
     </row>
@@ -8301,11 +8301,11 @@
       </c>
       <c r="C28" s="6">
         <f>'Cash Pool'!D6</f>
-        <v>80536.770799999998</v>
+        <v>81703.670799999993</v>
       </c>
       <c r="D28" s="6">
         <f>'Cash Pool'!E6</f>
-        <v>-68006.770799999998</v>
+        <v>-69173.670799999993</v>
       </c>
       <c r="E28" s="6">
         <f>'Cash Pool'!F6</f>
@@ -8313,7 +8313,7 @@
       </c>
       <c r="F28" s="8">
         <f>'Cash Pool'!G6</f>
-        <v>-2283.7867999999871</v>
+        <v>-3450.6867999999813</v>
       </c>
       <c r="G28" s="73"/>
     </row>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="B3">
         <f ca="1">TODAY()</f>
-        <v>46103</v>
+        <v>46105</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="E5" s="15">
         <f>Summary!B4</f>
-        <v>241562</v>
+        <v>245062</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8436,14 +8436,14 @@
       </c>
       <c r="B6" s="15">
         <f>Summary!B6</f>
-        <v>-37729</v>
+        <v>-34229</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E6" s="15">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>109544.92</v>
+        <v>107350.16</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8475,7 +8475,7 @@
         <v>47311</v>
       </c>
       <c r="C10" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A10)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A10)*Sales!$C$2:$C$997),0)</f>
         <v>45448</v>
       </c>
       <c r="D10" s="15">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="G10" s="15">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -8499,7 +8499,7 @@
         <v>4790</v>
       </c>
       <c r="C11" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A11)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A11)*Sales!$C$2:$C$997),0)</f>
         <v>19089</v>
       </c>
       <c r="D11" s="19">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G11" s="19">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -8523,12 +8523,12 @@
         <v>22172</v>
       </c>
       <c r="C12" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A12)*Sales!$C$2:$C$998),0)</f>
-        <v>14248</v>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A12)*Sales!$C$2:$C$997),0)</f>
+        <v>16548</v>
       </c>
       <c r="D12" s="15">
         <f t="shared" si="0"/>
-        <v>-7924</v>
+        <v>-5624</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -8540,7 +8540,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A13)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A13)*Sales!$C$2:$C$997),0)</f>
         <v>0</v>
       </c>
       <c r="D13" s="19">
@@ -8557,7 +8557,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A14)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A14)*Sales!$C$2:$C$997),0)</f>
         <v>0</v>
       </c>
       <c r="D14" s="15">
@@ -8574,7 +8574,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A15)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A15)*Sales!$C$2:$C$997),0)</f>
         <v>0</v>
       </c>
       <c r="D15" s="19">
@@ -8591,7 +8591,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A16)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A16)*Sales!$C$2:$C$997),0)</f>
         <v>0</v>
       </c>
       <c r="D16" s="15">
@@ -8608,7 +8608,7 @@
         <v>100869</v>
       </c>
       <c r="C17" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A17)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A17)*Sales!$C$2:$C$997),0)</f>
         <v>12600</v>
       </c>
       <c r="D17" s="19">
@@ -8625,7 +8625,7 @@
         <v>2304</v>
       </c>
       <c r="C18" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A18)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A18)*Sales!$C$2:$C$997),0)</f>
         <v>62800</v>
       </c>
       <c r="D18" s="15">
@@ -8642,7 +8642,7 @@
         <v>50547</v>
       </c>
       <c r="C19" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A19)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A19)*Sales!$C$2:$C$997),0)</f>
         <v>24259</v>
       </c>
       <c r="D19" s="19">
@@ -8659,7 +8659,7 @@
         <v>38048</v>
       </c>
       <c r="C20" s="15">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A20)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A20)*Sales!$C$2:$C$997),0)</f>
         <v>14200</v>
       </c>
       <c r="D20" s="15">
@@ -8676,7 +8676,7 @@
         <v>13250</v>
       </c>
       <c r="C21" s="19">
-        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$998,"MMM")=$A21)*Sales!$C$2:$C$998),0)</f>
+        <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$997,"MMM")=$A21)*Sales!$C$2:$C$997),0)</f>
         <v>52168</v>
       </c>
       <c r="D21" s="19">
@@ -8707,18 +8707,18 @@
       </c>
       <c r="G47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H47" s="76">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="J47" s="76" t="s">
         <v>135</v>
       </c>
       <c r="K47" s="77" cm="1">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$478=J47)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>68970</v>
+        <v>69946</v>
       </c>
     </row>
     <row r="48" spans="6:11">
@@ -8727,18 +8727,18 @@
       </c>
       <c r="G48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H48" s="76">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J48" s="76" t="s">
         <v>120</v>
       </c>
       <c r="K48" s="77" cm="1">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$478=J48)*(INVENTORY!$D$2:$D$478)*(INVENTORY!$G$2:$G$478))</f>
-        <v>39825.919999999998</v>
+        <v>36655.160000000003</v>
       </c>
     </row>
     <row r="49" spans="5:12">
@@ -9502,7 +9502,7 @@
         <v>1290</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="E48" s="91"/>
     </row>
@@ -9517,7 +9517,7 @@
         <v>3500</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -9531,7 +9531,7 @@
         <v>6328</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -9545,7 +9545,7 @@
         <v>3164</v>
       </c>
       <c r="D51" s="37" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -9601,7 +9601,7 @@
         <v>5594</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -9615,7 +9615,7 @@
         <v>2796</v>
       </c>
       <c r="D56" s="39" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -9643,7 +9643,7 @@
         <v>1663</v>
       </c>
       <c r="D58" s="39" t="s">
-        <v>746</v>
+        <v>740</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -12006,7 +12006,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:I262"/>
+  <dimension ref="A1:I261"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -14531,7 +14531,7 @@
         <v>46049</v>
       </c>
       <c r="B105" s="47" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C105" s="48">
         <v>1380</v>
@@ -14556,7 +14556,7 @@
         <v>46049</v>
       </c>
       <c r="B106" s="50" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C106" s="51">
         <v>1380</v>
@@ -14570,7 +14570,7 @@
       <c r="F106" s="50"/>
       <c r="G106" s="50"/>
       <c r="H106" s="69" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="I106" s="50" t="s">
         <v>276</v>
@@ -14581,7 +14581,7 @@
         <v>46049</v>
       </c>
       <c r="B107" s="47" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C107" s="48">
         <v>1200</v>
@@ -14595,7 +14595,7 @@
       <c r="F107" s="49"/>
       <c r="G107" s="49"/>
       <c r="H107" s="68" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="I107" s="47" t="s">
         <v>276</v>
@@ -14606,7 +14606,7 @@
         <v>46050</v>
       </c>
       <c r="B108" s="50" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C108" s="51">
         <v>1250</v>
@@ -14620,7 +14620,7 @@
       <c r="F108" s="50"/>
       <c r="G108" s="50"/>
       <c r="H108" s="69" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="I108" s="50" t="s">
         <v>276</v>
@@ -14631,7 +14631,7 @@
         <v>46051</v>
       </c>
       <c r="B109" s="47" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C109" s="48">
         <v>1380</v>
@@ -14656,7 +14656,7 @@
         <v>46051</v>
       </c>
       <c r="B110" s="50" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C110" s="51">
         <v>1380</v>
@@ -14687,7 +14687,7 @@
         <v>580</v>
       </c>
       <c r="D111" s="47" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E111" s="47" t="s">
         <v>48</v>
@@ -14695,7 +14695,7 @@
       <c r="F111" s="49"/>
       <c r="G111" s="49"/>
       <c r="H111" s="68" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="I111" s="47" t="s">
         <v>276</v>
@@ -14706,7 +14706,7 @@
         <v>46054</v>
       </c>
       <c r="B112" s="50" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="C112" s="51">
         <v>1800</v>
@@ -14720,7 +14720,7 @@
       <c r="F112" s="50"/>
       <c r="G112" s="50"/>
       <c r="H112" s="69" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="I112" s="50" t="s">
         <v>276</v>
@@ -14731,7 +14731,7 @@
         <v>46054</v>
       </c>
       <c r="B113" s="47" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="C113" s="48">
         <v>1550</v>
@@ -14795,7 +14795,7 @@
       <c r="F115" s="49"/>
       <c r="G115" s="49"/>
       <c r="H115" s="68" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="I115" s="47" t="s">
         <v>276</v>
@@ -14806,7 +14806,7 @@
         <v>46060</v>
       </c>
       <c r="B116" s="50" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C116" s="51">
         <v>1050</v>
@@ -14820,7 +14820,7 @@
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
       <c r="H116" s="69" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="I116" s="50" t="s">
         <v>276</v>
@@ -14831,7 +14831,7 @@
         <v>46062</v>
       </c>
       <c r="B117" s="47" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C117" s="48">
         <v>1000</v>
@@ -14856,7 +14856,7 @@
         <v>46065</v>
       </c>
       <c r="B118" s="50" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="C118" s="51">
         <v>799</v>
@@ -14881,7 +14881,7 @@
         <v>46055</v>
       </c>
       <c r="B119" s="47" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C119" s="48">
         <v>500</v>
@@ -14906,13 +14906,13 @@
         <v>46070</v>
       </c>
       <c r="B120" s="50" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="C120" s="51">
         <v>1450</v>
       </c>
       <c r="D120" s="50" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="E120" s="50" t="s">
         <v>46</v>
@@ -14945,7 +14945,7 @@
       <c r="F121" s="49"/>
       <c r="G121" s="49"/>
       <c r="H121" s="68" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="I121" s="47" t="s">
         <v>276</v>
@@ -14956,7 +14956,7 @@
         <v>46074</v>
       </c>
       <c r="B122" s="50" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="C122" s="51">
         <v>1200</v>
@@ -14970,7 +14970,7 @@
       <c r="F122" s="50"/>
       <c r="G122" s="50"/>
       <c r="H122" s="69" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="I122" s="50" t="s">
         <v>276</v>
@@ -14981,7 +14981,7 @@
         <v>46075</v>
       </c>
       <c r="B123" s="47" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C123" s="48">
         <v>1380</v>
@@ -15006,7 +15006,7 @@
         <v>46075</v>
       </c>
       <c r="B124" s="50" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C124" s="51">
         <v>2550</v>
@@ -15020,7 +15020,7 @@
       <c r="F124" s="50"/>
       <c r="G124" s="50"/>
       <c r="H124" s="69" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="I124" s="50" t="s">
         <v>276</v>
@@ -15045,7 +15045,7 @@
       <c r="F125" s="49"/>
       <c r="G125" s="49"/>
       <c r="H125" s="68" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="I125" s="47" t="s">
         <v>276</v>
@@ -15056,7 +15056,7 @@
         <v>46079</v>
       </c>
       <c r="B126" s="50" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C126" s="51">
         <v>500</v>
@@ -15070,7 +15070,7 @@
       <c r="F126" s="50"/>
       <c r="G126" s="50"/>
       <c r="H126" s="69" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="I126" s="50" t="s">
         <v>276</v>
@@ -15081,7 +15081,7 @@
         <v>46090</v>
       </c>
       <c r="B127" s="47" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C127" s="48">
         <v>850</v>
@@ -15095,7 +15095,7 @@
       <c r="F127" s="49"/>
       <c r="G127" s="49"/>
       <c r="H127" s="28" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="I127" s="47" t="s">
         <v>276</v>
@@ -15106,7 +15106,7 @@
         <v>46090</v>
       </c>
       <c r="B128" s="50" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C128" s="51">
         <v>1100</v>
@@ -15120,803 +15120,803 @@
       <c r="F128" s="50"/>
       <c r="G128" s="50"/>
       <c r="H128" s="69" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="I128" s="50" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="16">
-      <c r="A129" s="46">
+    <row r="129" spans="1:9">
+      <c r="A129" s="43">
         <v>46090</v>
       </c>
-      <c r="B129" s="47" t="s">
-        <v>694</v>
-      </c>
-      <c r="C129" s="48">
+      <c r="B129" s="50" t="s">
+        <v>692</v>
+      </c>
+      <c r="C129" s="51">
+        <v>800</v>
+      </c>
+      <c r="D129" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E129" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="F129" s="50"/>
+      <c r="G129" s="50"/>
+      <c r="H129" s="69" t="s">
+        <v>735</v>
+      </c>
+      <c r="I129" s="50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="16">
+      <c r="A130" s="46">
+        <v>46091</v>
+      </c>
+      <c r="B130" s="47" t="s">
+        <v>696</v>
+      </c>
+      <c r="C130" s="48">
+        <v>1099</v>
+      </c>
+      <c r="D130" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E130" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="F130" s="49"/>
+      <c r="G130" s="49"/>
+      <c r="H130" s="68" t="s">
+        <v>697</v>
+      </c>
+      <c r="I130" s="47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9">
+      <c r="A131" s="43">
+        <v>46092</v>
+      </c>
+      <c r="B131" s="50" t="s">
+        <v>690</v>
+      </c>
+      <c r="C131" s="51">
         <v>1200</v>
       </c>
-      <c r="D129" s="47" t="s">
+      <c r="D131" s="50" t="s">
         <v>281</v>
       </c>
-      <c r="E129" s="47" t="s">
+      <c r="E131" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="F129" s="49"/>
-      <c r="G129" s="49"/>
-      <c r="H129" s="68" t="s">
+      <c r="F131" s="50"/>
+      <c r="G131" s="50"/>
+      <c r="H131" s="69" t="s">
+        <v>698</v>
+      </c>
+      <c r="I131" s="50" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" ht="16">
+      <c r="A132" s="46">
+        <v>46092</v>
+      </c>
+      <c r="B132" s="47" t="s">
         <v>699</v>
       </c>
-      <c r="I129" s="47" t="s">
+      <c r="C132" s="48">
+        <v>1099</v>
+      </c>
+      <c r="D132" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E132" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="F132" s="49"/>
+      <c r="G132" s="49"/>
+      <c r="H132" s="68" t="s">
+        <v>700</v>
+      </c>
+      <c r="I132" s="47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9">
+      <c r="A133" s="43">
+        <v>46093</v>
+      </c>
+      <c r="B133" s="50" t="s">
+        <v>508</v>
+      </c>
+      <c r="C133" s="51">
+        <v>850</v>
+      </c>
+      <c r="D133" s="50" t="s">
+        <v>281</v>
+      </c>
+      <c r="E133" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="F133" s="50"/>
+      <c r="G133" s="50"/>
+      <c r="H133" s="69" t="s">
+        <v>736</v>
+      </c>
+      <c r="I133" s="50" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="130" spans="1:9">
-      <c r="A130" s="43">
-        <v>46090</v>
-      </c>
-      <c r="B130" s="50" t="s">
-        <v>695</v>
-      </c>
-      <c r="C130" s="51">
-        <v>800</v>
-      </c>
-      <c r="D130" s="50" t="s">
+    <row r="134" spans="1:9" ht="16">
+      <c r="A134" s="46">
+        <v>46093</v>
+      </c>
+      <c r="B134" s="47" t="s">
+        <v>324</v>
+      </c>
+      <c r="C134" s="48">
+        <v>650</v>
+      </c>
+      <c r="D134" s="47" t="s">
         <v>281</v>
       </c>
-      <c r="E130" s="50" t="s">
+      <c r="E134" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="F130" s="50"/>
-      <c r="G130" s="50"/>
-      <c r="H130" s="69" t="s">
-        <v>741</v>
-      </c>
-      <c r="I130" s="50" t="s">
+      <c r="F134" s="49"/>
+      <c r="G134" s="49"/>
+      <c r="H134" s="68" t="s">
+        <v>723</v>
+      </c>
+      <c r="I134" s="47" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="16">
-      <c r="A131" s="46">
-        <v>46091</v>
-      </c>
-      <c r="B131" s="47" t="s">
-        <v>701</v>
-      </c>
-      <c r="C131" s="48">
-        <v>1099</v>
-      </c>
-      <c r="D131" s="47" t="s">
+    <row r="135" spans="1:9">
+      <c r="A135" s="43">
+        <v>46097</v>
+      </c>
+      <c r="B135" s="50" t="s">
+        <v>729</v>
+      </c>
+      <c r="C135" s="51">
+        <v>1550</v>
+      </c>
+      <c r="D135" s="50" t="s">
         <v>281</v>
       </c>
-      <c r="E131" s="47" t="s">
+      <c r="E135" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="F131" s="49"/>
-      <c r="G131" s="49"/>
-      <c r="H131" s="68" t="s">
-        <v>702</v>
-      </c>
-      <c r="I131" s="47" t="s">
+      <c r="F135" s="50"/>
+      <c r="G135" s="50"/>
+      <c r="H135" s="69" t="s">
+        <v>730</v>
+      </c>
+      <c r="I135" s="50" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="132" spans="1:9">
-      <c r="A132" s="43">
-        <v>46092</v>
-      </c>
-      <c r="B132" s="50" t="s">
-        <v>692</v>
-      </c>
-      <c r="C132" s="51">
+    <row r="136" spans="1:9" ht="16">
+      <c r="A136" s="46">
+        <v>46097</v>
+      </c>
+      <c r="B136" s="47" t="s">
+        <v>733</v>
+      </c>
+      <c r="C136" s="48">
+        <v>850</v>
+      </c>
+      <c r="D136" s="47" t="s">
+        <v>281</v>
+      </c>
+      <c r="E136" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="F136" s="49"/>
+      <c r="G136" s="49"/>
+      <c r="H136" s="68" t="s">
+        <v>734</v>
+      </c>
+      <c r="I136" s="47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9">
+      <c r="A137" s="43">
+        <v>46100</v>
+      </c>
+      <c r="B137" s="50" t="s">
+        <v>749</v>
+      </c>
+      <c r="C137" s="51">
         <v>1200</v>
       </c>
-      <c r="D132" s="50" t="s">
+      <c r="D137" s="50" t="s">
         <v>281</v>
       </c>
-      <c r="E132" s="50" t="s">
+      <c r="E137" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="F132" s="50"/>
-      <c r="G132" s="50"/>
-      <c r="H132" s="69" t="s">
-        <v>703</v>
-      </c>
-      <c r="I132" s="50" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="133" spans="1:9" ht="16">
-      <c r="A133" s="46">
-        <v>46092</v>
-      </c>
-      <c r="B133" s="47" t="s">
-        <v>704</v>
-      </c>
-      <c r="C133" s="48">
-        <v>1099</v>
-      </c>
-      <c r="D133" s="47" t="s">
+      <c r="F137" s="50"/>
+      <c r="G137" s="50"/>
+      <c r="H137" s="69" t="s">
+        <v>99</v>
+      </c>
+      <c r="I137" s="50" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" ht="16">
+      <c r="A138" s="46">
+        <v>46104</v>
+      </c>
+      <c r="B138" s="47" t="s">
+        <v>485</v>
+      </c>
+      <c r="C138" s="48">
+        <v>1800</v>
+      </c>
+      <c r="D138" s="47" t="s">
+        <v>277</v>
+      </c>
+      <c r="E138" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="F138" s="49"/>
+      <c r="G138" s="49"/>
+      <c r="H138" s="68" t="s">
+        <v>751</v>
+      </c>
+      <c r="I138" s="47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" ht="28">
+      <c r="A139" s="43">
+        <v>46105</v>
+      </c>
+      <c r="B139" s="50" t="s">
+        <v>121</v>
+      </c>
+      <c r="C139" s="51">
+        <v>3500</v>
+      </c>
+      <c r="D139" s="50" t="s">
         <v>281</v>
       </c>
-      <c r="E133" s="47" t="s">
+      <c r="E139" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="F133" s="49"/>
-      <c r="G133" s="49"/>
-      <c r="H133" s="68" t="s">
-        <v>705</v>
-      </c>
-      <c r="I133" s="47" t="s">
+      <c r="F139" s="50"/>
+      <c r="G139" s="50"/>
+      <c r="H139" s="69" t="s">
+        <v>753</v>
+      </c>
+      <c r="I139" s="50" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="134" spans="1:9">
-      <c r="A134" s="43">
-        <v>46093</v>
-      </c>
-      <c r="B134" s="50" t="s">
-        <v>508</v>
-      </c>
-      <c r="C134" s="51">
-        <v>850</v>
-      </c>
-      <c r="D134" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="E134" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="F134" s="50"/>
-      <c r="G134" s="50"/>
-      <c r="H134" s="69" t="s">
-        <v>742</v>
-      </c>
-      <c r="I134" s="50" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="135" spans="1:9" ht="16">
-      <c r="A135" s="46">
-        <v>46093</v>
-      </c>
-      <c r="B135" s="47" t="s">
-        <v>324</v>
-      </c>
-      <c r="C135" s="48">
-        <v>650</v>
-      </c>
-      <c r="D135" s="47" t="s">
-        <v>281</v>
-      </c>
-      <c r="E135" s="47" t="s">
-        <v>46</v>
-      </c>
-      <c r="F135" s="49"/>
-      <c r="G135" s="49"/>
-      <c r="H135" s="68" t="s">
-        <v>728</v>
-      </c>
-      <c r="I135" s="47" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="136" spans="1:9">
-      <c r="A136" s="43">
-        <v>46097</v>
-      </c>
-      <c r="B136" s="50" t="s">
-        <v>734</v>
-      </c>
-      <c r="C136" s="51">
-        <v>1550</v>
-      </c>
-      <c r="D136" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="E136" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="F136" s="50"/>
-      <c r="G136" s="50"/>
-      <c r="H136" s="69" t="s">
-        <v>735</v>
-      </c>
-      <c r="I136" s="50" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="137" spans="1:9" ht="16">
-      <c r="A137" s="46">
-        <v>46097</v>
-      </c>
-      <c r="B137" s="47" t="s">
-        <v>739</v>
-      </c>
-      <c r="C137" s="48">
-        <v>850</v>
-      </c>
-      <c r="D137" s="47" t="s">
-        <v>281</v>
-      </c>
-      <c r="E137" s="47" t="s">
-        <v>46</v>
-      </c>
-      <c r="F137" s="49"/>
-      <c r="G137" s="49"/>
-      <c r="H137" s="68" t="s">
-        <v>740</v>
-      </c>
-      <c r="I137" s="47" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="138" spans="1:9">
-      <c r="A138" s="43">
-        <v>46100</v>
-      </c>
-      <c r="B138" s="50" t="s">
-        <v>755</v>
-      </c>
-      <c r="C138" s="51">
-        <v>1200</v>
-      </c>
-      <c r="D138" s="50" t="s">
-        <v>281</v>
-      </c>
-      <c r="E138" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="F138" s="50"/>
-      <c r="G138" s="50"/>
-      <c r="H138" s="69" t="s">
-        <v>99</v>
-      </c>
-      <c r="I138" s="50" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="139" spans="1:9" ht="16">
-      <c r="A139" s="46">
-        <v>46104</v>
-      </c>
-      <c r="B139" s="47" t="s">
-        <v>485</v>
-      </c>
-      <c r="C139" s="48">
-        <v>1800</v>
-      </c>
-      <c r="D139" s="47" t="s">
-        <v>277</v>
-      </c>
-      <c r="E139" s="47" t="s">
-        <v>47</v>
-      </c>
-      <c r="F139" s="49"/>
-      <c r="G139" s="49"/>
-      <c r="H139" s="68" t="s">
-        <v>757</v>
-      </c>
-      <c r="I139" s="47" t="s">
-        <v>276</v>
-      </c>
-    </row>
     <row r="140" spans="1:9">
-      <c r="A140" s="43"/>
-      <c r="B140" s="50"/>
-      <c r="C140" s="51"/>
-      <c r="D140" s="50"/>
-      <c r="E140" s="50"/>
-      <c r="F140" s="50"/>
-      <c r="G140" s="50"/>
-      <c r="H140" s="69"/>
-      <c r="I140" s="50"/>
+      <c r="A140" s="46"/>
+      <c r="B140" s="47"/>
+      <c r="C140" s="48"/>
+      <c r="D140" s="47"/>
+      <c r="E140" s="47"/>
+      <c r="F140" s="49"/>
+      <c r="G140" s="49"/>
+      <c r="H140" s="68"/>
+      <c r="I140" s="47"/>
     </row>
     <row r="141" spans="1:9">
-      <c r="A141" s="46"/>
-      <c r="B141" s="47"/>
-      <c r="C141" s="48"/>
-      <c r="D141" s="47"/>
-      <c r="E141" s="47"/>
-      <c r="F141" s="49"/>
-      <c r="G141" s="49"/>
-      <c r="H141" s="68"/>
-      <c r="I141" s="47"/>
+      <c r="A141" s="43"/>
+      <c r="B141" s="50"/>
+      <c r="C141" s="51"/>
+      <c r="D141" s="50"/>
+      <c r="E141" s="50"/>
+      <c r="F141" s="50"/>
+      <c r="G141" s="50"/>
+      <c r="H141" s="69"/>
+      <c r="I141" s="50"/>
     </row>
     <row r="142" spans="1:9">
-      <c r="A142" s="43"/>
-      <c r="B142" s="50"/>
-      <c r="C142" s="51"/>
-      <c r="D142" s="50"/>
-      <c r="E142" s="50"/>
-      <c r="F142" s="50"/>
-      <c r="G142" s="50"/>
-      <c r="H142" s="69"/>
-      <c r="I142" s="50"/>
+      <c r="A142" s="46"/>
+      <c r="B142" s="47"/>
+      <c r="C142" s="48"/>
+      <c r="D142" s="47"/>
+      <c r="E142" s="47"/>
+      <c r="F142" s="49"/>
+      <c r="G142" s="49"/>
+      <c r="H142" s="68"/>
+      <c r="I142" s="47"/>
     </row>
     <row r="143" spans="1:9">
-      <c r="A143" s="46"/>
-      <c r="B143" s="47"/>
-      <c r="C143" s="48"/>
-      <c r="D143" s="47"/>
-      <c r="E143" s="47"/>
-      <c r="F143" s="49"/>
-      <c r="G143" s="49"/>
-      <c r="H143" s="68"/>
-      <c r="I143" s="47"/>
+      <c r="A143" s="43"/>
+      <c r="B143" s="50"/>
+      <c r="C143" s="51"/>
+      <c r="D143" s="50"/>
+      <c r="E143" s="50"/>
+      <c r="F143" s="50"/>
+      <c r="G143" s="50"/>
+      <c r="H143" s="69"/>
+      <c r="I143" s="50"/>
     </row>
     <row r="144" spans="1:9">
-      <c r="A144" s="43"/>
-      <c r="B144" s="50"/>
-      <c r="C144" s="51"/>
-      <c r="D144" s="50"/>
-      <c r="E144" s="50"/>
-      <c r="F144" s="50"/>
-      <c r="G144" s="50"/>
-      <c r="H144" s="69"/>
-      <c r="I144" s="50"/>
+      <c r="A144" s="46"/>
+      <c r="B144" s="47"/>
+      <c r="C144" s="48"/>
+      <c r="D144" s="47"/>
+      <c r="E144" s="47"/>
+      <c r="F144" s="49"/>
+      <c r="G144" s="49"/>
+      <c r="H144" s="68"/>
+      <c r="I144" s="47"/>
     </row>
     <row r="145" spans="1:9">
-      <c r="A145" s="46"/>
-      <c r="B145" s="47"/>
-      <c r="C145" s="48"/>
-      <c r="D145" s="47"/>
-      <c r="E145" s="47"/>
-      <c r="F145" s="49"/>
-      <c r="G145" s="49"/>
-      <c r="H145" s="68"/>
-      <c r="I145" s="47"/>
+      <c r="A145" s="43"/>
+      <c r="B145" s="50"/>
+      <c r="C145" s="51"/>
+      <c r="D145" s="50"/>
+      <c r="E145" s="50"/>
+      <c r="F145" s="50"/>
+      <c r="G145" s="50"/>
+      <c r="H145" s="69"/>
+      <c r="I145" s="50"/>
     </row>
     <row r="146" spans="1:9">
-      <c r="A146" s="43"/>
-      <c r="B146" s="50"/>
-      <c r="C146" s="51"/>
-      <c r="D146" s="50"/>
-      <c r="E146" s="50"/>
-      <c r="F146" s="50"/>
-      <c r="G146" s="50"/>
-      <c r="H146" s="69"/>
-      <c r="I146" s="50"/>
+      <c r="A146" s="46"/>
+      <c r="B146" s="47"/>
+      <c r="C146" s="48"/>
+      <c r="D146" s="47"/>
+      <c r="E146" s="47"/>
+      <c r="F146" s="49"/>
+      <c r="G146" s="49"/>
+      <c r="H146" s="68"/>
+      <c r="I146" s="47"/>
     </row>
     <row r="147" spans="1:9">
-      <c r="A147" s="46"/>
-      <c r="B147" s="47"/>
-      <c r="C147" s="48"/>
-      <c r="D147" s="47"/>
-      <c r="E147" s="47"/>
-      <c r="F147" s="49"/>
-      <c r="G147" s="49"/>
-      <c r="H147" s="68"/>
-      <c r="I147" s="47"/>
+      <c r="A147" s="43"/>
+      <c r="B147" s="50"/>
+      <c r="C147" s="51"/>
+      <c r="D147" s="50"/>
+      <c r="E147" s="50"/>
+      <c r="F147" s="50"/>
+      <c r="G147" s="50"/>
+      <c r="H147" s="69"/>
+      <c r="I147" s="50"/>
     </row>
     <row r="148" spans="1:9">
-      <c r="A148" s="43"/>
-      <c r="B148" s="50"/>
-      <c r="C148" s="51"/>
-      <c r="D148" s="50"/>
-      <c r="E148" s="50"/>
-      <c r="F148" s="50"/>
-      <c r="G148" s="50"/>
-      <c r="H148" s="69"/>
-      <c r="I148" s="50"/>
+      <c r="A148" s="46"/>
+      <c r="B148" s="47"/>
+      <c r="C148" s="48"/>
+      <c r="D148" s="47"/>
+      <c r="E148" s="47"/>
+      <c r="F148" s="49"/>
+      <c r="G148" s="49"/>
+      <c r="H148" s="68"/>
+      <c r="I148" s="47"/>
     </row>
     <row r="149" spans="1:9">
-      <c r="A149" s="46"/>
-      <c r="B149" s="47"/>
-      <c r="C149" s="48"/>
-      <c r="D149" s="47"/>
-      <c r="E149" s="47"/>
-      <c r="F149" s="49"/>
-      <c r="G149" s="49"/>
-      <c r="H149" s="68"/>
-      <c r="I149" s="47"/>
+      <c r="A149" s="43"/>
+      <c r="B149" s="50"/>
+      <c r="C149" s="51"/>
+      <c r="D149" s="50"/>
+      <c r="E149" s="50"/>
+      <c r="F149" s="50"/>
+      <c r="G149" s="50"/>
+      <c r="H149" s="69"/>
+      <c r="I149" s="50"/>
     </row>
     <row r="150" spans="1:9">
-      <c r="A150" s="43"/>
-      <c r="B150" s="50"/>
-      <c r="C150" s="51"/>
-      <c r="D150" s="50"/>
-      <c r="E150" s="50"/>
-      <c r="F150" s="50"/>
-      <c r="G150" s="50"/>
-      <c r="H150" s="69"/>
-      <c r="I150" s="50"/>
+      <c r="A150" s="46"/>
+      <c r="B150" s="47"/>
+      <c r="C150" s="48"/>
+      <c r="D150" s="47"/>
+      <c r="E150" s="47"/>
+      <c r="F150" s="49"/>
+      <c r="G150" s="49"/>
+      <c r="H150" s="68"/>
+      <c r="I150" s="47"/>
     </row>
     <row r="151" spans="1:9">
-      <c r="A151" s="46"/>
-      <c r="B151" s="47"/>
-      <c r="C151" s="48"/>
-      <c r="D151" s="47"/>
-      <c r="E151" s="47"/>
-      <c r="F151" s="49"/>
-      <c r="G151" s="49"/>
-      <c r="H151" s="68"/>
-      <c r="I151" s="47"/>
+      <c r="A151" s="43"/>
+      <c r="B151" s="50"/>
+      <c r="C151" s="51"/>
+      <c r="D151" s="50"/>
+      <c r="E151" s="50"/>
+      <c r="F151" s="50"/>
+      <c r="G151" s="50"/>
+      <c r="H151" s="69"/>
+      <c r="I151" s="50"/>
     </row>
     <row r="152" spans="1:9">
-      <c r="A152" s="43"/>
-      <c r="B152" s="50"/>
-      <c r="C152" s="51"/>
-      <c r="D152" s="50"/>
-      <c r="E152" s="50"/>
-      <c r="F152" s="50"/>
-      <c r="G152" s="50"/>
-      <c r="H152" s="69"/>
-      <c r="I152" s="50"/>
+      <c r="A152" s="46"/>
+      <c r="B152" s="47"/>
+      <c r="C152" s="48"/>
+      <c r="D152" s="47"/>
+      <c r="E152" s="47"/>
+      <c r="F152" s="49"/>
+      <c r="G152" s="49"/>
+      <c r="H152" s="68"/>
+      <c r="I152" s="47"/>
     </row>
     <row r="153" spans="1:9">
-      <c r="A153" s="46"/>
-      <c r="B153" s="47"/>
-      <c r="C153" s="48"/>
-      <c r="D153" s="47"/>
-      <c r="E153" s="47"/>
-      <c r="F153" s="49"/>
-      <c r="G153" s="49"/>
-      <c r="H153" s="68"/>
-      <c r="I153" s="47"/>
+      <c r="A153" s="43"/>
+      <c r="B153" s="50"/>
+      <c r="C153" s="51"/>
+      <c r="D153" s="50"/>
+      <c r="E153" s="50"/>
+      <c r="F153" s="50"/>
+      <c r="G153" s="50"/>
+      <c r="H153" s="69"/>
+      <c r="I153" s="50"/>
     </row>
     <row r="154" spans="1:9">
-      <c r="A154" s="43"/>
-      <c r="B154" s="50"/>
-      <c r="C154" s="51"/>
-      <c r="D154" s="50"/>
-      <c r="E154" s="50"/>
-      <c r="F154" s="50"/>
-      <c r="G154" s="50"/>
-      <c r="H154" s="69"/>
-      <c r="I154" s="50"/>
+      <c r="A154" s="46"/>
+      <c r="B154" s="47"/>
+      <c r="C154" s="48"/>
+      <c r="D154" s="47"/>
+      <c r="E154" s="47"/>
+      <c r="F154" s="49"/>
+      <c r="G154" s="49"/>
+      <c r="H154" s="68"/>
+      <c r="I154" s="47"/>
     </row>
     <row r="155" spans="1:9">
-      <c r="A155" s="46"/>
-      <c r="B155" s="47"/>
-      <c r="C155" s="48"/>
-      <c r="D155" s="47"/>
-      <c r="E155" s="47"/>
-      <c r="F155" s="49"/>
-      <c r="G155" s="49"/>
-      <c r="H155" s="68"/>
-      <c r="I155" s="47"/>
+      <c r="A155" s="43"/>
+      <c r="B155" s="50"/>
+      <c r="C155" s="51"/>
+      <c r="D155" s="50"/>
+      <c r="E155" s="50"/>
+      <c r="F155" s="50"/>
+      <c r="G155" s="50"/>
+      <c r="H155" s="69"/>
+      <c r="I155" s="50"/>
     </row>
     <row r="156" spans="1:9">
-      <c r="A156" s="43"/>
-      <c r="B156" s="50"/>
-      <c r="C156" s="51"/>
-      <c r="D156" s="50"/>
-      <c r="E156" s="50"/>
-      <c r="F156" s="50"/>
-      <c r="G156" s="50"/>
-      <c r="H156" s="69"/>
-      <c r="I156" s="50"/>
+      <c r="A156" s="46"/>
+      <c r="B156" s="47"/>
+      <c r="C156" s="48"/>
+      <c r="D156" s="47"/>
+      <c r="E156" s="47"/>
+      <c r="F156" s="49"/>
+      <c r="G156" s="49"/>
+      <c r="H156" s="68"/>
+      <c r="I156" s="47"/>
     </row>
     <row r="157" spans="1:9">
-      <c r="A157" s="46"/>
-      <c r="B157" s="47"/>
-      <c r="C157" s="48"/>
-      <c r="D157" s="47"/>
-      <c r="E157" s="47"/>
-      <c r="F157" s="49"/>
-      <c r="G157" s="49"/>
-      <c r="H157" s="68"/>
-      <c r="I157" s="47"/>
+      <c r="A157" s="43"/>
+      <c r="B157" s="50"/>
+      <c r="C157" s="51"/>
+      <c r="D157" s="50"/>
+      <c r="E157" s="50"/>
+      <c r="F157" s="50"/>
+      <c r="G157" s="50"/>
+      <c r="H157" s="69"/>
+      <c r="I157" s="50"/>
     </row>
     <row r="158" spans="1:9">
-      <c r="A158" s="43"/>
-      <c r="B158" s="50"/>
-      <c r="C158" s="51"/>
-      <c r="D158" s="50"/>
-      <c r="E158" s="50"/>
-      <c r="F158" s="50"/>
-      <c r="G158" s="50"/>
-      <c r="H158" s="69"/>
-      <c r="I158" s="50"/>
+      <c r="A158" s="46"/>
+      <c r="B158" s="47"/>
+      <c r="C158" s="48"/>
+      <c r="D158" s="47"/>
+      <c r="E158" s="47"/>
+      <c r="F158" s="49"/>
+      <c r="G158" s="49"/>
+      <c r="H158" s="68"/>
+      <c r="I158" s="47"/>
     </row>
     <row r="159" spans="1:9">
-      <c r="A159" s="46"/>
-      <c r="B159" s="47"/>
-      <c r="C159" s="48"/>
-      <c r="D159" s="47"/>
-      <c r="E159" s="47"/>
-      <c r="F159" s="49"/>
-      <c r="G159" s="49"/>
-      <c r="H159" s="68"/>
-      <c r="I159" s="47"/>
+      <c r="A159" s="43"/>
+      <c r="B159" s="50"/>
+      <c r="C159" s="51"/>
+      <c r="D159" s="50"/>
+      <c r="E159" s="50"/>
+      <c r="F159" s="50"/>
+      <c r="G159" s="50"/>
+      <c r="H159" s="69"/>
+      <c r="I159" s="50"/>
     </row>
     <row r="160" spans="1:9">
-      <c r="A160" s="43"/>
-      <c r="B160" s="50"/>
-      <c r="C160" s="51"/>
-      <c r="D160" s="50"/>
-      <c r="E160" s="50"/>
-      <c r="F160" s="50"/>
-      <c r="G160" s="50"/>
-      <c r="H160" s="69"/>
-      <c r="I160" s="50"/>
+      <c r="A160" s="46"/>
+      <c r="B160" s="47"/>
+      <c r="C160" s="48"/>
+      <c r="D160" s="47"/>
+      <c r="E160" s="47"/>
+      <c r="F160" s="49"/>
+      <c r="G160" s="49"/>
+      <c r="H160" s="68"/>
+      <c r="I160" s="47"/>
     </row>
     <row r="161" spans="1:9">
-      <c r="A161" s="46"/>
-      <c r="B161" s="47"/>
-      <c r="C161" s="48"/>
-      <c r="D161" s="47"/>
-      <c r="E161" s="47"/>
-      <c r="F161" s="49"/>
-      <c r="G161" s="49"/>
-      <c r="H161" s="68"/>
-      <c r="I161" s="47"/>
+      <c r="A161" s="43"/>
+      <c r="B161" s="50"/>
+      <c r="C161" s="51"/>
+      <c r="D161" s="50"/>
+      <c r="E161" s="50"/>
+      <c r="F161" s="50"/>
+      <c r="G161" s="50"/>
+      <c r="H161" s="69"/>
+      <c r="I161" s="50"/>
     </row>
     <row r="162" spans="1:9">
-      <c r="A162" s="43"/>
-      <c r="B162" s="50"/>
-      <c r="C162" s="51"/>
-      <c r="D162" s="50"/>
-      <c r="E162" s="50"/>
-      <c r="F162" s="50"/>
-      <c r="G162" s="50"/>
-      <c r="H162" s="69"/>
-      <c r="I162" s="50"/>
+      <c r="A162" s="46"/>
+      <c r="B162" s="47"/>
+      <c r="C162" s="48"/>
+      <c r="D162" s="47"/>
+      <c r="E162" s="47"/>
+      <c r="F162" s="49"/>
+      <c r="G162" s="49"/>
+      <c r="H162" s="68"/>
+      <c r="I162" s="47"/>
     </row>
     <row r="163" spans="1:9">
-      <c r="A163" s="46"/>
-      <c r="B163" s="47"/>
-      <c r="C163" s="48"/>
-      <c r="D163" s="47"/>
-      <c r="E163" s="47"/>
-      <c r="F163" s="49"/>
-      <c r="G163" s="49"/>
-      <c r="H163" s="68"/>
-      <c r="I163" s="47"/>
+      <c r="A163" s="43"/>
+      <c r="B163" s="50"/>
+      <c r="C163" s="51"/>
+      <c r="D163" s="50"/>
+      <c r="E163" s="50"/>
+      <c r="F163" s="50"/>
+      <c r="G163" s="50"/>
+      <c r="H163" s="69"/>
+      <c r="I163" s="50"/>
     </row>
     <row r="164" spans="1:9">
-      <c r="A164" s="43"/>
-      <c r="B164" s="50"/>
-      <c r="C164" s="51"/>
-      <c r="D164" s="50"/>
-      <c r="E164" s="50"/>
-      <c r="F164" s="50"/>
-      <c r="G164" s="50"/>
-      <c r="H164" s="69"/>
-      <c r="I164" s="50"/>
+      <c r="A164" s="46"/>
+      <c r="B164" s="47"/>
+      <c r="C164" s="48"/>
+      <c r="D164" s="47"/>
+      <c r="E164" s="47"/>
+      <c r="F164" s="49"/>
+      <c r="G164" s="49"/>
+      <c r="H164" s="68"/>
+      <c r="I164" s="47"/>
     </row>
     <row r="165" spans="1:9">
-      <c r="A165" s="46"/>
-      <c r="B165" s="47"/>
-      <c r="C165" s="48"/>
-      <c r="D165" s="47"/>
-      <c r="E165" s="47"/>
-      <c r="F165" s="49"/>
-      <c r="G165" s="49"/>
-      <c r="H165" s="68"/>
-      <c r="I165" s="47"/>
+      <c r="A165" s="43"/>
+      <c r="B165" s="50"/>
+      <c r="C165" s="51"/>
+      <c r="D165" s="50"/>
+      <c r="E165" s="50"/>
+      <c r="F165" s="50"/>
+      <c r="G165" s="50"/>
+      <c r="H165" s="69"/>
+      <c r="I165" s="50"/>
     </row>
     <row r="166" spans="1:9">
-      <c r="A166" s="43"/>
-      <c r="B166" s="50"/>
-      <c r="C166" s="51"/>
-      <c r="D166" s="50"/>
-      <c r="E166" s="50"/>
-      <c r="F166" s="50"/>
-      <c r="G166" s="50"/>
-      <c r="H166" s="69"/>
-      <c r="I166" s="50"/>
+      <c r="A166" s="46"/>
+      <c r="B166" s="47"/>
+      <c r="C166" s="48"/>
+      <c r="D166" s="47"/>
+      <c r="E166" s="47"/>
+      <c r="F166" s="49"/>
+      <c r="G166" s="49"/>
+      <c r="H166" s="68"/>
+      <c r="I166" s="47"/>
     </row>
     <row r="167" spans="1:9">
-      <c r="A167" s="46"/>
-      <c r="B167" s="47"/>
-      <c r="C167" s="48"/>
-      <c r="D167" s="47"/>
-      <c r="E167" s="47"/>
-      <c r="F167" s="49"/>
-      <c r="G167" s="49"/>
-      <c r="H167" s="68"/>
-      <c r="I167" s="47"/>
+      <c r="A167" s="43"/>
+      <c r="B167" s="50"/>
+      <c r="C167" s="51"/>
+      <c r="D167" s="50"/>
+      <c r="E167" s="50"/>
+      <c r="F167" s="50"/>
+      <c r="G167" s="50"/>
+      <c r="H167" s="69"/>
+      <c r="I167" s="50"/>
     </row>
     <row r="168" spans="1:9">
-      <c r="A168" s="43"/>
-      <c r="B168" s="50"/>
-      <c r="C168" s="51"/>
-      <c r="D168" s="50"/>
-      <c r="E168" s="50"/>
-      <c r="F168" s="50"/>
-      <c r="G168" s="50"/>
-      <c r="H168" s="69"/>
-      <c r="I168" s="50"/>
+      <c r="A168" s="46"/>
+      <c r="B168" s="47"/>
+      <c r="C168" s="48"/>
+      <c r="D168" s="47"/>
+      <c r="E168" s="47"/>
+      <c r="F168" s="49"/>
+      <c r="G168" s="49"/>
+      <c r="H168" s="68"/>
+      <c r="I168" s="47"/>
     </row>
     <row r="169" spans="1:9">
-      <c r="A169" s="46"/>
-      <c r="B169" s="47"/>
-      <c r="C169" s="48"/>
-      <c r="D169" s="47"/>
-      <c r="E169" s="47"/>
-      <c r="F169" s="49"/>
-      <c r="G169" s="49"/>
-      <c r="H169" s="68"/>
-      <c r="I169" s="47"/>
+      <c r="A169" s="43"/>
+      <c r="B169" s="50"/>
+      <c r="C169" s="51"/>
+      <c r="D169" s="50"/>
+      <c r="E169" s="50"/>
+      <c r="F169" s="50"/>
+      <c r="G169" s="50"/>
+      <c r="H169" s="69"/>
+      <c r="I169" s="50"/>
     </row>
     <row r="170" spans="1:9">
-      <c r="A170" s="43"/>
-      <c r="B170" s="50"/>
-      <c r="C170" s="51"/>
-      <c r="D170" s="50"/>
-      <c r="E170" s="50"/>
-      <c r="F170" s="50"/>
-      <c r="G170" s="50"/>
-      <c r="H170" s="69"/>
-      <c r="I170" s="50"/>
+      <c r="A170" s="46"/>
+      <c r="B170" s="47"/>
+      <c r="C170" s="48"/>
+      <c r="D170" s="47"/>
+      <c r="E170" s="47"/>
+      <c r="F170" s="49"/>
+      <c r="G170" s="49"/>
+      <c r="H170" s="68"/>
+      <c r="I170" s="47"/>
     </row>
     <row r="171" spans="1:9">
-      <c r="A171" s="46"/>
-      <c r="B171" s="47"/>
-      <c r="C171" s="48"/>
-      <c r="D171" s="47"/>
-      <c r="E171" s="47"/>
-      <c r="F171" s="49"/>
-      <c r="G171" s="49"/>
-      <c r="H171" s="68"/>
-      <c r="I171" s="47"/>
+      <c r="A171" s="43"/>
+      <c r="B171" s="50"/>
+      <c r="C171" s="51"/>
+      <c r="D171" s="50"/>
+      <c r="E171" s="50"/>
+      <c r="F171" s="50"/>
+      <c r="G171" s="50"/>
+      <c r="H171" s="69"/>
+      <c r="I171" s="50"/>
     </row>
     <row r="172" spans="1:9">
-      <c r="A172" s="43"/>
-      <c r="B172" s="50"/>
-      <c r="C172" s="51"/>
-      <c r="D172" s="50"/>
-      <c r="E172" s="50"/>
-      <c r="F172" s="50"/>
-      <c r="G172" s="50"/>
-      <c r="H172" s="69"/>
-      <c r="I172" s="50"/>
+      <c r="A172" s="46"/>
+      <c r="B172" s="47"/>
+      <c r="C172" s="48"/>
+      <c r="D172" s="47"/>
+      <c r="E172" s="47"/>
+      <c r="F172" s="49"/>
+      <c r="G172" s="49"/>
+      <c r="H172" s="68"/>
+      <c r="I172" s="47"/>
     </row>
     <row r="173" spans="1:9">
-      <c r="A173" s="46"/>
-      <c r="B173" s="47"/>
-      <c r="C173" s="48"/>
-      <c r="D173" s="47"/>
-      <c r="E173" s="47"/>
-      <c r="F173" s="49"/>
-      <c r="G173" s="49"/>
-      <c r="H173" s="68"/>
-      <c r="I173" s="47"/>
+      <c r="A173" s="43"/>
+      <c r="B173" s="50"/>
+      <c r="C173" s="51"/>
+      <c r="D173" s="50"/>
+      <c r="E173" s="50"/>
+      <c r="F173" s="50"/>
+      <c r="G173" s="50"/>
+      <c r="H173" s="69"/>
+      <c r="I173" s="50"/>
     </row>
     <row r="174" spans="1:9">
-      <c r="A174" s="43"/>
-      <c r="B174" s="50"/>
-      <c r="C174" s="51"/>
-      <c r="D174" s="50"/>
-      <c r="E174" s="50"/>
-      <c r="F174" s="50"/>
-      <c r="G174" s="50"/>
-      <c r="H174" s="69"/>
-      <c r="I174" s="50"/>
+      <c r="A174" s="46"/>
+      <c r="B174" s="47"/>
+      <c r="C174" s="48"/>
+      <c r="D174" s="47"/>
+      <c r="E174" s="47"/>
+      <c r="F174" s="49"/>
+      <c r="G174" s="49"/>
+      <c r="H174" s="68"/>
+      <c r="I174" s="47"/>
     </row>
     <row r="175" spans="1:9">
-      <c r="A175" s="46"/>
-      <c r="B175" s="47"/>
-      <c r="C175" s="48"/>
-      <c r="D175" s="47"/>
-      <c r="E175" s="47"/>
-      <c r="F175" s="49"/>
-      <c r="G175" s="49"/>
-      <c r="H175" s="68"/>
-      <c r="I175" s="47"/>
+      <c r="A175" s="43"/>
+      <c r="B175" s="50"/>
+      <c r="C175" s="51"/>
+      <c r="D175" s="50"/>
+      <c r="E175" s="50"/>
+      <c r="F175" s="50"/>
+      <c r="G175" s="50"/>
+      <c r="H175" s="69"/>
+      <c r="I175" s="50"/>
     </row>
     <row r="176" spans="1:9">
-      <c r="A176" s="43"/>
-      <c r="B176" s="50"/>
-      <c r="C176" s="51"/>
-      <c r="D176" s="50"/>
-      <c r="E176" s="50"/>
-      <c r="F176" s="50"/>
-      <c r="G176" s="50"/>
-      <c r="H176" s="69"/>
-      <c r="I176" s="50"/>
+      <c r="A176" s="46"/>
+      <c r="B176" s="47"/>
+      <c r="C176" s="48"/>
+      <c r="D176" s="47"/>
+      <c r="E176" s="47"/>
+      <c r="F176" s="49"/>
+      <c r="G176" s="49"/>
+      <c r="H176" s="68"/>
+      <c r="I176" s="47"/>
     </row>
     <row r="177" spans="1:9">
-      <c r="A177" s="46"/>
-      <c r="B177" s="47"/>
-      <c r="C177" s="48"/>
-      <c r="D177" s="47"/>
-      <c r="E177" s="47"/>
-      <c r="F177" s="49"/>
-      <c r="G177" s="49"/>
-      <c r="H177" s="68"/>
-      <c r="I177" s="47"/>
+      <c r="A177" s="43"/>
+      <c r="B177" s="50"/>
+      <c r="C177" s="51"/>
+      <c r="D177" s="50"/>
+      <c r="E177" s="50"/>
+      <c r="F177" s="50"/>
+      <c r="G177" s="50"/>
+      <c r="H177" s="69"/>
+      <c r="I177" s="50"/>
     </row>
     <row r="178" spans="1:9">
-      <c r="A178" s="43"/>
-      <c r="B178" s="50"/>
-      <c r="C178" s="51"/>
-      <c r="D178" s="50"/>
-      <c r="E178" s="50"/>
-      <c r="F178" s="50"/>
-      <c r="G178" s="50"/>
-      <c r="H178" s="69"/>
-      <c r="I178" s="50"/>
+      <c r="A178" s="46"/>
+      <c r="B178" s="47"/>
+      <c r="C178" s="48"/>
+      <c r="D178" s="47"/>
+      <c r="E178" s="47"/>
+      <c r="F178" s="49"/>
+      <c r="G178" s="49"/>
+      <c r="H178" s="68"/>
+      <c r="I178" s="47"/>
     </row>
     <row r="179" spans="1:9">
-      <c r="A179" s="46"/>
-      <c r="B179" s="47"/>
-      <c r="C179" s="48"/>
-      <c r="D179" s="47"/>
-      <c r="E179" s="47"/>
-      <c r="F179" s="49"/>
-      <c r="G179" s="49"/>
-      <c r="H179" s="68"/>
-      <c r="I179" s="47"/>
+      <c r="A179" s="43"/>
+      <c r="B179" s="50"/>
+      <c r="C179" s="51"/>
+      <c r="D179" s="50"/>
+      <c r="E179" s="50"/>
+      <c r="F179" s="50"/>
+      <c r="G179" s="50"/>
+      <c r="H179" s="69"/>
+      <c r="I179" s="50"/>
     </row>
     <row r="180" spans="1:9">
-      <c r="A180" s="43"/>
-      <c r="B180" s="50"/>
-      <c r="C180" s="51"/>
-      <c r="D180" s="50"/>
-      <c r="E180" s="50"/>
-      <c r="F180" s="50"/>
-      <c r="G180" s="50"/>
-      <c r="H180" s="69"/>
-      <c r="I180" s="50"/>
+      <c r="A180" s="46"/>
+      <c r="B180" s="47"/>
+      <c r="C180" s="48"/>
+      <c r="D180" s="47"/>
+      <c r="E180" s="47"/>
+      <c r="F180" s="49"/>
+      <c r="G180" s="49"/>
+      <c r="H180" s="68"/>
+      <c r="I180" s="47"/>
     </row>
     <row r="181" spans="1:9">
-      <c r="A181" s="46"/>
-      <c r="B181" s="47"/>
-      <c r="C181" s="48"/>
-      <c r="D181" s="47"/>
-      <c r="E181" s="47"/>
-      <c r="F181" s="49"/>
-      <c r="G181" s="49"/>
-      <c r="H181" s="68"/>
-      <c r="I181" s="47"/>
+      <c r="A181" s="43"/>
+      <c r="B181" s="50"/>
+      <c r="C181" s="51"/>
+      <c r="D181" s="50"/>
+      <c r="E181" s="50"/>
+      <c r="F181" s="50"/>
+      <c r="G181" s="50"/>
+      <c r="H181" s="69"/>
+      <c r="I181" s="50"/>
     </row>
     <row r="182" spans="1:9">
-      <c r="A182" s="43"/>
-      <c r="B182" s="50"/>
-      <c r="C182" s="51"/>
-      <c r="D182" s="50"/>
-      <c r="E182" s="50"/>
-      <c r="F182" s="50"/>
-      <c r="G182" s="50"/>
-      <c r="H182" s="69"/>
-      <c r="I182" s="50"/>
+      <c r="A182" s="46"/>
+      <c r="B182" s="47"/>
+      <c r="C182" s="48"/>
+      <c r="D182" s="47"/>
+      <c r="E182" s="47"/>
+      <c r="F182" s="49"/>
+      <c r="G182" s="49"/>
+      <c r="H182" s="68"/>
+      <c r="I182" s="47"/>
     </row>
     <row r="183" spans="1:9">
-      <c r="A183" s="46"/>
-      <c r="B183" s="47"/>
-      <c r="C183" s="48"/>
-      <c r="D183" s="47"/>
-      <c r="E183" s="47"/>
-      <c r="F183" s="49"/>
-      <c r="G183" s="49"/>
-      <c r="H183" s="68"/>
-      <c r="I183" s="47"/>
+      <c r="A183" s="43"/>
+      <c r="B183" s="50"/>
+      <c r="C183" s="51"/>
+      <c r="D183" s="50"/>
+      <c r="E183" s="50"/>
+      <c r="F183" s="50"/>
+      <c r="G183" s="50"/>
+      <c r="H183" s="69"/>
+      <c r="I183" s="50"/>
     </row>
     <row r="184" spans="1:9">
-      <c r="A184" s="43"/>
-      <c r="B184" s="50"/>
-      <c r="C184" s="51"/>
-      <c r="D184" s="50"/>
-      <c r="E184" s="50"/>
-      <c r="F184" s="50"/>
-      <c r="G184" s="50"/>
-      <c r="H184" s="69"/>
-      <c r="I184" s="50"/>
+      <c r="A184" s="46"/>
+      <c r="B184" s="47"/>
+      <c r="C184" s="48"/>
+      <c r="D184" s="47"/>
+      <c r="E184" s="47"/>
+      <c r="F184" s="49"/>
+      <c r="G184" s="49"/>
+      <c r="H184" s="68"/>
+      <c r="I184" s="47"/>
     </row>
     <row r="185" spans="1:9">
-      <c r="A185" s="46"/>
-      <c r="B185" s="47"/>
-      <c r="C185" s="48"/>
-      <c r="D185" s="47"/>
-      <c r="E185" s="47"/>
-      <c r="F185" s="49"/>
-      <c r="G185" s="49"/>
-      <c r="H185" s="68"/>
-      <c r="I185" s="47"/>
+      <c r="A185" s="43"/>
+      <c r="B185" s="50"/>
+      <c r="C185" s="51"/>
+      <c r="D185" s="50"/>
+      <c r="E185" s="50"/>
+      <c r="F185" s="50"/>
+      <c r="G185" s="50"/>
+      <c r="H185" s="69"/>
+      <c r="I185" s="50"/>
     </row>
     <row r="186" spans="1:9">
-      <c r="A186" s="43"/>
-      <c r="B186" s="50"/>
-      <c r="C186" s="51"/>
-      <c r="D186" s="50"/>
-      <c r="E186" s="50"/>
-      <c r="F186" s="50"/>
-      <c r="G186" s="50"/>
-      <c r="H186" s="69"/>
-      <c r="I186" s="50"/>
+      <c r="A186" s="46"/>
+      <c r="B186" s="47"/>
+      <c r="C186" s="48"/>
+      <c r="D186" s="47"/>
+      <c r="E186" s="47"/>
+      <c r="F186" s="49"/>
+      <c r="G186" s="49"/>
+      <c r="H186" s="68"/>
+      <c r="I186" s="47"/>
     </row>
     <row r="187" spans="1:9">
       <c r="A187" s="46"/>
@@ -15930,831 +15930,820 @@
       <c r="I187" s="47"/>
     </row>
     <row r="188" spans="1:9">
-      <c r="A188" s="46"/>
-      <c r="B188" s="47"/>
-      <c r="C188" s="48"/>
-      <c r="D188" s="47"/>
-      <c r="E188" s="47"/>
-      <c r="F188" s="49"/>
-      <c r="G188" s="49"/>
-      <c r="H188" s="68"/>
-      <c r="I188" s="47"/>
+      <c r="A188" s="43"/>
+      <c r="B188" s="50"/>
+      <c r="C188" s="51"/>
+      <c r="D188" s="50"/>
+      <c r="E188" s="50"/>
+      <c r="F188" s="50"/>
+      <c r="G188" s="50"/>
+      <c r="H188" s="69"/>
+      <c r="I188" s="50"/>
     </row>
     <row r="189" spans="1:9">
-      <c r="A189" s="43"/>
-      <c r="B189" s="50"/>
-      <c r="C189" s="51"/>
-      <c r="D189" s="50"/>
-      <c r="E189" s="50"/>
-      <c r="F189" s="50"/>
-      <c r="G189" s="50"/>
-      <c r="H189" s="69"/>
-      <c r="I189" s="50"/>
+      <c r="A189" s="46"/>
+      <c r="B189" s="47"/>
+      <c r="C189" s="48"/>
+      <c r="D189" s="47"/>
+      <c r="E189" s="47"/>
+      <c r="F189" s="49"/>
+      <c r="G189" s="49"/>
+      <c r="H189" s="68"/>
+      <c r="I189" s="47"/>
     </row>
     <row r="190" spans="1:9">
-      <c r="A190" s="46"/>
-      <c r="B190" s="47"/>
-      <c r="C190" s="48"/>
-      <c r="D190" s="47"/>
-      <c r="E190" s="47"/>
-      <c r="F190" s="49"/>
-      <c r="G190" s="49"/>
-      <c r="H190" s="68"/>
-      <c r="I190" s="47"/>
+      <c r="A190" s="43"/>
+      <c r="B190" s="50"/>
+      <c r="C190" s="51"/>
+      <c r="D190" s="50"/>
+      <c r="E190" s="50"/>
+      <c r="F190" s="50"/>
+      <c r="G190" s="50"/>
+      <c r="H190" s="69"/>
+      <c r="I190" s="50"/>
     </row>
     <row r="191" spans="1:9">
-      <c r="A191" s="43"/>
-      <c r="B191" s="50"/>
-      <c r="C191" s="51"/>
-      <c r="D191" s="50"/>
-      <c r="E191" s="50"/>
-      <c r="F191" s="50"/>
-      <c r="G191" s="50"/>
-      <c r="H191" s="69"/>
-      <c r="I191" s="50"/>
+      <c r="A191" s="46"/>
+      <c r="B191" s="47"/>
+      <c r="C191" s="48"/>
+      <c r="D191" s="47"/>
+      <c r="E191" s="47"/>
+      <c r="F191" s="49"/>
+      <c r="G191" s="49"/>
+      <c r="H191" s="68"/>
+      <c r="I191" s="47"/>
     </row>
     <row r="192" spans="1:9">
-      <c r="A192" s="46"/>
-      <c r="B192" s="47"/>
-      <c r="C192" s="48"/>
-      <c r="D192" s="47"/>
-      <c r="E192" s="47"/>
-      <c r="F192" s="49"/>
-      <c r="G192" s="49"/>
-      <c r="H192" s="68"/>
-      <c r="I192" s="47"/>
+      <c r="A192" s="43"/>
+      <c r="B192" s="50"/>
+      <c r="C192" s="51"/>
+      <c r="D192" s="50"/>
+      <c r="E192" s="50"/>
+      <c r="F192" s="50"/>
+      <c r="G192" s="50"/>
+      <c r="H192" s="69"/>
+      <c r="I192" s="50"/>
     </row>
     <row r="193" spans="1:9">
-      <c r="A193" s="43"/>
-      <c r="B193" s="50"/>
-      <c r="C193" s="51"/>
-      <c r="D193" s="50"/>
-      <c r="E193" s="50"/>
-      <c r="F193" s="50"/>
-      <c r="G193" s="50"/>
-      <c r="H193" s="69"/>
-      <c r="I193" s="50"/>
+      <c r="A193" s="46"/>
+      <c r="B193" s="47"/>
+      <c r="C193" s="48"/>
+      <c r="D193" s="47"/>
+      <c r="E193" s="47"/>
+      <c r="F193" s="49"/>
+      <c r="G193" s="49"/>
+      <c r="H193" s="68"/>
+      <c r="I193" s="47"/>
     </row>
     <row r="194" spans="1:9">
-      <c r="A194" s="46"/>
-      <c r="B194" s="47"/>
-      <c r="C194" s="48"/>
-      <c r="D194" s="47"/>
-      <c r="E194" s="47"/>
-      <c r="F194" s="49"/>
-      <c r="G194" s="49"/>
-      <c r="H194" s="68"/>
-      <c r="I194" s="47"/>
+      <c r="A194" s="43"/>
+      <c r="B194" s="50"/>
+      <c r="C194" s="51"/>
+      <c r="D194" s="50"/>
+      <c r="E194" s="50"/>
+      <c r="F194" s="50"/>
+      <c r="G194" s="50"/>
+      <c r="H194" s="69"/>
+      <c r="I194" s="50"/>
     </row>
     <row r="195" spans="1:9">
-      <c r="A195" s="43"/>
-      <c r="B195" s="50"/>
-      <c r="C195" s="51"/>
-      <c r="D195" s="50"/>
-      <c r="E195" s="50"/>
-      <c r="F195" s="50"/>
-      <c r="G195" s="50"/>
-      <c r="H195" s="69"/>
-      <c r="I195" s="50"/>
+      <c r="A195" s="46"/>
+      <c r="B195" s="47"/>
+      <c r="C195" s="48"/>
+      <c r="D195" s="47"/>
+      <c r="E195" s="47"/>
+      <c r="F195" s="49"/>
+      <c r="G195" s="49"/>
+      <c r="H195" s="68"/>
+      <c r="I195" s="47"/>
     </row>
     <row r="196" spans="1:9">
-      <c r="A196" s="46"/>
-      <c r="B196" s="47"/>
-      <c r="C196" s="48"/>
-      <c r="D196" s="47"/>
-      <c r="E196" s="47"/>
-      <c r="F196" s="49"/>
-      <c r="G196" s="49"/>
-      <c r="H196" s="68"/>
-      <c r="I196" s="47"/>
+      <c r="A196" s="43"/>
+      <c r="B196" s="50"/>
+      <c r="C196" s="51"/>
+      <c r="D196" s="50"/>
+      <c r="E196" s="50"/>
+      <c r="F196" s="50"/>
+      <c r="G196" s="50"/>
+      <c r="H196" s="69"/>
+      <c r="I196" s="50"/>
     </row>
     <row r="197" spans="1:9">
-      <c r="A197" s="43"/>
-      <c r="B197" s="50"/>
-      <c r="C197" s="51"/>
-      <c r="D197" s="50"/>
-      <c r="E197" s="50"/>
-      <c r="F197" s="50"/>
-      <c r="G197" s="50"/>
-      <c r="H197" s="69"/>
-      <c r="I197" s="50"/>
+      <c r="A197" s="46"/>
+      <c r="B197" s="47"/>
+      <c r="C197" s="48"/>
+      <c r="D197" s="47"/>
+      <c r="E197" s="47"/>
+      <c r="F197" s="49"/>
+      <c r="G197" s="49"/>
+      <c r="H197" s="68"/>
+      <c r="I197" s="47"/>
     </row>
     <row r="198" spans="1:9">
-      <c r="A198" s="46"/>
-      <c r="B198" s="47"/>
-      <c r="C198" s="48"/>
-      <c r="D198" s="47"/>
-      <c r="E198" s="47"/>
-      <c r="F198" s="49"/>
-      <c r="G198" s="49"/>
-      <c r="H198" s="68"/>
-      <c r="I198" s="47"/>
+      <c r="A198" s="43"/>
+      <c r="B198" s="50"/>
+      <c r="C198" s="51"/>
+      <c r="D198" s="50"/>
+      <c r="E198" s="50"/>
+      <c r="F198" s="50"/>
+      <c r="G198" s="50"/>
+      <c r="H198" s="69"/>
+      <c r="I198" s="50"/>
     </row>
     <row r="199" spans="1:9">
-      <c r="A199" s="43"/>
-      <c r="B199" s="50"/>
-      <c r="C199" s="51"/>
-      <c r="D199" s="50"/>
-      <c r="E199" s="50"/>
-      <c r="F199" s="50"/>
-      <c r="G199" s="50"/>
-      <c r="H199" s="69"/>
-      <c r="I199" s="50"/>
+      <c r="A199" s="46"/>
+      <c r="B199" s="47"/>
+      <c r="C199" s="48"/>
+      <c r="D199" s="47"/>
+      <c r="E199" s="47"/>
+      <c r="F199" s="49"/>
+      <c r="G199" s="49"/>
+      <c r="H199" s="68"/>
+      <c r="I199" s="47"/>
     </row>
     <row r="200" spans="1:9">
-      <c r="A200" s="46"/>
-      <c r="B200" s="47"/>
-      <c r="C200" s="48"/>
-      <c r="D200" s="47"/>
-      <c r="E200" s="47"/>
-      <c r="F200" s="49"/>
-      <c r="G200" s="49"/>
-      <c r="H200" s="68"/>
-      <c r="I200" s="47"/>
+      <c r="A200" s="43"/>
+      <c r="B200" s="50"/>
+      <c r="C200" s="51"/>
+      <c r="D200" s="50"/>
+      <c r="E200" s="50"/>
+      <c r="F200" s="50"/>
+      <c r="G200" s="50"/>
+      <c r="H200" s="69"/>
+      <c r="I200" s="50"/>
     </row>
     <row r="201" spans="1:9">
-      <c r="A201" s="43"/>
-      <c r="B201" s="50"/>
-      <c r="C201" s="51"/>
-      <c r="D201" s="50"/>
-      <c r="E201" s="50"/>
-      <c r="F201" s="50"/>
-      <c r="G201" s="50"/>
-      <c r="H201" s="69"/>
-      <c r="I201" s="50"/>
+      <c r="A201" s="46"/>
+      <c r="B201" s="47"/>
+      <c r="C201" s="48"/>
+      <c r="D201" s="47"/>
+      <c r="E201" s="47"/>
+      <c r="F201" s="49"/>
+      <c r="G201" s="49"/>
+      <c r="H201" s="68"/>
+      <c r="I201" s="47"/>
     </row>
     <row r="202" spans="1:9">
-      <c r="A202" s="46"/>
-      <c r="B202" s="47"/>
-      <c r="C202" s="48"/>
-      <c r="D202" s="47"/>
-      <c r="E202" s="47"/>
-      <c r="F202" s="49"/>
-      <c r="G202" s="49"/>
-      <c r="H202" s="68"/>
-      <c r="I202" s="47"/>
+      <c r="A202" s="43"/>
+      <c r="B202" s="50"/>
+      <c r="C202" s="51"/>
+      <c r="D202" s="50"/>
+      <c r="E202" s="50"/>
+      <c r="F202" s="50"/>
+      <c r="G202" s="50"/>
+      <c r="H202" s="69"/>
+      <c r="I202" s="50"/>
     </row>
     <row r="203" spans="1:9">
-      <c r="A203" s="43"/>
-      <c r="B203" s="50"/>
-      <c r="C203" s="51"/>
-      <c r="D203" s="50"/>
-      <c r="E203" s="50"/>
-      <c r="F203" s="50"/>
-      <c r="G203" s="50"/>
-      <c r="H203" s="69"/>
-      <c r="I203" s="50"/>
+      <c r="A203" s="46"/>
+      <c r="B203" s="47"/>
+      <c r="C203" s="48"/>
+      <c r="D203" s="47"/>
+      <c r="E203" s="47"/>
+      <c r="F203" s="49"/>
+      <c r="G203" s="49"/>
+      <c r="H203" s="68"/>
+      <c r="I203" s="47"/>
     </row>
     <row r="204" spans="1:9">
-      <c r="A204" s="46"/>
-      <c r="B204" s="47"/>
-      <c r="C204" s="48"/>
-      <c r="D204" s="47"/>
-      <c r="E204" s="47"/>
-      <c r="F204" s="49"/>
-      <c r="G204" s="49"/>
-      <c r="H204" s="68"/>
-      <c r="I204" s="47"/>
+      <c r="A204" s="43"/>
+      <c r="B204" s="50"/>
+      <c r="C204" s="51"/>
+      <c r="D204" s="50"/>
+      <c r="E204" s="50"/>
+      <c r="F204" s="50"/>
+      <c r="G204" s="50"/>
+      <c r="H204" s="69"/>
+      <c r="I204" s="50"/>
     </row>
     <row r="205" spans="1:9">
-      <c r="A205" s="43"/>
-      <c r="B205" s="50"/>
-      <c r="C205" s="51"/>
-      <c r="D205" s="50"/>
-      <c r="E205" s="50"/>
-      <c r="F205" s="50"/>
-      <c r="G205" s="50"/>
-      <c r="H205" s="69"/>
-      <c r="I205" s="50"/>
+      <c r="A205" s="46"/>
+      <c r="B205" s="47"/>
+      <c r="C205" s="48"/>
+      <c r="D205" s="47"/>
+      <c r="E205" s="47"/>
+      <c r="F205" s="49"/>
+      <c r="G205" s="49"/>
+      <c r="H205" s="68"/>
+      <c r="I205" s="47"/>
     </row>
     <row r="206" spans="1:9">
-      <c r="A206" s="46"/>
-      <c r="B206" s="47"/>
-      <c r="C206" s="48"/>
-      <c r="D206" s="47"/>
-      <c r="E206" s="47"/>
-      <c r="F206" s="49"/>
-      <c r="G206" s="49"/>
-      <c r="H206" s="68"/>
-      <c r="I206" s="47"/>
+      <c r="A206" s="43"/>
+      <c r="B206" s="50"/>
+      <c r="C206" s="51"/>
+      <c r="D206" s="50"/>
+      <c r="E206" s="50"/>
+      <c r="F206" s="50"/>
+      <c r="G206" s="50"/>
+      <c r="H206" s="69"/>
+      <c r="I206" s="50"/>
     </row>
     <row r="207" spans="1:9">
-      <c r="A207" s="43"/>
-      <c r="B207" s="50"/>
-      <c r="C207" s="51"/>
-      <c r="D207" s="50"/>
-      <c r="E207" s="50"/>
-      <c r="F207" s="50"/>
-      <c r="G207" s="50"/>
-      <c r="H207" s="69"/>
-      <c r="I207" s="50"/>
+      <c r="A207" s="46"/>
+      <c r="B207" s="47"/>
+      <c r="C207" s="48"/>
+      <c r="D207" s="47"/>
+      <c r="E207" s="47"/>
+      <c r="F207" s="49"/>
+      <c r="G207" s="49"/>
+      <c r="H207" s="68"/>
+      <c r="I207" s="47"/>
     </row>
     <row r="208" spans="1:9">
-      <c r="A208" s="46"/>
-      <c r="B208" s="47"/>
-      <c r="C208" s="48"/>
-      <c r="D208" s="47"/>
-      <c r="E208" s="47"/>
-      <c r="F208" s="49"/>
-      <c r="G208" s="49"/>
-      <c r="H208" s="68"/>
-      <c r="I208" s="47"/>
+      <c r="A208" s="43"/>
+      <c r="B208" s="50"/>
+      <c r="C208" s="51"/>
+      <c r="D208" s="50"/>
+      <c r="E208" s="50"/>
+      <c r="F208" s="50"/>
+      <c r="G208" s="50"/>
+      <c r="H208" s="69"/>
+      <c r="I208" s="50"/>
     </row>
     <row r="209" spans="1:9">
-      <c r="A209" s="43"/>
-      <c r="B209" s="50"/>
-      <c r="C209" s="51"/>
-      <c r="D209" s="50"/>
-      <c r="E209" s="50"/>
-      <c r="F209" s="50"/>
-      <c r="G209" s="50"/>
-      <c r="H209" s="69"/>
-      <c r="I209" s="50"/>
+      <c r="A209" s="46"/>
+      <c r="B209" s="47"/>
+      <c r="C209" s="48"/>
+      <c r="D209" s="47"/>
+      <c r="E209" s="47"/>
+      <c r="F209" s="49"/>
+      <c r="G209" s="49"/>
+      <c r="H209" s="68"/>
+      <c r="I209" s="47"/>
     </row>
     <row r="210" spans="1:9">
-      <c r="A210" s="46"/>
-      <c r="B210" s="47"/>
-      <c r="C210" s="48"/>
-      <c r="D210" s="47"/>
-      <c r="E210" s="47"/>
-      <c r="F210" s="49"/>
-      <c r="G210" s="49"/>
-      <c r="H210" s="68"/>
-      <c r="I210" s="47"/>
+      <c r="A210" s="43"/>
+      <c r="B210" s="50"/>
+      <c r="C210" s="51"/>
+      <c r="D210" s="50"/>
+      <c r="E210" s="50"/>
+      <c r="F210" s="50"/>
+      <c r="G210" s="50"/>
+      <c r="H210" s="69"/>
+      <c r="I210" s="50"/>
     </row>
     <row r="211" spans="1:9">
-      <c r="A211" s="43"/>
-      <c r="B211" s="50"/>
-      <c r="C211" s="51"/>
-      <c r="D211" s="50"/>
-      <c r="E211" s="50"/>
-      <c r="F211" s="50"/>
-      <c r="G211" s="50"/>
-      <c r="H211" s="69"/>
-      <c r="I211" s="50"/>
+      <c r="A211" s="46"/>
+      <c r="B211" s="47"/>
+      <c r="C211" s="48"/>
+      <c r="D211" s="47"/>
+      <c r="E211" s="47"/>
+      <c r="F211" s="49"/>
+      <c r="G211" s="49"/>
+      <c r="H211" s="68"/>
+      <c r="I211" s="47"/>
     </row>
     <row r="212" spans="1:9">
-      <c r="A212" s="46"/>
-      <c r="B212" s="47"/>
-      <c r="C212" s="48"/>
-      <c r="D212" s="47"/>
-      <c r="E212" s="47"/>
-      <c r="F212" s="49"/>
-      <c r="G212" s="49"/>
-      <c r="H212" s="68"/>
-      <c r="I212" s="47"/>
+      <c r="A212" s="43"/>
+      <c r="B212" s="50"/>
+      <c r="C212" s="51"/>
+      <c r="D212" s="50"/>
+      <c r="E212" s="50"/>
+      <c r="F212" s="50"/>
+      <c r="G212" s="50"/>
+      <c r="H212" s="69"/>
+      <c r="I212" s="50"/>
     </row>
     <row r="213" spans="1:9">
-      <c r="A213" s="43"/>
-      <c r="B213" s="50"/>
-      <c r="C213" s="51"/>
-      <c r="D213" s="50"/>
-      <c r="E213" s="50"/>
-      <c r="F213" s="50"/>
-      <c r="G213" s="50"/>
-      <c r="H213" s="69"/>
-      <c r="I213" s="50"/>
+      <c r="A213" s="46"/>
+      <c r="B213" s="47"/>
+      <c r="C213" s="48"/>
+      <c r="D213" s="47"/>
+      <c r="E213" s="47"/>
+      <c r="F213" s="49"/>
+      <c r="G213" s="49"/>
+      <c r="H213" s="68"/>
+      <c r="I213" s="47"/>
     </row>
     <row r="214" spans="1:9">
-      <c r="A214" s="46"/>
-      <c r="B214" s="47"/>
-      <c r="C214" s="48"/>
-      <c r="D214" s="47"/>
-      <c r="E214" s="47"/>
-      <c r="F214" s="49"/>
-      <c r="G214" s="49"/>
-      <c r="H214" s="68"/>
-      <c r="I214" s="47"/>
+      <c r="A214" s="43"/>
+      <c r="B214" s="50"/>
+      <c r="C214" s="51"/>
+      <c r="D214" s="50"/>
+      <c r="E214" s="50"/>
+      <c r="F214" s="50"/>
+      <c r="G214" s="50"/>
+      <c r="H214" s="69"/>
+      <c r="I214" s="50"/>
     </row>
     <row r="215" spans="1:9">
-      <c r="A215" s="43"/>
-      <c r="B215" s="50"/>
-      <c r="C215" s="51"/>
-      <c r="D215" s="50"/>
-      <c r="E215" s="50"/>
-      <c r="F215" s="50"/>
-      <c r="G215" s="50"/>
-      <c r="H215" s="69"/>
-      <c r="I215" s="50"/>
+      <c r="A215" s="46"/>
+      <c r="B215" s="47"/>
+      <c r="C215" s="48"/>
+      <c r="D215" s="47"/>
+      <c r="E215" s="47"/>
+      <c r="F215" s="49"/>
+      <c r="G215" s="49"/>
+      <c r="H215" s="68"/>
+      <c r="I215" s="47"/>
     </row>
     <row r="216" spans="1:9">
-      <c r="A216" s="46"/>
-      <c r="B216" s="47"/>
-      <c r="C216" s="48"/>
-      <c r="D216" s="47"/>
-      <c r="E216" s="47"/>
-      <c r="F216" s="49"/>
-      <c r="G216" s="49"/>
-      <c r="H216" s="68"/>
-      <c r="I216" s="47"/>
+      <c r="A216" s="43"/>
+      <c r="B216" s="50"/>
+      <c r="C216" s="51"/>
+      <c r="D216" s="50"/>
+      <c r="E216" s="50"/>
+      <c r="F216" s="50"/>
+      <c r="G216" s="50"/>
+      <c r="H216" s="69"/>
+      <c r="I216" s="50"/>
     </row>
     <row r="217" spans="1:9">
-      <c r="A217" s="43"/>
-      <c r="B217" s="50"/>
-      <c r="C217" s="51"/>
-      <c r="D217" s="50"/>
-      <c r="E217" s="50"/>
-      <c r="F217" s="50"/>
-      <c r="G217" s="50"/>
-      <c r="H217" s="69"/>
-      <c r="I217" s="50"/>
+      <c r="A217" s="46"/>
+      <c r="B217" s="47"/>
+      <c r="C217" s="48"/>
+      <c r="D217" s="47"/>
+      <c r="E217" s="47"/>
+      <c r="F217" s="49"/>
+      <c r="G217" s="49"/>
+      <c r="H217" s="68"/>
+      <c r="I217" s="47"/>
     </row>
     <row r="218" spans="1:9">
-      <c r="A218" s="46"/>
-      <c r="B218" s="47"/>
-      <c r="C218" s="48"/>
-      <c r="D218" s="47"/>
-      <c r="E218" s="47"/>
-      <c r="F218" s="49"/>
-      <c r="G218" s="49"/>
-      <c r="H218" s="68"/>
-      <c r="I218" s="47"/>
+      <c r="A218" s="43"/>
+      <c r="B218" s="50"/>
+      <c r="C218" s="51"/>
+      <c r="D218" s="50"/>
+      <c r="E218" s="50"/>
+      <c r="F218" s="50"/>
+      <c r="G218" s="50"/>
+      <c r="H218" s="69"/>
+      <c r="I218" s="50"/>
     </row>
     <row r="219" spans="1:9">
-      <c r="A219" s="43"/>
-      <c r="B219" s="50"/>
-      <c r="C219" s="51"/>
-      <c r="D219" s="50"/>
-      <c r="E219" s="50"/>
-      <c r="F219" s="50"/>
-      <c r="G219" s="50"/>
-      <c r="H219" s="69"/>
-      <c r="I219" s="50"/>
+      <c r="A219" s="46"/>
+      <c r="B219" s="47"/>
+      <c r="C219" s="48"/>
+      <c r="D219" s="47"/>
+      <c r="E219" s="47"/>
+      <c r="F219" s="49"/>
+      <c r="G219" s="49"/>
+      <c r="H219" s="68"/>
+      <c r="I219" s="47"/>
     </row>
     <row r="220" spans="1:9">
-      <c r="A220" s="46"/>
-      <c r="B220" s="47"/>
-      <c r="C220" s="48"/>
-      <c r="D220" s="47"/>
-      <c r="E220" s="47"/>
-      <c r="F220" s="49"/>
-      <c r="G220" s="49"/>
-      <c r="H220" s="68"/>
-      <c r="I220" s="47"/>
+      <c r="A220" s="43"/>
+      <c r="B220" s="50"/>
+      <c r="C220" s="51"/>
+      <c r="D220" s="50"/>
+      <c r="E220" s="50"/>
+      <c r="F220" s="50"/>
+      <c r="G220" s="50"/>
+      <c r="H220" s="69"/>
+      <c r="I220" s="50"/>
     </row>
     <row r="221" spans="1:9">
-      <c r="A221" s="43"/>
-      <c r="B221" s="50"/>
-      <c r="C221" s="51"/>
-      <c r="D221" s="50"/>
-      <c r="E221" s="50"/>
-      <c r="F221" s="50"/>
-      <c r="G221" s="50"/>
-      <c r="H221" s="69"/>
-      <c r="I221" s="50"/>
+      <c r="A221" s="46"/>
+      <c r="B221" s="47"/>
+      <c r="C221" s="48"/>
+      <c r="D221" s="47"/>
+      <c r="E221" s="47"/>
+      <c r="F221" s="49"/>
+      <c r="G221" s="49"/>
+      <c r="H221" s="68"/>
+      <c r="I221" s="47"/>
     </row>
     <row r="222" spans="1:9">
-      <c r="A222" s="46"/>
-      <c r="B222" s="47"/>
-      <c r="C222" s="48"/>
-      <c r="D222" s="47"/>
-      <c r="E222" s="47"/>
-      <c r="F222" s="49"/>
-      <c r="G222" s="49"/>
-      <c r="H222" s="68"/>
-      <c r="I222" s="47"/>
+      <c r="A222" s="43"/>
+      <c r="B222" s="50"/>
+      <c r="C222" s="51"/>
+      <c r="D222" s="50"/>
+      <c r="E222" s="50"/>
+      <c r="F222" s="50"/>
+      <c r="G222" s="50"/>
+      <c r="H222" s="69"/>
+      <c r="I222" s="50"/>
     </row>
     <row r="223" spans="1:9">
-      <c r="A223" s="43"/>
-      <c r="B223" s="50"/>
-      <c r="C223" s="51"/>
-      <c r="D223" s="50"/>
-      <c r="E223" s="50"/>
-      <c r="F223" s="50"/>
-      <c r="G223" s="50"/>
-      <c r="H223" s="69"/>
-      <c r="I223" s="50"/>
+      <c r="A223" s="46"/>
+      <c r="B223" s="47"/>
+      <c r="C223" s="48"/>
+      <c r="D223" s="47"/>
+      <c r="E223" s="47"/>
+      <c r="F223" s="49"/>
+      <c r="G223" s="49"/>
+      <c r="H223" s="68"/>
+      <c r="I223" s="47"/>
     </row>
     <row r="224" spans="1:9">
-      <c r="A224" s="46"/>
-      <c r="B224" s="47"/>
-      <c r="C224" s="48"/>
-      <c r="D224" s="47"/>
-      <c r="E224" s="47"/>
-      <c r="F224" s="49"/>
-      <c r="G224" s="49"/>
-      <c r="H224" s="68"/>
-      <c r="I224" s="47"/>
+      <c r="A224" s="43"/>
+      <c r="B224" s="50"/>
+      <c r="C224" s="51"/>
+      <c r="D224" s="50"/>
+      <c r="E224" s="50"/>
+      <c r="F224" s="50"/>
+      <c r="G224" s="50"/>
+      <c r="H224" s="69"/>
+      <c r="I224" s="50"/>
     </row>
     <row r="225" spans="1:9">
-      <c r="A225" s="43"/>
-      <c r="B225" s="50"/>
-      <c r="C225" s="51"/>
-      <c r="D225" s="50"/>
-      <c r="E225" s="50"/>
-      <c r="F225" s="50"/>
-      <c r="G225" s="50"/>
-      <c r="H225" s="69"/>
-      <c r="I225" s="50"/>
+      <c r="A225" s="46"/>
+      <c r="B225" s="47"/>
+      <c r="C225" s="48"/>
+      <c r="D225" s="47"/>
+      <c r="E225" s="47"/>
+      <c r="F225" s="49"/>
+      <c r="G225" s="49"/>
+      <c r="H225" s="68"/>
+      <c r="I225" s="47"/>
     </row>
     <row r="226" spans="1:9">
-      <c r="A226" s="46"/>
-      <c r="B226" s="47"/>
-      <c r="C226" s="48"/>
-      <c r="D226" s="47"/>
-      <c r="E226" s="47"/>
-      <c r="F226" s="49"/>
-      <c r="G226" s="49"/>
-      <c r="H226" s="68"/>
-      <c r="I226" s="47"/>
+      <c r="A226" s="43"/>
+      <c r="B226" s="50"/>
+      <c r="C226" s="51"/>
+      <c r="D226" s="50"/>
+      <c r="E226" s="50"/>
+      <c r="F226" s="50"/>
+      <c r="G226" s="50"/>
+      <c r="H226" s="69"/>
+      <c r="I226" s="50"/>
     </row>
     <row r="227" spans="1:9">
-      <c r="A227" s="43"/>
-      <c r="B227" s="50"/>
-      <c r="C227" s="51"/>
-      <c r="D227" s="50"/>
-      <c r="E227" s="50"/>
-      <c r="F227" s="50"/>
-      <c r="G227" s="50"/>
-      <c r="H227" s="69"/>
-      <c r="I227" s="50"/>
+      <c r="A227" s="46"/>
+      <c r="B227" s="47"/>
+      <c r="C227" s="48"/>
+      <c r="D227" s="47"/>
+      <c r="E227" s="47"/>
+      <c r="F227" s="49"/>
+      <c r="G227" s="49"/>
+      <c r="H227" s="68"/>
+      <c r="I227" s="47"/>
     </row>
     <row r="228" spans="1:9">
-      <c r="A228" s="46"/>
-      <c r="B228" s="47"/>
-      <c r="C228" s="48"/>
-      <c r="D228" s="47"/>
-      <c r="E228" s="47"/>
-      <c r="F228" s="49"/>
-      <c r="G228" s="49"/>
-      <c r="H228" s="68"/>
-      <c r="I228" s="47"/>
+      <c r="A228" s="43"/>
+      <c r="B228" s="50"/>
+      <c r="C228" s="51"/>
+      <c r="D228" s="50"/>
+      <c r="E228" s="50"/>
+      <c r="F228" s="50"/>
+      <c r="G228" s="50"/>
+      <c r="H228" s="69"/>
+      <c r="I228" s="50"/>
     </row>
     <row r="229" spans="1:9">
-      <c r="A229" s="43"/>
-      <c r="B229" s="50"/>
-      <c r="C229" s="51"/>
-      <c r="D229" s="50"/>
-      <c r="E229" s="50"/>
-      <c r="F229" s="50"/>
-      <c r="G229" s="50"/>
-      <c r="H229" s="69"/>
-      <c r="I229" s="50"/>
+      <c r="A229" s="46"/>
+      <c r="B229" s="47"/>
+      <c r="C229" s="48"/>
+      <c r="D229" s="47"/>
+      <c r="E229" s="47"/>
+      <c r="F229" s="49"/>
+      <c r="G229" s="49"/>
+      <c r="H229" s="68"/>
+      <c r="I229" s="47"/>
     </row>
     <row r="230" spans="1:9">
-      <c r="A230" s="46"/>
-      <c r="B230" s="47"/>
-      <c r="C230" s="48"/>
-      <c r="D230" s="47"/>
-      <c r="E230" s="47"/>
-      <c r="F230" s="49"/>
-      <c r="G230" s="49"/>
-      <c r="H230" s="68"/>
-      <c r="I230" s="47"/>
+      <c r="A230" s="43"/>
+      <c r="B230" s="50"/>
+      <c r="C230" s="51"/>
+      <c r="D230" s="50"/>
+      <c r="E230" s="50"/>
+      <c r="F230" s="50"/>
+      <c r="G230" s="50"/>
+      <c r="H230" s="69"/>
+      <c r="I230" s="50"/>
     </row>
     <row r="231" spans="1:9">
-      <c r="A231" s="43"/>
-      <c r="B231" s="50"/>
-      <c r="C231" s="51"/>
-      <c r="D231" s="50"/>
-      <c r="E231" s="50"/>
-      <c r="F231" s="50"/>
-      <c r="G231" s="50"/>
-      <c r="H231" s="69"/>
-      <c r="I231" s="50"/>
+      <c r="A231" s="46"/>
+      <c r="B231" s="47"/>
+      <c r="C231" s="48"/>
+      <c r="D231" s="47"/>
+      <c r="E231" s="47"/>
+      <c r="F231" s="49"/>
+      <c r="G231" s="49"/>
+      <c r="H231" s="68"/>
+      <c r="I231" s="47"/>
     </row>
     <row r="232" spans="1:9">
-      <c r="A232" s="46"/>
-      <c r="B232" s="47"/>
-      <c r="C232" s="48"/>
-      <c r="D232" s="47"/>
-      <c r="E232" s="47"/>
-      <c r="F232" s="49"/>
-      <c r="G232" s="49"/>
-      <c r="H232" s="68"/>
-      <c r="I232" s="47"/>
+      <c r="A232" s="43"/>
+      <c r="B232" s="50"/>
+      <c r="C232" s="51"/>
+      <c r="D232" s="50"/>
+      <c r="E232" s="50"/>
+      <c r="F232" s="50"/>
+      <c r="G232" s="50"/>
+      <c r="H232" s="69"/>
+      <c r="I232" s="50"/>
     </row>
     <row r="233" spans="1:9">
-      <c r="A233" s="43"/>
-      <c r="B233" s="50"/>
-      <c r="C233" s="51"/>
-      <c r="D233" s="50"/>
-      <c r="E233" s="50"/>
-      <c r="F233" s="50"/>
-      <c r="G233" s="50"/>
-      <c r="H233" s="69"/>
-      <c r="I233" s="50"/>
+      <c r="A233" s="46"/>
+      <c r="B233" s="47"/>
+      <c r="C233" s="48"/>
+      <c r="D233" s="47"/>
+      <c r="E233" s="47"/>
+      <c r="F233" s="49"/>
+      <c r="G233" s="49"/>
+      <c r="H233" s="68"/>
+      <c r="I233" s="47"/>
     </row>
     <row r="234" spans="1:9">
-      <c r="A234" s="46"/>
-      <c r="B234" s="47"/>
-      <c r="C234" s="48"/>
-      <c r="D234" s="47"/>
-      <c r="E234" s="47"/>
-      <c r="F234" s="49"/>
-      <c r="G234" s="49"/>
-      <c r="H234" s="68"/>
-      <c r="I234" s="47"/>
+      <c r="A234" s="43"/>
+      <c r="B234" s="50"/>
+      <c r="C234" s="51"/>
+      <c r="D234" s="50"/>
+      <c r="E234" s="50"/>
+      <c r="F234" s="50"/>
+      <c r="G234" s="50"/>
+      <c r="H234" s="69"/>
+      <c r="I234" s="50"/>
     </row>
     <row r="235" spans="1:9">
-      <c r="A235" s="43"/>
-      <c r="B235" s="50"/>
-      <c r="C235" s="51"/>
-      <c r="D235" s="50"/>
-      <c r="E235" s="50"/>
-      <c r="F235" s="50"/>
-      <c r="G235" s="50"/>
-      <c r="H235" s="69"/>
-      <c r="I235" s="50"/>
+      <c r="A235" s="46"/>
+      <c r="B235" s="47"/>
+      <c r="C235" s="48"/>
+      <c r="D235" s="47"/>
+      <c r="E235" s="47"/>
+      <c r="F235" s="49"/>
+      <c r="G235" s="49"/>
+      <c r="H235" s="68"/>
+      <c r="I235" s="47"/>
     </row>
     <row r="236" spans="1:9">
-      <c r="A236" s="46"/>
-      <c r="B236" s="47"/>
-      <c r="C236" s="48"/>
-      <c r="D236" s="47"/>
-      <c r="E236" s="47"/>
-      <c r="F236" s="49"/>
-      <c r="G236" s="49"/>
-      <c r="H236" s="68"/>
-      <c r="I236" s="47"/>
+      <c r="A236" s="43"/>
+      <c r="B236" s="50"/>
+      <c r="C236" s="51"/>
+      <c r="D236" s="50"/>
+      <c r="E236" s="50"/>
+      <c r="F236" s="50"/>
+      <c r="G236" s="50"/>
+      <c r="H236" s="69"/>
+      <c r="I236" s="50"/>
     </row>
     <row r="237" spans="1:9">
-      <c r="A237" s="43"/>
-      <c r="B237" s="50"/>
-      <c r="C237" s="51"/>
-      <c r="D237" s="50"/>
-      <c r="E237" s="50"/>
-      <c r="F237" s="50"/>
-      <c r="G237" s="50"/>
-      <c r="H237" s="69"/>
-      <c r="I237" s="50"/>
+      <c r="A237" s="46"/>
+      <c r="B237" s="47"/>
+      <c r="C237" s="48"/>
+      <c r="D237" s="47"/>
+      <c r="E237" s="47"/>
+      <c r="F237" s="49"/>
+      <c r="G237" s="49"/>
+      <c r="H237" s="68"/>
+      <c r="I237" s="47"/>
     </row>
     <row r="238" spans="1:9">
-      <c r="A238" s="46"/>
-      <c r="B238" s="47"/>
-      <c r="C238" s="48"/>
-      <c r="D238" s="47"/>
-      <c r="E238" s="47"/>
-      <c r="F238" s="49"/>
-      <c r="G238" s="49"/>
-      <c r="H238" s="68"/>
-      <c r="I238" s="47"/>
+      <c r="A238" s="43"/>
+      <c r="B238" s="50"/>
+      <c r="C238" s="51"/>
+      <c r="D238" s="50"/>
+      <c r="E238" s="50"/>
+      <c r="F238" s="50"/>
+      <c r="G238" s="50"/>
+      <c r="H238" s="69"/>
+      <c r="I238" s="50"/>
     </row>
     <row r="239" spans="1:9">
-      <c r="A239" s="43"/>
-      <c r="B239" s="50"/>
-      <c r="C239" s="51"/>
-      <c r="D239" s="50"/>
-      <c r="E239" s="50"/>
-      <c r="F239" s="50"/>
-      <c r="G239" s="50"/>
-      <c r="H239" s="69"/>
-      <c r="I239" s="50"/>
+      <c r="A239" s="46"/>
+      <c r="B239" s="47"/>
+      <c r="C239" s="48"/>
+      <c r="D239" s="47"/>
+      <c r="E239" s="47"/>
+      <c r="F239" s="49"/>
+      <c r="G239" s="49"/>
+      <c r="H239" s="68"/>
+      <c r="I239" s="47"/>
     </row>
     <row r="240" spans="1:9">
-      <c r="A240" s="46"/>
-      <c r="B240" s="47"/>
-      <c r="C240" s="48"/>
-      <c r="D240" s="47"/>
-      <c r="E240" s="47"/>
-      <c r="F240" s="49"/>
-      <c r="G240" s="49"/>
-      <c r="H240" s="68"/>
-      <c r="I240" s="47"/>
+      <c r="A240" s="43"/>
+      <c r="B240" s="50"/>
+      <c r="C240" s="51"/>
+      <c r="D240" s="50"/>
+      <c r="E240" s="50"/>
+      <c r="F240" s="50"/>
+      <c r="G240" s="50"/>
+      <c r="H240" s="69"/>
+      <c r="I240" s="50"/>
     </row>
     <row r="241" spans="1:9">
-      <c r="A241" s="43"/>
-      <c r="B241" s="50"/>
-      <c r="C241" s="51"/>
-      <c r="D241" s="50"/>
-      <c r="E241" s="50"/>
-      <c r="F241" s="50"/>
-      <c r="G241" s="50"/>
-      <c r="H241" s="69"/>
-      <c r="I241" s="50"/>
+      <c r="A241" s="46"/>
+      <c r="B241" s="47"/>
+      <c r="C241" s="48"/>
+      <c r="D241" s="47"/>
+      <c r="E241" s="47"/>
+      <c r="F241" s="49"/>
+      <c r="G241" s="49"/>
+      <c r="H241" s="68"/>
+      <c r="I241" s="47"/>
     </row>
     <row r="242" spans="1:9">
-      <c r="A242" s="46"/>
-      <c r="B242" s="47"/>
-      <c r="C242" s="48"/>
-      <c r="D242" s="47"/>
-      <c r="E242" s="47"/>
-      <c r="F242" s="49"/>
-      <c r="G242" s="49"/>
-      <c r="H242" s="68"/>
-      <c r="I242" s="47"/>
+      <c r="A242" s="43"/>
+      <c r="B242" s="50"/>
+      <c r="C242" s="51"/>
+      <c r="D242" s="50"/>
+      <c r="E242" s="50"/>
+      <c r="F242" s="50"/>
+      <c r="G242" s="50"/>
+      <c r="H242" s="69"/>
+      <c r="I242" s="50"/>
     </row>
     <row r="243" spans="1:9">
-      <c r="A243" s="43"/>
-      <c r="B243" s="50"/>
-      <c r="C243" s="51"/>
-      <c r="D243" s="50"/>
-      <c r="E243" s="50"/>
-      <c r="F243" s="50"/>
-      <c r="G243" s="50"/>
-      <c r="H243" s="69"/>
-      <c r="I243" s="50"/>
+      <c r="A243" s="46"/>
+      <c r="B243" s="47"/>
+      <c r="C243" s="48"/>
+      <c r="D243" s="47"/>
+      <c r="E243" s="47"/>
+      <c r="F243" s="49"/>
+      <c r="G243" s="49"/>
+      <c r="H243" s="68"/>
+      <c r="I243" s="47"/>
     </row>
     <row r="244" spans="1:9">
-      <c r="A244" s="46"/>
-      <c r="B244" s="47"/>
-      <c r="C244" s="48"/>
-      <c r="D244" s="47"/>
-      <c r="E244" s="47"/>
-      <c r="F244" s="49"/>
-      <c r="G244" s="49"/>
-      <c r="H244" s="68"/>
-      <c r="I244" s="47"/>
+      <c r="A244" s="43"/>
+      <c r="B244" s="50"/>
+      <c r="C244" s="51"/>
+      <c r="D244" s="50"/>
+      <c r="E244" s="50"/>
+      <c r="F244" s="50"/>
+      <c r="G244" s="50"/>
+      <c r="H244" s="69"/>
+      <c r="I244" s="50"/>
     </row>
     <row r="245" spans="1:9">
-      <c r="A245" s="43"/>
-      <c r="B245" s="50"/>
-      <c r="C245" s="51"/>
-      <c r="D245" s="50"/>
-      <c r="E245" s="50"/>
-      <c r="F245" s="50"/>
-      <c r="G245" s="50"/>
-      <c r="H245" s="69"/>
-      <c r="I245" s="50"/>
+      <c r="A245" s="46"/>
+      <c r="B245" s="47"/>
+      <c r="C245" s="48"/>
+      <c r="D245" s="47"/>
+      <c r="E245" s="47"/>
+      <c r="F245" s="49"/>
+      <c r="G245" s="49"/>
+      <c r="H245" s="68"/>
+      <c r="I245" s="47"/>
     </row>
     <row r="246" spans="1:9">
-      <c r="A246" s="46"/>
-      <c r="B246" s="47"/>
-      <c r="C246" s="48"/>
-      <c r="D246" s="47"/>
-      <c r="E246" s="47"/>
-      <c r="F246" s="49"/>
-      <c r="G246" s="49"/>
-      <c r="H246" s="68"/>
-      <c r="I246" s="47"/>
+      <c r="A246" s="43"/>
+      <c r="B246" s="50"/>
+      <c r="C246" s="51"/>
+      <c r="D246" s="50"/>
+      <c r="E246" s="50"/>
+      <c r="F246" s="50"/>
+      <c r="G246" s="50"/>
+      <c r="H246" s="69"/>
+      <c r="I246" s="50"/>
     </row>
     <row r="247" spans="1:9">
-      <c r="A247" s="43"/>
-      <c r="B247" s="50"/>
-      <c r="C247" s="51"/>
-      <c r="D247" s="50"/>
-      <c r="E247" s="50"/>
-      <c r="F247" s="50"/>
-      <c r="G247" s="50"/>
-      <c r="H247" s="69"/>
-      <c r="I247" s="50"/>
+      <c r="A247" s="46"/>
+      <c r="B247" s="47"/>
+      <c r="C247" s="48"/>
+      <c r="D247" s="47"/>
+      <c r="E247" s="47"/>
+      <c r="F247" s="49"/>
+      <c r="G247" s="49"/>
+      <c r="H247" s="68"/>
+      <c r="I247" s="47"/>
     </row>
     <row r="248" spans="1:9">
-      <c r="A248" s="46"/>
-      <c r="B248" s="47"/>
-      <c r="C248" s="48"/>
-      <c r="D248" s="47"/>
-      <c r="E248" s="47"/>
-      <c r="F248" s="49"/>
-      <c r="G248" s="49"/>
-      <c r="H248" s="68"/>
-      <c r="I248" s="47"/>
+      <c r="A248" s="43"/>
+      <c r="B248" s="50"/>
+      <c r="C248" s="51"/>
+      <c r="D248" s="50"/>
+      <c r="E248" s="50"/>
+      <c r="F248" s="50"/>
+      <c r="G248" s="50"/>
+      <c r="H248" s="69"/>
+      <c r="I248" s="50"/>
     </row>
     <row r="249" spans="1:9">
-      <c r="A249" s="43"/>
-      <c r="B249" s="50"/>
-      <c r="C249" s="51"/>
-      <c r="D249" s="50"/>
-      <c r="E249" s="50"/>
-      <c r="F249" s="50"/>
-      <c r="G249" s="50"/>
-      <c r="H249" s="69"/>
-      <c r="I249" s="50"/>
+      <c r="A249" s="46"/>
+      <c r="B249" s="47"/>
+      <c r="C249" s="48"/>
+      <c r="D249" s="47"/>
+      <c r="E249" s="47"/>
+      <c r="F249" s="49"/>
+      <c r="G249" s="49"/>
+      <c r="H249" s="68"/>
+      <c r="I249" s="47"/>
     </row>
     <row r="250" spans="1:9">
-      <c r="A250" s="46"/>
-      <c r="B250" s="47"/>
-      <c r="C250" s="48"/>
-      <c r="D250" s="47"/>
-      <c r="E250" s="47"/>
-      <c r="F250" s="49"/>
-      <c r="G250" s="49"/>
-      <c r="H250" s="68"/>
-      <c r="I250" s="47"/>
+      <c r="A250" s="43"/>
+      <c r="B250" s="50"/>
+      <c r="C250" s="51"/>
+      <c r="D250" s="50"/>
+      <c r="E250" s="50"/>
+      <c r="F250" s="50"/>
+      <c r="G250" s="50"/>
+      <c r="H250" s="69"/>
+      <c r="I250" s="50"/>
     </row>
     <row r="251" spans="1:9">
-      <c r="A251" s="43"/>
-      <c r="B251" s="50"/>
-      <c r="C251" s="51"/>
-      <c r="D251" s="50"/>
-      <c r="E251" s="50"/>
-      <c r="F251" s="50"/>
-      <c r="G251" s="50"/>
-      <c r="H251" s="69"/>
-      <c r="I251" s="50"/>
+      <c r="A251" s="46"/>
+      <c r="B251" s="47"/>
+      <c r="C251" s="48"/>
+      <c r="D251" s="47"/>
+      <c r="E251" s="47"/>
+      <c r="F251" s="49"/>
+      <c r="G251" s="49"/>
+      <c r="H251" s="68"/>
+      <c r="I251" s="47"/>
     </row>
     <row r="252" spans="1:9">
-      <c r="A252" s="46"/>
-      <c r="B252" s="47"/>
-      <c r="C252" s="48"/>
-      <c r="D252" s="47"/>
-      <c r="E252" s="47"/>
-      <c r="F252" s="49"/>
-      <c r="G252" s="49"/>
-      <c r="H252" s="68"/>
-      <c r="I252" s="47"/>
+      <c r="A252" s="43"/>
+      <c r="B252" s="50"/>
+      <c r="C252" s="51"/>
+      <c r="D252" s="50"/>
+      <c r="E252" s="50"/>
+      <c r="F252" s="50"/>
+      <c r="G252" s="50"/>
+      <c r="H252" s="69"/>
+      <c r="I252" s="50"/>
     </row>
     <row r="253" spans="1:9">
-      <c r="A253" s="43"/>
-      <c r="B253" s="50"/>
-      <c r="C253" s="51"/>
-      <c r="D253" s="50"/>
-      <c r="E253" s="50"/>
-      <c r="F253" s="50"/>
-      <c r="G253" s="50"/>
-      <c r="H253" s="69"/>
-      <c r="I253" s="50"/>
+      <c r="A253" s="46"/>
+      <c r="B253" s="47"/>
+      <c r="C253" s="48"/>
+      <c r="D253" s="47"/>
+      <c r="E253" s="47"/>
+      <c r="F253" s="49"/>
+      <c r="G253" s="49"/>
+      <c r="H253" s="68"/>
+      <c r="I253" s="47"/>
     </row>
     <row r="254" spans="1:9">
-      <c r="A254" s="46"/>
-      <c r="B254" s="47"/>
-      <c r="C254" s="48"/>
-      <c r="D254" s="47"/>
-      <c r="E254" s="47"/>
-      <c r="F254" s="49"/>
-      <c r="G254" s="49"/>
-      <c r="H254" s="68"/>
-      <c r="I254" s="47"/>
+      <c r="A254" s="43"/>
+      <c r="B254" s="50"/>
+      <c r="C254" s="51"/>
+      <c r="D254" s="50"/>
+      <c r="E254" s="50"/>
+      <c r="F254" s="50"/>
+      <c r="G254" s="50"/>
+      <c r="H254" s="69"/>
+      <c r="I254" s="50"/>
     </row>
     <row r="255" spans="1:9">
-      <c r="A255" s="43"/>
-      <c r="B255" s="50"/>
-      <c r="C255" s="51"/>
-      <c r="D255" s="50"/>
-      <c r="E255" s="50"/>
-      <c r="F255" s="50"/>
-      <c r="G255" s="50"/>
-      <c r="H255" s="69"/>
-      <c r="I255" s="50"/>
+      <c r="A255" s="46"/>
+      <c r="B255" s="47"/>
+      <c r="C255" s="48"/>
+      <c r="D255" s="47"/>
+      <c r="E255" s="47"/>
+      <c r="F255" s="49"/>
+      <c r="G255" s="49"/>
+      <c r="H255" s="68"/>
+      <c r="I255" s="47"/>
     </row>
     <row r="256" spans="1:9">
-      <c r="A256" s="46"/>
-      <c r="B256" s="47"/>
-      <c r="C256" s="48"/>
-      <c r="D256" s="47"/>
-      <c r="E256" s="47"/>
-      <c r="F256" s="49"/>
-      <c r="G256" s="49"/>
-      <c r="H256" s="68"/>
-      <c r="I256" s="47"/>
+      <c r="A256" s="43"/>
+      <c r="B256" s="50"/>
+      <c r="C256" s="51"/>
+      <c r="D256" s="50"/>
+      <c r="E256" s="50"/>
+      <c r="F256" s="50"/>
+      <c r="G256" s="50"/>
+      <c r="H256" s="69"/>
+      <c r="I256" s="50"/>
     </row>
     <row r="257" spans="1:9">
-      <c r="A257" s="43"/>
-      <c r="B257" s="50"/>
-      <c r="C257" s="51"/>
-      <c r="D257" s="50"/>
-      <c r="E257" s="50"/>
-      <c r="F257" s="50"/>
-      <c r="G257" s="50"/>
-      <c r="H257" s="69"/>
-      <c r="I257" s="50"/>
+      <c r="A257" s="46"/>
+      <c r="B257" s="47"/>
+      <c r="C257" s="48"/>
+      <c r="D257" s="47"/>
+      <c r="E257" s="47"/>
+      <c r="F257" s="49"/>
+      <c r="G257" s="49"/>
+      <c r="H257" s="68"/>
+      <c r="I257" s="47"/>
     </row>
     <row r="258" spans="1:9">
-      <c r="A258" s="46"/>
-      <c r="B258" s="47"/>
-      <c r="C258" s="48"/>
-      <c r="D258" s="47"/>
-      <c r="E258" s="47"/>
-      <c r="F258" s="49"/>
-      <c r="G258" s="49"/>
-      <c r="H258" s="68"/>
-      <c r="I258" s="47"/>
+      <c r="A258" s="43"/>
+      <c r="B258" s="50"/>
+      <c r="C258" s="51"/>
+      <c r="D258" s="50"/>
+      <c r="E258" s="50"/>
+      <c r="F258" s="50"/>
+      <c r="G258" s="50"/>
+      <c r="H258" s="69"/>
+      <c r="I258" s="50"/>
     </row>
     <row r="259" spans="1:9">
-      <c r="A259" s="43"/>
-      <c r="B259" s="50"/>
-      <c r="C259" s="51"/>
-      <c r="D259" s="50"/>
-      <c r="E259" s="50"/>
-      <c r="F259" s="50"/>
-      <c r="G259" s="50"/>
-      <c r="H259" s="69"/>
-      <c r="I259" s="50"/>
+      <c r="A259" s="46"/>
+      <c r="B259" s="47"/>
+      <c r="C259" s="48"/>
+      <c r="D259" s="47"/>
+      <c r="E259" s="47"/>
+      <c r="F259" s="49"/>
+      <c r="G259" s="49"/>
+      <c r="H259" s="68"/>
+      <c r="I259" s="47"/>
     </row>
     <row r="260" spans="1:9">
-      <c r="A260" s="46"/>
-      <c r="B260" s="47"/>
-      <c r="C260" s="48"/>
-      <c r="D260" s="47"/>
-      <c r="E260" s="47"/>
-      <c r="F260" s="49"/>
-      <c r="G260" s="49"/>
-      <c r="H260" s="68"/>
-      <c r="I260" s="47"/>
+      <c r="A260" s="43"/>
+      <c r="B260" s="50"/>
+      <c r="C260" s="51"/>
+      <c r="D260" s="50"/>
+      <c r="E260" s="50"/>
+      <c r="F260" s="50"/>
+      <c r="G260" s="50"/>
+      <c r="H260" s="69"/>
+      <c r="I260" s="50"/>
     </row>
     <row r="261" spans="1:9">
-      <c r="A261" s="43"/>
-      <c r="B261" s="50"/>
-      <c r="C261" s="51"/>
-      <c r="D261" s="50"/>
-      <c r="E261" s="50"/>
-      <c r="F261" s="50"/>
-      <c r="G261" s="50"/>
-      <c r="H261" s="69"/>
-      <c r="I261" s="50"/>
-    </row>
-    <row r="262" spans="1:9">
-      <c r="A262" s="42"/>
-      <c r="B262" s="23"/>
-      <c r="C262" s="24"/>
-      <c r="D262" s="23"/>
-      <c r="E262" s="23"/>
-      <c r="I262" s="23"/>
+      <c r="A261" s="42"/>
+      <c r="B261" s="23"/>
+      <c r="C261" s="24"/>
+      <c r="D261" s="23"/>
+      <c r="E261" s="23"/>
+      <c r="I261" s="23"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I98" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I9999" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I9998" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19597,7 +19586,7 @@
         <v>3600</v>
       </c>
       <c r="L52" s="30" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M52" s="30"/>
       <c r="N52" s="30" t="s">
@@ -19653,7 +19642,7 @@
         <v>1941</v>
       </c>
       <c r="L53" s="28" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="M53" s="28"/>
       <c r="N53" s="28" t="s">
@@ -19663,7 +19652,7 @@
         <v>195</v>
       </c>
       <c r="P53" s="28" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="Q53" s="28"/>
       <c r="R53" s="28"/>
@@ -19765,7 +19754,7 @@
         <v>995</v>
       </c>
       <c r="L55" s="28" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="M55" s="28" t="s">
         <v>46</v>
@@ -19988,7 +19977,7 @@
         <v>180</v>
       </c>
       <c r="O59" s="28" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="P59" s="28" t="s">
         <v>203</v>
@@ -20037,7 +20026,7 @@
         <v>1080</v>
       </c>
       <c r="L60" s="30" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="M60" s="30" t="s">
         <v>46</v>
@@ -20093,17 +20082,17 @@
         <v>4384</v>
       </c>
       <c r="L61" s="28" t="s">
-        <v>744</v>
+        <v>738</v>
       </c>
       <c r="M61" s="28"/>
       <c r="N61" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O61" s="28" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="P61" s="28" t="s">
-        <v>745</v>
+        <v>739</v>
       </c>
       <c r="Q61" s="28" t="s">
         <v>478</v>
@@ -20151,7 +20140,7 @@
         <v>562</v>
       </c>
       <c r="L62" s="30" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="M62" s="30"/>
       <c r="N62" s="30" t="s">
@@ -20563,7 +20552,7 @@
         <v>0</v>
       </c>
       <c r="L70" s="30" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="M70" s="30"/>
       <c r="N70" s="30" t="s">
@@ -21151,7 +21140,7 @@
         <v>0</v>
       </c>
       <c r="L81" s="28" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="M81" s="28"/>
       <c r="N81" s="28" t="s">
@@ -21203,7 +21192,7 @@
         <v>0</v>
       </c>
       <c r="L82" s="30" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="M82" s="30"/>
       <c r="N82" s="30" t="s">
@@ -21363,7 +21352,7 @@
         <v>895</v>
       </c>
       <c r="L85" s="28" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="M85" s="28"/>
       <c r="N85" s="28" t="s">
@@ -21417,7 +21406,7 @@
         <v>2090</v>
       </c>
       <c r="L86" s="30" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="M86" s="30"/>
       <c r="N86" s="30" t="s">
@@ -21679,7 +21668,7 @@
         <v>389</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="M91" s="28"/>
       <c r="N91" s="28" t="s">
@@ -21731,7 +21720,7 @@
         <v>0</v>
       </c>
       <c r="L92" s="30" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30" t="s">
@@ -22453,10 +22442,10 @@
         <v>1600</v>
       </c>
       <c r="F106" s="31">
+        <v>0</v>
+      </c>
+      <c r="G106" s="31">
         <v>1</v>
-      </c>
-      <c r="G106" s="31">
-        <v>0</v>
       </c>
       <c r="H106" s="30">
         <f t="shared" si="9"/>
@@ -22468,18 +22457,16 @@
       </c>
       <c r="J106" s="30">
         <f t="shared" si="10"/>
-        <v>976</v>
+        <v>0</v>
       </c>
       <c r="K106" s="30">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="L106" s="30" t="s">
-        <v>700</v>
-      </c>
+        <v>976</v>
+      </c>
+      <c r="L106" s="30"/>
       <c r="M106" s="30"/>
       <c r="N106" s="30" t="s">
-        <v>122</v>
+        <v>191</v>
       </c>
       <c r="O106" s="30" t="s">
         <v>197</v>
@@ -22918,7 +22905,7 @@
       <c r="S114" s="30"/>
       <c r="T114" s="30"/>
     </row>
-    <row r="115" spans="1:20" ht="15" customHeight="1">
+    <row r="115" spans="1:20" ht="34" customHeight="1">
       <c r="A115" s="28" t="s">
         <v>454</v>
       </c>
@@ -22935,10 +22922,10 @@
         <v>1599</v>
       </c>
       <c r="F115" s="29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G115" s="29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H115" s="28">
         <f t="shared" si="9"/>
@@ -22950,14 +22937,14 @@
       </c>
       <c r="J115" s="28">
         <f t="shared" si="10"/>
-        <v>3764.2799999999997</v>
+        <v>5019.04</v>
       </c>
       <c r="K115" s="28">
         <f t="shared" si="11"/>
-        <v>2509.52</v>
+        <v>1254.76</v>
       </c>
       <c r="L115" s="28" t="s">
-        <v>736</v>
+        <v>757</v>
       </c>
       <c r="M115" s="28"/>
       <c r="N115" s="28" t="s">
@@ -22965,7 +22952,7 @@
       </c>
       <c r="O115" s="28"/>
       <c r="P115" s="89" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="Q115" s="28"/>
       <c r="R115" s="28"/>
@@ -23011,7 +22998,7 @@
         <v>891.5</v>
       </c>
       <c r="L116" s="30" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="M116" s="30"/>
       <c r="N116" s="30" t="s">
@@ -23019,7 +23006,7 @@
       </c>
       <c r="O116" s="30"/>
       <c r="P116" s="30" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
       <c r="Q116" s="30"/>
       <c r="R116" s="30"/>
@@ -23233,7 +23220,7 @@
       </c>
       <c r="O120" s="30"/>
       <c r="P120" s="30" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
       <c r="Q120" s="30"/>
       <c r="R120" s="30"/>
@@ -23287,7 +23274,7 @@
       </c>
       <c r="O121" s="28"/>
       <c r="P121" s="28" t="s">
-        <v>727</v>
+        <v>722</v>
       </c>
       <c r="Q121" s="28"/>
       <c r="R121" s="28"/>
@@ -23333,14 +23320,14 @@
         <v>3525</v>
       </c>
       <c r="L122" s="30" t="s">
-        <v>756</v>
+        <v>750</v>
       </c>
       <c r="M122" s="30"/>
       <c r="N122" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O122" s="30" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="P122" s="30"/>
       <c r="Q122" s="30"/>
@@ -23387,7 +23374,7 @@
         <v>0</v>
       </c>
       <c r="L123" s="81" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="M123" s="81"/>
       <c r="N123" s="81" t="s">
@@ -23547,7 +23534,7 @@
         <v>0</v>
       </c>
       <c r="L126" s="30" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="M126" s="30"/>
       <c r="N126" s="30" t="s">
@@ -23683,10 +23670,10 @@
         <v>1650</v>
       </c>
       <c r="F129" s="82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G129" s="82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H129" s="80">
         <f t="shared" si="15"/>
@@ -23698,16 +23685,18 @@
       </c>
       <c r="J129" s="81">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>1155</v>
       </c>
       <c r="K129" s="81">
         <f t="shared" si="17"/>
-        <v>1155</v>
-      </c>
-      <c r="L129" s="28"/>
+        <v>0</v>
+      </c>
+      <c r="L129" s="28" t="s">
+        <v>756</v>
+      </c>
       <c r="M129" s="28"/>
       <c r="N129" s="28" t="s">
-        <v>222</v>
+        <v>122</v>
       </c>
       <c r="O129" s="28"/>
       <c r="P129" s="28"/>
@@ -23855,7 +23844,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="30" t="s">
-        <v>687</v>
+        <v>758</v>
       </c>
       <c r="M132" s="30"/>
       <c r="N132" s="30" t="s">
@@ -24007,7 +23996,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="28" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="M135" s="28"/>
       <c r="N135" s="28" t="s">
@@ -24059,7 +24048,7 @@
         <v>1816</v>
       </c>
       <c r="L136" s="30" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="M136" s="30"/>
       <c r="N136" s="30" t="s">
@@ -24067,7 +24056,7 @@
       </c>
       <c r="O136" s="30"/>
       <c r="P136" s="30" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="Q136" s="30"/>
       <c r="R136" s="30"/>
@@ -24215,7 +24204,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="28" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="M139" s="28"/>
       <c r="N139" s="28" t="s">
@@ -24233,7 +24222,7 @@
         <v>580</v>
       </c>
       <c r="B140" s="30" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C140" s="30" t="s">
         <v>120</v>
@@ -24267,7 +24256,7 @@
         <v>699</v>
       </c>
       <c r="L140" s="30" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="M140" s="30"/>
       <c r="N140" s="30" t="s">
@@ -24369,7 +24358,7 @@
         <v>600</v>
       </c>
       <c r="L142" s="30" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="M142" s="30"/>
       <c r="N142" s="30" t="s">
@@ -24523,7 +24512,7 @@
         <v>0</v>
       </c>
       <c r="L145" s="28" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="M145" s="28"/>
       <c r="N145" s="28" t="s">
@@ -24536,12 +24525,12 @@
       <c r="S145" s="28"/>
       <c r="T145" s="28"/>
     </row>
-    <row r="146" spans="1:20" ht="30">
+    <row r="146" spans="1:20" ht="15">
       <c r="A146" s="30" t="s">
         <v>610</v>
       </c>
       <c r="B146" s="30" t="s">
-        <v>634</v>
+        <v>755</v>
       </c>
       <c r="C146" s="30" t="s">
         <v>120</v>
@@ -24553,10 +24542,10 @@
         <v>1200</v>
       </c>
       <c r="F146" s="85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G146" s="85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H146" s="86">
         <f t="shared" ref="H146:H150" si="27">F146+IF(LEN(G146)=0,0,G146)</f>
@@ -24568,16 +24557,18 @@
       </c>
       <c r="J146" s="84">
         <f t="shared" ref="J146:J150" si="28">F146*I146</f>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="K146" s="84">
         <f t="shared" ref="K146:K150" si="29">IF(LEN(G146)=0,0,G146)*I146</f>
-        <v>2283</v>
-      </c>
-      <c r="L146" s="30"/>
+        <v>1522</v>
+      </c>
+      <c r="L146" s="30" t="s">
+        <v>754</v>
+      </c>
       <c r="M146" s="30"/>
       <c r="N146" s="30" t="s">
-        <v>222</v>
+        <v>180</v>
       </c>
       <c r="O146" s="30"/>
       <c r="P146" s="30"/>
@@ -24591,7 +24582,7 @@
         <v>611</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="C147" s="28" t="s">
         <v>120</v>
@@ -24625,7 +24616,7 @@
         <v>2157</v>
       </c>
       <c r="L147" s="28" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="M147" s="28"/>
       <c r="N147" s="28" t="s">
@@ -24677,7 +24668,7 @@
         <v>502</v>
       </c>
       <c r="L148" s="30" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="M148" s="30"/>
       <c r="N148" s="30" t="s">
@@ -24829,14 +24820,14 @@
         <v>1290</v>
       </c>
       <c r="L151" s="28" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="M151" s="28"/>
       <c r="N151" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O151" s="28" t="s">
-        <v>715</v>
+        <v>710</v>
       </c>
       <c r="P151" s="28" t="s">
         <v>617</v>
@@ -24885,14 +24876,14 @@
         <v>885</v>
       </c>
       <c r="L152" s="30" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="M152" s="30"/>
       <c r="N152" s="30" t="s">
         <v>180</v>
       </c>
       <c r="O152" s="30" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="P152" s="30" t="s">
         <v>620</v>
@@ -24904,10 +24895,10 @@
     </row>
     <row r="153" spans="1:20" ht="15">
       <c r="A153" s="28" t="s">
+        <v>639</v>
+      </c>
+      <c r="B153" s="28" t="s">
         <v>640</v>
-      </c>
-      <c r="B153" s="28" t="s">
-        <v>641</v>
       </c>
       <c r="C153" s="28" t="s">
         <v>120</v>
@@ -24947,7 +24938,7 @@
       </c>
       <c r="O153" s="28"/>
       <c r="P153" s="28" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="Q153" s="28"/>
       <c r="R153" s="28"/>
@@ -24956,10 +24947,10 @@
     </row>
     <row r="154" spans="1:20" ht="15">
       <c r="A154" s="30" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="B154" s="30" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="C154" s="30" t="s">
         <v>135</v>
@@ -24998,7 +24989,7 @@
         <v>222</v>
       </c>
       <c r="O154" s="30" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="P154" s="30"/>
       <c r="Q154" s="30"/>
@@ -25008,10 +24999,10 @@
     </row>
     <row r="155" spans="1:20" ht="15">
       <c r="A155" s="28" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="B155" s="28" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="C155" s="28" t="s">
         <v>135</v>
@@ -25050,7 +25041,7 @@
         <v>222</v>
       </c>
       <c r="O155" s="28" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="P155" s="28"/>
       <c r="Q155" s="28"/>
@@ -25060,10 +25051,10 @@
     </row>
     <row r="156" spans="1:20" ht="15">
       <c r="A156" s="30" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="B156" s="30" t="s">
-        <v>722</v>
+        <v>717</v>
       </c>
       <c r="C156" s="30" t="s">
         <v>135</v>
@@ -25102,7 +25093,7 @@
         <v>222</v>
       </c>
       <c r="O156" s="30" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
       <c r="P156" s="30"/>
       <c r="Q156" s="30"/>
@@ -25112,10 +25103,10 @@
     </row>
     <row r="157" spans="1:20" ht="15">
       <c r="A157" s="28" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="B157" s="28" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="C157" s="28" t="s">
         <v>135</v>
@@ -25149,14 +25140,14 @@
         <v>1575</v>
       </c>
       <c r="L157" s="28" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="M157" s="28"/>
       <c r="N157" s="28" t="s">
         <v>180</v>
       </c>
       <c r="O157" s="28" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="P157" s="28"/>
       <c r="Q157" s="28"/>
@@ -25166,10 +25157,10 @@
     </row>
     <row r="158" spans="1:20" ht="15">
       <c r="A158" s="30" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="B158" s="30" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="C158" s="30" t="s">
         <v>135</v>
@@ -25208,7 +25199,7 @@
         <v>222</v>
       </c>
       <c r="O158" s="30" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="P158" s="30"/>
       <c r="Q158" s="30"/>
@@ -25218,10 +25209,10 @@
     </row>
     <row r="159" spans="1:20" ht="15">
       <c r="A159" s="28" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="B159" s="28" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="C159" s="28" t="s">
         <v>135</v>
@@ -25260,7 +25251,7 @@
         <v>222</v>
       </c>
       <c r="O159" s="28" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="P159" s="28"/>
       <c r="Q159" s="28"/>
@@ -25270,10 +25261,10 @@
     </row>
     <row r="160" spans="1:20" ht="15">
       <c r="A160" s="30" t="s">
+        <v>741</v>
+      </c>
+      <c r="B160" s="30" t="s">
         <v>747</v>
-      </c>
-      <c r="B160" s="30" t="s">
-        <v>753</v>
       </c>
       <c r="C160" s="30" t="s">
         <v>120</v>
@@ -25307,7 +25298,7 @@
         <v>0</v>
       </c>
       <c r="L160" s="30" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="M160" s="30"/>
       <c r="N160" s="30" t="s">
@@ -25322,10 +25313,10 @@
     </row>
     <row r="161" spans="1:20" ht="15">
       <c r="A161" s="28" t="s">
+        <v>742</v>
+      </c>
+      <c r="B161" s="28" t="s">
         <v>748</v>
-      </c>
-      <c r="B161" s="28" t="s">
-        <v>754</v>
       </c>
       <c r="C161" s="28" t="s">
         <v>120</v>
@@ -25359,7 +25350,7 @@
         <v>0</v>
       </c>
       <c r="L161" s="28" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="M161" s="28"/>
       <c r="N161" s="28" t="s">
@@ -25374,10 +25365,10 @@
     </row>
     <row r="162" spans="1:20" ht="15">
       <c r="A162" s="30" t="s">
-        <v>749</v>
+        <v>743</v>
       </c>
       <c r="B162" s="30" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="C162" s="30" t="s">
         <v>120</v>
@@ -25424,10 +25415,10 @@
     </row>
     <row r="163" spans="1:20" ht="15">
       <c r="A163" s="28" t="s">
-        <v>750</v>
+        <v>744</v>
       </c>
       <c r="B163" s="28" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="C163" s="28" t="s">
         <v>120</v>
@@ -26341,7 +26332,7 @@
       </c>
       <c r="B4" s="6">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>220613</v>
+        <v>224113</v>
       </c>
       <c r="C4" s="6">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE)</f>
@@ -26349,11 +26340,11 @@
       </c>
       <c r="D4" s="6">
         <f>Summary!$B$4*C4</f>
-        <v>80536.770799999998</v>
+        <v>81703.670799999993</v>
       </c>
       <c r="E4" s="6">
         <f>B4-D4</f>
-        <v>140076.2292</v>
+        <v>142409.32920000001</v>
       </c>
       <c r="F4" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26361,7 +26352,7 @@
       </c>
       <c r="G4" s="8">
         <f>E4+F4</f>
-        <v>2766.203199999989</v>
+        <v>5099.3031999999948</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -26378,11 +26369,11 @@
       </c>
       <c r="D5" s="7">
         <f>Summary!$B$4*C5</f>
-        <v>80488.458400000003</v>
+        <v>81654.6584</v>
       </c>
       <c r="E5" s="7">
         <f>B5-D5</f>
-        <v>-72069.458400000003</v>
+        <v>-73235.6584</v>
       </c>
       <c r="F5" s="7">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26390,7 +26381,7 @@
       </c>
       <c r="G5" s="9">
         <f>E5+F5</f>
-        <v>-482.41640000000189</v>
+        <v>-1648.616399999999</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -26407,11 +26398,11 @@
       </c>
       <c r="D6" s="6">
         <f>Summary!$B$4*C6</f>
-        <v>80536.770799999998</v>
+        <v>81703.670799999993</v>
       </c>
       <c r="E6" s="6">
         <f>B6-D6</f>
-        <v>-68006.770799999998</v>
+        <v>-69173.670799999993</v>
       </c>
       <c r="F6" s="6">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -26419,7 +26410,7 @@
       </c>
       <c r="G6" s="8">
         <f>E6+F6</f>
-        <v>-2283.7867999999871</v>
+        <v>-3450.6867999999813</v>
       </c>
     </row>
     <row r="9" spans="1:7">

</xml_diff>